<commit_message>
add more generic translations
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/salmanraza/Documents/GitHub/tamanu-source-dbt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86D550A1-1D68-0549-A6A6-4A762DACFACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CEA5841-B2E1-A44E-B88A-085C9BF2BE66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1160" yWindow="980" windowWidth="27640" windowHeight="15440" xr2:uid="{FB1CF5DC-2DD9-EF4F-98DC-2283187EABD8}"/>
   </bookViews>
@@ -1610,21 +1610,12 @@
     <t>Encounter start date</t>
   </si>
   <si>
-    <t>report.reporting.division</t>
-  </si>
-  <si>
     <t>Division</t>
   </si>
   <si>
-    <t>report.reporting.logChangeCreatedAt</t>
-  </si>
-  <si>
     <t>Date and time created</t>
   </si>
   <si>
-    <t>report.reporting.medicalArea</t>
-  </si>
-  <si>
     <t>Medical area</t>
   </si>
   <si>
@@ -1670,9 +1661,6 @@
     <t>Registration status</t>
   </si>
   <si>
-    <t>report.reporting.subDivision</t>
-  </si>
-  <si>
     <t>Sub-division</t>
   </si>
   <si>
@@ -1686,6 +1674,18 @@
   </si>
   <si>
     <t>Date vaccine not given</t>
+  </si>
+  <si>
+    <t>report.reporting.patientSubDivision</t>
+  </si>
+  <si>
+    <t>report.reporting.patientDivision</t>
+  </si>
+  <si>
+    <t>report.reporting.patientMedicalArea</t>
+  </si>
+  <si>
+    <t>report.reporting.logChangeRecordCreatedDateTime</t>
   </si>
 </sst>
 </file>
@@ -2711,971 +2711,971 @@
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A81" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>524</v>
+      <c r="A81" t="s">
+        <v>157</v>
+      </c>
+      <c r="B81" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B82" t="s">
-        <v>11</v>
+        <v>159</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B83" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B84" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B85" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="B86" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="B87" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B88" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B89" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B90" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B91" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="B92" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B93" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>180</v>
+        <v>519</v>
       </c>
       <c r="B94" t="s">
-        <v>181</v>
+        <v>522</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>519</v>
+        <v>182</v>
       </c>
       <c r="B95" t="s">
-        <v>522</v>
+        <v>183</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>182</v>
+        <v>520</v>
       </c>
       <c r="B96" t="s">
-        <v>183</v>
+        <v>521</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>520</v>
+        <v>184</v>
       </c>
       <c r="B97" t="s">
-        <v>521</v>
+        <v>185</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B98" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B99" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B100" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B101" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B102" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B103" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B104" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B105" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B106" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B107" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B108" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B109" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B110" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B111" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B112" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B113" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B114" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B115" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B116" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B117" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B118" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B119" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B120" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B121" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B122" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B123" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B124" t="s">
-        <v>237</v>
+        <v>185</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B125" t="s">
-        <v>185</v>
+        <v>240</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B126" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B127" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B128" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B129" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B130" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B131" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B132" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B133" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B134" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B135" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B136" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B137" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B138" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B139" t="s">
-        <v>266</v>
+        <v>219</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B140" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B141" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B142" t="s">
-        <v>221</v>
+        <v>271</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B143" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B144" t="s">
-        <v>273</v>
+        <v>231</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B145" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B146" t="s">
-        <v>240</v>
+        <v>277</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B147" t="s">
-        <v>277</v>
+        <v>227</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B148" t="s">
-        <v>227</v>
+        <v>280</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B149" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B150" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B151" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B152" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B153" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B154" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B155" t="s">
-        <v>292</v>
+        <v>237</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B156" t="s">
-        <v>237</v>
+        <v>295</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B157" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B158" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B159" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B160" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B161" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B162" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B163" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B164" t="s">
-        <v>309</v>
+        <v>62</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B165" t="s">
-        <v>62</v>
+        <v>19</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B166" t="s">
-        <v>19</v>
+        <v>313</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B167" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B168" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B169" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B170" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B171" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A172" t="s">
-        <v>322</v>
-      </c>
-      <c r="B172" t="s">
-        <v>323</v>
+      <c r="A172" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="B172" s="1" t="s">
+        <v>524</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A173" s="1" t="s">
-        <v>525</v>
-      </c>
-      <c r="B173" s="1" t="s">
-        <v>526</v>
+      <c r="A173" t="s">
+        <v>324</v>
+      </c>
+      <c r="B173" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B174" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A175" s="1" t="s">
-        <v>527</v>
-      </c>
-      <c r="B175" s="1" t="s">
-        <v>528</v>
+      <c r="A175" t="s">
+        <v>328</v>
+      </c>
+      <c r="B175" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="B176" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="B177" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="B178" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
-        <v>332</v>
+        <v>517</v>
       </c>
       <c r="B179" t="s">
-        <v>333</v>
+        <v>518</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B180" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
-        <v>517</v>
+        <v>338</v>
       </c>
       <c r="B181" t="s">
-        <v>518</v>
+        <v>339</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="B182" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="B183" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A184" t="s">
-        <v>340</v>
-      </c>
-      <c r="B184" t="s">
-        <v>341</v>
+      <c r="A184" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="B184" s="1" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B185" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A186" s="1" t="s">
-        <v>529</v>
-      </c>
-      <c r="B186" s="1" t="s">
-        <v>530</v>
+      <c r="A186" t="s">
+        <v>346</v>
+      </c>
+      <c r="B186" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="B187" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="B188" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B189" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="B190" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A191" t="s">
-        <v>352</v>
-      </c>
-      <c r="B191" t="s">
-        <v>353</v>
+      <c r="A191" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="B191" s="1" t="s">
+        <v>523</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B192" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B193" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B194" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B195" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B196" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B197" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B198" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B199" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B200" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A201" t="s">
-        <v>372</v>
-      </c>
-      <c r="B201" t="s">
-        <v>373</v>
+      <c r="A201" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="B201" s="1" t="s">
+        <v>525</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.2">
@@ -3800,338 +3800,338 @@
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A217" s="1" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A218" t="s">
-        <v>402</v>
-      </c>
-      <c r="B218" t="s">
-        <v>403</v>
+      <c r="A218" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="B218" s="1" t="s">
+        <v>540</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B219" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B220" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B221" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B222" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B223" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B224" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B225" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B226" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B227" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B228" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B229" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B230" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B231" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B232" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B233" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B234" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B235" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B236" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="B237" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B238" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B239" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B240" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
+        <v>446</v>
+      </c>
+      <c r="B241" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A242" t="s">
         <v>448</v>
       </c>
-      <c r="B241" t="s">
+      <c r="B242" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="242" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A242" s="1" t="s">
-        <v>533</v>
-      </c>
-      <c r="B242" s="1" t="s">
-        <v>534</v>
-      </c>
-    </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A243" t="s">
+      <c r="A243" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="B243" s="1" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A244" t="s">
         <v>451</v>
       </c>
-      <c r="B243" t="s">
+      <c r="B244" t="s">
         <v>452</v>
-      </c>
-    </row>
-    <row r="244" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A244" s="1" t="s">
-        <v>535</v>
-      </c>
-      <c r="B244" s="1" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A245" s="1" t="s">
-        <v>537</v>
+        <v>532</v>
       </c>
       <c r="B245" s="1" t="s">
-        <v>538</v>
+        <v>533</v>
       </c>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A246" s="1" t="s">
-        <v>539</v>
+        <v>534</v>
       </c>
       <c r="B246" s="1" t="s">
-        <v>540</v>
+        <v>535</v>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A247" t="s">
-        <v>449</v>
-      </c>
-      <c r="B247" t="s">
-        <v>450</v>
+      <c r="A247" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="B247" s="1" t="s">
+        <v>537</v>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="B248" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
-        <v>460</v>
+        <v>453</v>
       </c>
       <c r="B249" t="s">
-        <v>461</v>
+        <v>454</v>
       </c>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B250" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="B251" t="s">
-        <v>47</v>
+        <v>463</v>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B252" t="s">
-        <v>457</v>
+        <v>47</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
+        <v>456</v>
+      </c>
+      <c r="B253" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A254" t="s">
         <v>458</v>
       </c>
-      <c r="B253" t="s">
+      <c r="B254" t="s">
         <v>459</v>
       </c>
     </row>
-    <row r="254" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A254" s="1" t="s">
-        <v>541</v>
-      </c>
-      <c r="B254" s="1" t="s">
-        <v>542</v>
-      </c>
-    </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A255" t="s">
-        <v>464</v>
-      </c>
-      <c r="B255" t="s">
-        <v>465</v>
+      <c r="A255" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="B255" s="1" t="s">
+        <v>539</v>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="B256" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
+        <v>466</v>
+      </c>
+      <c r="B257" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A258" t="s">
         <v>468</v>
       </c>
-      <c r="B257" t="s">
+      <c r="B258" t="s">
         <v>273</v>
-      </c>
-    </row>
-    <row r="258" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A258" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="B258" s="1" t="s">
-        <v>544</v>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.2">
@@ -4232,10 +4232,10 @@
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A271" s="1" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
       <c r="B271" s="1" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.2">
@@ -4264,10 +4264,10 @@
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A275" s="1" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="B275" s="1" t="s">
-        <v>548</v>
+        <v>544</v>
       </c>
     </row>
     <row r="276" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
MAUI-5871 Upgrade to Tamanu 2.40
- Changes to procedures module
- Update to procedures line list report
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="555">
   <si>
     <t>stringId</t>
   </si>
@@ -1339,10 +1339,10 @@
     <t>Procedure anaesthetist</t>
   </si>
   <si>
-    <t>report.reporting.procedureAssistant</t>
-  </si>
-  <si>
-    <t>Procedure assistant</t>
+    <t>report.reporting.procedureAssistantAnaesthetist</t>
+  </si>
+  <si>
+    <t>Procedure assistant anesthetist</t>
   </si>
   <si>
     <t>report.reporting.procedureClinician</t>
@@ -1403,6 +1403,18 @@
   </si>
   <si>
     <t>Procedure start (date and time)</t>
+  </si>
+  <si>
+    <t>report.reporting.procedureTimeIn</t>
+  </si>
+  <si>
+    <t>Procedure time in</t>
+  </si>
+  <si>
+    <t>report.reporting.procedureTimeOut</t>
+  </si>
+  <si>
+    <t>Procedure time out</t>
   </si>
   <si>
     <t>report.reporting.referralCompletedBy</t>
@@ -2032,7 +2044,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B285"/>
+  <dimension ref="A1:B287"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="3" width="58.14785714285715" customWidth="1" bestFit="1"/>
@@ -3407,7 +3419,7 @@
         <v>327</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="19.5">
       <c r="A172" s="2" t="s">
         <v>328</v>
       </c>
@@ -3980,23 +3992,23 @@
         <v>468</v>
       </c>
       <c r="B243" s="1" t="s">
-        <v>241</v>
+        <v>469</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="244" customHeight="1" ht="18.75">
-      <c r="A244" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="B244" s="2" t="s">
+      <c r="A244" s="1" t="s">
         <v>470</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>471</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="245" customHeight="1" ht="18.75">
       <c r="A245" s="1" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B245" s="1" t="s">
-        <v>472</v>
+        <v>241</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="246" customHeight="1" ht="18.75">
@@ -4008,10 +4020,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="247" customHeight="1" ht="18.75">
-      <c r="A247" s="2" t="s">
+      <c r="A247" s="1" t="s">
         <v>475</v>
       </c>
-      <c r="B247" s="2" t="s">
+      <c r="B247" s="1" t="s">
         <v>476</v>
       </c>
     </row>
@@ -4024,18 +4036,18 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="249" customHeight="1" ht="18.75">
-      <c r="A249" s="1" t="s">
+      <c r="A249" s="2" t="s">
         <v>479</v>
       </c>
-      <c r="B249" s="1" t="s">
+      <c r="B249" s="2" t="s">
         <v>480</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="250" customHeight="1" ht="18.75">
-      <c r="A250" s="1" t="s">
+      <c r="A250" s="2" t="s">
         <v>481</v>
       </c>
-      <c r="B250" s="1" t="s">
+      <c r="B250" s="2" t="s">
         <v>482</v>
       </c>
     </row>
@@ -4060,30 +4072,30 @@
         <v>487</v>
       </c>
       <c r="B253" s="1" t="s">
-        <v>47</v>
+        <v>488</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="254" customHeight="1" ht="18.75">
       <c r="A254" s="1" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B254" s="1" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="255" customHeight="1" ht="18.75">
       <c r="A255" s="1" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>491</v>
+        <v>47</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="256" customHeight="1" ht="18.75">
-      <c r="A256" s="2" t="s">
+      <c r="A256" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="B256" s="2" t="s">
+      <c r="B256" s="1" t="s">
         <v>493</v>
       </c>
     </row>
@@ -4096,10 +4108,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="258" customHeight="1" ht="18.75">
-      <c r="A258" s="1" t="s">
+      <c r="A258" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="B258" s="1" t="s">
+      <c r="B258" s="2" t="s">
         <v>497</v>
       </c>
     </row>
@@ -4108,23 +4120,23 @@
         <v>498</v>
       </c>
       <c r="B259" s="1" t="s">
-        <v>277</v>
+        <v>499</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="260" customHeight="1" ht="18.75">
       <c r="A260" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="18.75">
       <c r="A261" s="1" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B261" s="1" t="s">
-        <v>502</v>
+        <v>277</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="18.75">
@@ -4208,10 +4220,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="18.75">
-      <c r="A272" s="2" t="s">
+      <c r="A272" s="1" t="s">
         <v>523</v>
       </c>
-      <c r="B272" s="2" t="s">
+      <c r="B272" s="1" t="s">
         <v>524</v>
       </c>
     </row>
@@ -4224,10 +4236,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="18.75">
-      <c r="A274" s="1" t="s">
+      <c r="A274" s="2" t="s">
         <v>527</v>
       </c>
-      <c r="B274" s="1" t="s">
+      <c r="B274" s="2" t="s">
         <v>528</v>
       </c>
     </row>
@@ -4240,10 +4252,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="276" customHeight="1" ht="18.75">
-      <c r="A276" s="2" t="s">
+      <c r="A276" s="1" t="s">
         <v>531</v>
       </c>
-      <c r="B276" s="2" t="s">
+      <c r="B276" s="1" t="s">
         <v>532</v>
       </c>
     </row>
@@ -4256,10 +4268,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="18.75">
-      <c r="A278" s="1" t="s">
+      <c r="A278" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="B278" s="1" t="s">
+      <c r="B278" s="2" t="s">
         <v>536</v>
       </c>
     </row>
@@ -4317,6 +4329,22 @@
       </c>
       <c r="B285" s="1" t="s">
         <v>550</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="286" customHeight="1" ht="18.75">
+      <c r="A286" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="B286" s="1" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="287" customHeight="1" ht="18.75">
+      <c r="A287" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="B287" s="1" t="s">
+        <v>554</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MAUI-5871 Upgrade to Tamanu 2.40 (#232)
- Changes to procedures module
- Update to procedures line list report
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="555">
   <si>
     <t>stringId</t>
   </si>
@@ -1339,10 +1339,10 @@
     <t>Procedure anaesthetist</t>
   </si>
   <si>
-    <t>report.reporting.procedureAssistant</t>
-  </si>
-  <si>
-    <t>Procedure assistant</t>
+    <t>report.reporting.procedureAssistantAnaesthetist</t>
+  </si>
+  <si>
+    <t>Procedure assistant anesthetist</t>
   </si>
   <si>
     <t>report.reporting.procedureClinician</t>
@@ -1403,6 +1403,18 @@
   </si>
   <si>
     <t>Procedure start (date and time)</t>
+  </si>
+  <si>
+    <t>report.reporting.procedureTimeIn</t>
+  </si>
+  <si>
+    <t>Procedure time in</t>
+  </si>
+  <si>
+    <t>report.reporting.procedureTimeOut</t>
+  </si>
+  <si>
+    <t>Procedure time out</t>
   </si>
   <si>
     <t>report.reporting.referralCompletedBy</t>
@@ -2032,7 +2044,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B285"/>
+  <dimension ref="A1:B287"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="3" width="58.14785714285715" customWidth="1" bestFit="1"/>
@@ -3407,7 +3419,7 @@
         <v>327</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="19.5">
       <c r="A172" s="2" t="s">
         <v>328</v>
       </c>
@@ -3980,23 +3992,23 @@
         <v>468</v>
       </c>
       <c r="B243" s="1" t="s">
-        <v>241</v>
+        <v>469</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="244" customHeight="1" ht="18.75">
-      <c r="A244" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="B244" s="2" t="s">
+      <c r="A244" s="1" t="s">
         <v>470</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>471</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="245" customHeight="1" ht="18.75">
       <c r="A245" s="1" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B245" s="1" t="s">
-        <v>472</v>
+        <v>241</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="246" customHeight="1" ht="18.75">
@@ -4008,10 +4020,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="247" customHeight="1" ht="18.75">
-      <c r="A247" s="2" t="s">
+      <c r="A247" s="1" t="s">
         <v>475</v>
       </c>
-      <c r="B247" s="2" t="s">
+      <c r="B247" s="1" t="s">
         <v>476</v>
       </c>
     </row>
@@ -4024,18 +4036,18 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="249" customHeight="1" ht="18.75">
-      <c r="A249" s="1" t="s">
+      <c r="A249" s="2" t="s">
         <v>479</v>
       </c>
-      <c r="B249" s="1" t="s">
+      <c r="B249" s="2" t="s">
         <v>480</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="250" customHeight="1" ht="18.75">
-      <c r="A250" s="1" t="s">
+      <c r="A250" s="2" t="s">
         <v>481</v>
       </c>
-      <c r="B250" s="1" t="s">
+      <c r="B250" s="2" t="s">
         <v>482</v>
       </c>
     </row>
@@ -4060,30 +4072,30 @@
         <v>487</v>
       </c>
       <c r="B253" s="1" t="s">
-        <v>47</v>
+        <v>488</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="254" customHeight="1" ht="18.75">
       <c r="A254" s="1" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B254" s="1" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="255" customHeight="1" ht="18.75">
       <c r="A255" s="1" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>491</v>
+        <v>47</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="256" customHeight="1" ht="18.75">
-      <c r="A256" s="2" t="s">
+      <c r="A256" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="B256" s="2" t="s">
+      <c r="B256" s="1" t="s">
         <v>493</v>
       </c>
     </row>
@@ -4096,10 +4108,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="258" customHeight="1" ht="18.75">
-      <c r="A258" s="1" t="s">
+      <c r="A258" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="B258" s="1" t="s">
+      <c r="B258" s="2" t="s">
         <v>497</v>
       </c>
     </row>
@@ -4108,23 +4120,23 @@
         <v>498</v>
       </c>
       <c r="B259" s="1" t="s">
-        <v>277</v>
+        <v>499</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="260" customHeight="1" ht="18.75">
       <c r="A260" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="18.75">
       <c r="A261" s="1" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B261" s="1" t="s">
-        <v>502</v>
+        <v>277</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="18.75">
@@ -4208,10 +4220,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="18.75">
-      <c r="A272" s="2" t="s">
+      <c r="A272" s="1" t="s">
         <v>523</v>
       </c>
-      <c r="B272" s="2" t="s">
+      <c r="B272" s="1" t="s">
         <v>524</v>
       </c>
     </row>
@@ -4224,10 +4236,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="18.75">
-      <c r="A274" s="1" t="s">
+      <c r="A274" s="2" t="s">
         <v>527</v>
       </c>
-      <c r="B274" s="1" t="s">
+      <c r="B274" s="2" t="s">
         <v>528</v>
       </c>
     </row>
@@ -4240,10 +4252,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="276" customHeight="1" ht="18.75">
-      <c r="A276" s="2" t="s">
+      <c r="A276" s="1" t="s">
         <v>531</v>
       </c>
-      <c r="B276" s="2" t="s">
+      <c r="B276" s="1" t="s">
         <v>532</v>
       </c>
     </row>
@@ -4256,10 +4268,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="18.75">
-      <c r="A278" s="1" t="s">
+      <c r="A278" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="B278" s="1" t="s">
+      <c r="B278" s="2" t="s">
         <v>536</v>
       </c>
     </row>
@@ -4317,6 +4329,22 @@
       </c>
       <c r="B285" s="1" t="s">
         <v>550</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="286" customHeight="1" ht="18.75">
+      <c r="A286" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="B286" s="1" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="287" customHeight="1" ht="18.75">
+      <c r="A287" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="B287" s="1" t="s">
+        <v>554</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Usage quality metrics on patients
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="575">
   <si>
     <t>stringId</t>
   </si>
@@ -1271,6 +1271,66 @@
   </si>
   <si>
     <t>Social security number</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotal</t>
+  </si>
+  <si>
+    <t>Total patients</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalBirthRegistrations</t>
+  </si>
+  <si>
+    <t>Total birth registrations</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalIncorrectRegistrationsForAgedUnder6Months</t>
+  </si>
+  <si>
+    <t>Total incorrect registrations for aged under 6 months</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalMerged</t>
+  </si>
+  <si>
+    <t>Total patients merged</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalPatientRegistrations</t>
+  </si>
+  <si>
+    <t>Total patient registrations</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithIncompleteName</t>
+  </si>
+  <si>
+    <t>Total patients with incomplete name</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithInvalidDateOfBirth</t>
+  </si>
+  <si>
+    <t>Total patients with invalid date of birth</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithMissingContact</t>
+  </si>
+  <si>
+    <t>Total patients with missing contact</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithMissingDateOfBirth</t>
+  </si>
+  <si>
+    <t>Total patients with missing date of birth</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithMissingLocation</t>
+  </si>
+  <si>
+    <t>Total patients with missing location</t>
   </si>
   <si>
     <t>report.reporting.patientStreetVillage</t>
@@ -2044,11 +2104,11 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B287"/>
+  <dimension ref="A1:B297"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="58.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="3" width="64.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="3" width="35.71928571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -3387,7 +3447,7 @@
         <v>319</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="19.5">
       <c r="A168" s="1" t="s">
         <v>320</v>
       </c>
@@ -3395,7 +3455,7 @@
         <v>321</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="19.5">
       <c r="A169" s="1" t="s">
         <v>322</v>
       </c>
@@ -3403,7 +3463,7 @@
         <v>323</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="19.5">
       <c r="A170" s="1" t="s">
         <v>324</v>
       </c>
@@ -3411,7 +3471,7 @@
         <v>325</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="19.5">
       <c r="A171" s="1" t="s">
         <v>326</v>
       </c>
@@ -3419,7 +3479,7 @@
         <v>327</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="20.25">
       <c r="A172" s="2" t="s">
         <v>328</v>
       </c>
@@ -3427,7 +3487,7 @@
         <v>329</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="19.5">
       <c r="A173" s="1" t="s">
         <v>330</v>
       </c>
@@ -3435,7 +3495,7 @@
         <v>331</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="19.5">
       <c r="A174" s="1" t="s">
         <v>332</v>
       </c>
@@ -3443,7 +3503,7 @@
         <v>333</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="19.5">
       <c r="A175" s="1" t="s">
         <v>334</v>
       </c>
@@ -3451,7 +3511,7 @@
         <v>335</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="19.5">
       <c r="A176" s="1" t="s">
         <v>336</v>
       </c>
@@ -3459,7 +3519,7 @@
         <v>337</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="19.5">
       <c r="A177" s="1" t="s">
         <v>338</v>
       </c>
@@ -3467,7 +3527,7 @@
         <v>339</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="19.5">
       <c r="A178" s="1" t="s">
         <v>340</v>
       </c>
@@ -3475,7 +3535,7 @@
         <v>341</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="19.5">
       <c r="A179" s="1" t="s">
         <v>342</v>
       </c>
@@ -3483,7 +3543,7 @@
         <v>343</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="19.5">
       <c r="A180" s="1" t="s">
         <v>344</v>
       </c>
@@ -3491,7 +3551,7 @@
         <v>345</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="19.5">
       <c r="A181" s="1" t="s">
         <v>346</v>
       </c>
@@ -3499,7 +3559,7 @@
         <v>347</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="19.5">
       <c r="A182" s="1" t="s">
         <v>348</v>
       </c>
@@ -3507,7 +3567,7 @@
         <v>349</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="19.5">
       <c r="A183" s="1" t="s">
         <v>350</v>
       </c>
@@ -3515,7 +3575,7 @@
         <v>351</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="20.25">
       <c r="A184" s="2" t="s">
         <v>352</v>
       </c>
@@ -3523,7 +3583,7 @@
         <v>353</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="19.5">
       <c r="A185" s="1" t="s">
         <v>354</v>
       </c>
@@ -3531,7 +3591,7 @@
         <v>355</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="19.5">
       <c r="A186" s="1" t="s">
         <v>356</v>
       </c>
@@ -3539,7 +3599,7 @@
         <v>357</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="19.5">
       <c r="A187" s="1" t="s">
         <v>358</v>
       </c>
@@ -3547,7 +3607,7 @@
         <v>359</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="19.5">
       <c r="A188" s="1" t="s">
         <v>360</v>
       </c>
@@ -3555,7 +3615,7 @@
         <v>361</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="19.5">
       <c r="A189" s="1" t="s">
         <v>362</v>
       </c>
@@ -3563,7 +3623,7 @@
         <v>363</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="19.5">
       <c r="A190" s="1" t="s">
         <v>364</v>
       </c>
@@ -3571,7 +3631,7 @@
         <v>365</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="19.5">
       <c r="A191" s="1" t="s">
         <v>366</v>
       </c>
@@ -3579,7 +3639,7 @@
         <v>367</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="20.25">
       <c r="A192" s="2" t="s">
         <v>368</v>
       </c>
@@ -3587,7 +3647,7 @@
         <v>369</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="19.5">
       <c r="A193" s="1" t="s">
         <v>370</v>
       </c>
@@ -3595,7 +3655,7 @@
         <v>371</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="19.5">
       <c r="A194" s="1" t="s">
         <v>372</v>
       </c>
@@ -3603,7 +3663,7 @@
         <v>373</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="19.5">
       <c r="A195" s="1" t="s">
         <v>374</v>
       </c>
@@ -3611,7 +3671,7 @@
         <v>375</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="19.5">
       <c r="A196" s="1" t="s">
         <v>376</v>
       </c>
@@ -3619,7 +3679,7 @@
         <v>377</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="19.5">
       <c r="A197" s="1" t="s">
         <v>378</v>
       </c>
@@ -3627,7 +3687,7 @@
         <v>379</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="19.5">
       <c r="A198" s="1" t="s">
         <v>380</v>
       </c>
@@ -3635,7 +3695,7 @@
         <v>381</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="19.5">
       <c r="A199" s="1" t="s">
         <v>382</v>
       </c>
@@ -3643,7 +3703,7 @@
         <v>383</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="19.5">
       <c r="A200" s="1" t="s">
         <v>384</v>
       </c>
@@ -3651,7 +3711,7 @@
         <v>385</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="19.5">
       <c r="A201" s="1" t="s">
         <v>386</v>
       </c>
@@ -3659,7 +3719,7 @@
         <v>387</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="20.25">
       <c r="A202" s="2" t="s">
         <v>388</v>
       </c>
@@ -3667,7 +3727,7 @@
         <v>389</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="19.5">
       <c r="A203" s="1" t="s">
         <v>390</v>
       </c>
@@ -3675,7 +3735,7 @@
         <v>391</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="19.5">
       <c r="A204" s="1" t="s">
         <v>392</v>
       </c>
@@ -3683,7 +3743,7 @@
         <v>393</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="19.5">
       <c r="A205" s="1" t="s">
         <v>394</v>
       </c>
@@ -3691,7 +3751,7 @@
         <v>395</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="19.5">
       <c r="A206" s="1" t="s">
         <v>396</v>
       </c>
@@ -3699,7 +3759,7 @@
         <v>397</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="19.5">
       <c r="A207" s="1" t="s">
         <v>398</v>
       </c>
@@ -3707,7 +3767,7 @@
         <v>399</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="19.5">
       <c r="A208" s="1" t="s">
         <v>400</v>
       </c>
@@ -3787,23 +3847,23 @@
         <v>417</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="218" customHeight="1" ht="18.75">
-      <c r="A218" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="218" customHeight="1" ht="19.5">
+      <c r="A218" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="B218" s="2" t="s">
+      <c r="B218" s="1" t="s">
         <v>419</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="219" customHeight="1" ht="18.75">
-      <c r="A219" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="219" customHeight="1" ht="19.5">
+      <c r="A219" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="B219" s="2" t="s">
+      <c r="B219" s="1" t="s">
         <v>421</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="220" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="220" customHeight="1" ht="19.5">
       <c r="A220" s="1" t="s">
         <v>422</v>
       </c>
@@ -3811,7 +3871,7 @@
         <v>423</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="221" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="221" customHeight="1" ht="19.5">
       <c r="A221" s="1" t="s">
         <v>424</v>
       </c>
@@ -3819,7 +3879,7 @@
         <v>425</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="222" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="222" customHeight="1" ht="19.5">
       <c r="A222" s="1" t="s">
         <v>426</v>
       </c>
@@ -3827,7 +3887,7 @@
         <v>427</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="223" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="223" customHeight="1" ht="19.5">
       <c r="A223" s="1" t="s">
         <v>428</v>
       </c>
@@ -3835,7 +3895,7 @@
         <v>429</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="224" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="224" customHeight="1" ht="19.5">
       <c r="A224" s="1" t="s">
         <v>430</v>
       </c>
@@ -3843,7 +3903,7 @@
         <v>431</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="225" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="225" customHeight="1" ht="19.5">
       <c r="A225" s="1" t="s">
         <v>432</v>
       </c>
@@ -3851,7 +3911,7 @@
         <v>433</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="226" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="226" customHeight="1" ht="19.5">
       <c r="A226" s="1" t="s">
         <v>434</v>
       </c>
@@ -3859,7 +3919,7 @@
         <v>435</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="227" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="227" customHeight="1" ht="19.5">
       <c r="A227" s="1" t="s">
         <v>436</v>
       </c>
@@ -3868,18 +3928,18 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="228" customHeight="1" ht="18.75">
-      <c r="A228" s="1" t="s">
+      <c r="A228" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="B228" s="1" t="s">
+      <c r="B228" s="2" t="s">
         <v>439</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="229" customHeight="1" ht="18.75">
-      <c r="A229" s="1" t="s">
+      <c r="A229" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="B229" s="1" t="s">
+      <c r="B229" s="2" t="s">
         <v>441</v>
       </c>
     </row>
@@ -4008,215 +4068,215 @@
         <v>472</v>
       </c>
       <c r="B245" s="1" t="s">
-        <v>241</v>
+        <v>473</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="246" customHeight="1" ht="18.75">
-      <c r="A246" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="B246" s="2" t="s">
+      <c r="A246" s="1" t="s">
         <v>474</v>
+      </c>
+      <c r="B246" s="1" t="s">
+        <v>475</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="247" customHeight="1" ht="18.75">
       <c r="A247" s="1" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B247" s="1" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="248" customHeight="1" ht="18.75">
-      <c r="A248" s="2" t="s">
-        <v>477</v>
-      </c>
-      <c r="B248" s="2" t="s">
+      <c r="A248" s="1" t="s">
         <v>478</v>
       </c>
+      <c r="B248" s="1" t="s">
+        <v>479</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="249" customHeight="1" ht="18.75">
-      <c r="A249" s="2" t="s">
-        <v>479</v>
-      </c>
-      <c r="B249" s="2" t="s">
+      <c r="A249" s="1" t="s">
         <v>480</v>
       </c>
+      <c r="B249" s="1" t="s">
+        <v>481</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="250" customHeight="1" ht="18.75">
-      <c r="A250" s="2" t="s">
-        <v>481</v>
-      </c>
-      <c r="B250" s="2" t="s">
+      <c r="A250" s="1" t="s">
         <v>482</v>
+      </c>
+      <c r="B250" s="1" t="s">
+        <v>483</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="251" customHeight="1" ht="18.75">
       <c r="A251" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B251" s="1" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="252" customHeight="1" ht="18.75">
       <c r="A252" s="1" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B252" s="1" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="253" customHeight="1" ht="18.75">
       <c r="A253" s="1" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B253" s="1" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="254" customHeight="1" ht="18.75">
       <c r="A254" s="1" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B254" s="1" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="255" customHeight="1" ht="18.75">
       <c r="A255" s="1" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>47</v>
+        <v>241</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="256" customHeight="1" ht="18.75">
-      <c r="A256" s="1" t="s">
-        <v>492</v>
-      </c>
-      <c r="B256" s="1" t="s">
+      <c r="A256" s="2" t="s">
         <v>493</v>
+      </c>
+      <c r="B256" s="2" t="s">
+        <v>494</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="257" customHeight="1" ht="18.75">
       <c r="A257" s="1" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B257" s="1" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="258" customHeight="1" ht="18.75">
       <c r="A258" s="2" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="259" customHeight="1" ht="18.75">
-      <c r="A259" s="1" t="s">
-        <v>498</v>
-      </c>
-      <c r="B259" s="1" t="s">
+      <c r="A259" s="2" t="s">
         <v>499</v>
       </c>
+      <c r="B259" s="2" t="s">
+        <v>500</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="260" customHeight="1" ht="18.75">
-      <c r="A260" s="1" t="s">
-        <v>500</v>
-      </c>
-      <c r="B260" s="1" t="s">
+      <c r="A260" s="2" t="s">
         <v>501</v>
+      </c>
+      <c r="B260" s="2" t="s">
+        <v>502</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="18.75">
       <c r="A261" s="1" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B261" s="1" t="s">
-        <v>277</v>
+        <v>504</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="18.75">
       <c r="A262" s="1" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="263" customHeight="1" ht="18.75">
       <c r="A263" s="1" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B263" s="1" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="264" customHeight="1" ht="18.75">
       <c r="A264" s="1" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B264" s="1" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="265" customHeight="1" ht="18.75">
       <c r="A265" s="1" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B265" s="1" t="s">
-        <v>510</v>
+        <v>47</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="266" customHeight="1" ht="18.75">
       <c r="A266" s="1" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B266" s="1" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="267" customHeight="1" ht="18.75">
       <c r="A267" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B267" s="1" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="268" customHeight="1" ht="18.75">
-      <c r="A268" s="1" t="s">
-        <v>515</v>
-      </c>
-      <c r="B268" s="1" t="s">
+      <c r="A268" s="2" t="s">
         <v>516</v>
+      </c>
+      <c r="B268" s="2" t="s">
+        <v>517</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="269" customHeight="1" ht="18.75">
       <c r="A269" s="1" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B269" s="1" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="270" customHeight="1" ht="18.75">
       <c r="A270" s="1" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B270" s="1" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="271" customHeight="1" ht="18.75">
       <c r="A271" s="1" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B271" s="1" t="s">
-        <v>522</v>
+        <v>277</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="18.75">
@@ -4236,10 +4296,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="18.75">
-      <c r="A274" s="2" t="s">
+      <c r="A274" s="1" t="s">
         <v>527</v>
       </c>
-      <c r="B274" s="2" t="s">
+      <c r="B274" s="1" t="s">
         <v>528</v>
       </c>
     </row>
@@ -4268,10 +4328,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="18.75">
-      <c r="A278" s="2" t="s">
+      <c r="A278" s="1" t="s">
         <v>535</v>
       </c>
-      <c r="B278" s="2" t="s">
+      <c r="B278" s="1" t="s">
         <v>536</v>
       </c>
     </row>
@@ -4316,10 +4376,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="284" customHeight="1" ht="18.75">
-      <c r="A284" s="1" t="s">
+      <c r="A284" s="2" t="s">
         <v>547</v>
       </c>
-      <c r="B284" s="1" t="s">
+      <c r="B284" s="2" t="s">
         <v>548</v>
       </c>
     </row>
@@ -4345,6 +4405,86 @@
       </c>
       <c r="B287" s="1" t="s">
         <v>554</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="288" customHeight="1" ht="18.75">
+      <c r="A288" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="B288" s="2" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="289" customHeight="1" ht="18.75">
+      <c r="A289" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="B289" s="1" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="290" customHeight="1" ht="18.75">
+      <c r="A290" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="291" customHeight="1" ht="18.75">
+      <c r="A291" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="B291" s="1" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="292" customHeight="1" ht="18.75">
+      <c r="A292" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="B292" s="1" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="293" customHeight="1" ht="18.75">
+      <c r="A293" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="B293" s="1" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="294" customHeight="1" ht="18.75">
+      <c r="A294" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="B294" s="1" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="295" customHeight="1" ht="18.75">
+      <c r="A295" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="B295" s="1" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="296" customHeight="1" ht="18.75">
+      <c r="A296" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="B296" s="1" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="297" customHeight="1" ht="18.75">
+      <c r="A297" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="B297" s="1" t="s">
+        <v>574</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Generic Medication Dispensed v2.38 (#243)
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -1,23 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10921"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/salmanraza/Documents/GitHub/tamanu-source-dbt/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD87B249-52E5-194F-AD43-9BBE9D9AB31D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Translated String"/>
+    <sheet name="Translated String" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Translated String'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Translated String'!$A$1:$B$288</definedName>
   </definedNames>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="557">
   <si>
     <t>stringId</t>
   </si>
@@ -1670,13 +1676,30 @@
   </si>
   <si>
     <t>Schedule</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedicationCode</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedication</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionQuantity</t>
+  </si>
+  <si>
+    <t>Medication</t>
+  </si>
+  <si>
+    <t>Quantity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1719,26 +1742,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1749,10 +1777,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -1790,71 +1818,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1882,7 +1910,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1905,11 +1933,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1918,13 +1946,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1934,7 +1962,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1943,7 +1971,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1952,7 +1980,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1960,10 +1988,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -2028,2298 +2056,2327 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B285"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B288"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" style="3" width="58.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="58.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>27</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>33</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="1" t="s">
+    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>35</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="1" t="s">
+    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>37</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="1" t="s">
+    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="1" t="s">
+    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>41</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="1" t="s">
+    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>43</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="1" t="s">
+    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>45</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="1" t="s">
+    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="1" t="s">
+    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" t="s">
         <v>49</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="1" t="s">
+    <row r="26" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" t="s">
         <v>51</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
-      <c r="A27" s="1" t="s">
+    <row r="27" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
         <v>53</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
-      <c r="A28" s="1" t="s">
+    <row r="28" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>55</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
-      <c r="A29" s="1" t="s">
+    <row r="29" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" t="s">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
-      <c r="A30" s="1" t="s">
+    <row r="30" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" t="s">
         <v>58</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
-      <c r="A31" s="1" t="s">
+    <row r="31" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
         <v>59</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>60</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
-      <c r="A32" s="1" t="s">
+    <row r="32" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>61</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
         <v>62</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="1" t="s">
+    <row r="33" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
         <v>63</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" t="s">
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
-      <c r="A34" s="1" t="s">
+    <row r="34" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
         <v>64</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" t="s">
         <v>65</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
-      <c r="A35" s="1" t="s">
+    <row r="35" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
         <v>66</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" t="s">
         <v>67</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
-      <c r="A36" s="1" t="s">
+    <row r="36" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" t="s">
         <v>69</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
-      <c r="A37" s="1" t="s">
+    <row r="37" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
         <v>70</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" t="s">
         <v>71</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
-      <c r="A38" s="1" t="s">
+    <row r="38" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
         <v>72</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" t="s">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
-      <c r="A39" s="1" t="s">
+    <row r="39" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
         <v>73</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" t="s">
         <v>74</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
-      <c r="A40" s="1" t="s">
+    <row r="40" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
         <v>75</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" t="s">
         <v>76</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
-      <c r="A41" s="1" t="s">
+    <row r="41" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
         <v>77</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" t="s">
         <v>78</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
-      <c r="A42" s="1" t="s">
+    <row r="42" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
         <v>79</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" t="s">
         <v>80</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
-      <c r="A43" s="1" t="s">
+    <row r="43" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
         <v>81</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" t="s">
         <v>82</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
-      <c r="A44" s="1" t="s">
+    <row r="44" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
         <v>83</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" t="s">
         <v>84</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
-      <c r="A45" s="1" t="s">
+    <row r="45" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
         <v>85</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" t="s">
         <v>86</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
-      <c r="A46" s="1" t="s">
+    <row r="46" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
         <v>87</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" t="s">
         <v>88</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
-      <c r="A47" s="1" t="s">
+    <row r="47" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>89</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" t="s">
         <v>90</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
-      <c r="A48" s="1" t="s">
+    <row r="48" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
         <v>91</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" t="s">
         <v>92</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
-      <c r="A49" s="1" t="s">
+    <row r="49" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
         <v>93</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" t="s">
         <v>94</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
-      <c r="A50" s="1" t="s">
+    <row r="50" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
         <v>95</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" t="s">
         <v>96</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
-      <c r="A51" s="1" t="s">
+    <row r="51" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
         <v>97</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" t="s">
         <v>98</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
-      <c r="A52" s="1" t="s">
+    <row r="52" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
         <v>99</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" t="s">
         <v>100</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
-      <c r="A53" s="1" t="s">
+    <row r="53" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
         <v>101</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" t="s">
         <v>102</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
-      <c r="A54" s="1" t="s">
+    <row r="54" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
         <v>103</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" t="s">
         <v>104</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
-      <c r="A55" s="1" t="s">
+    <row r="55" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
         <v>105</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" t="s">
         <v>106</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
-      <c r="A56" s="1" t="s">
+    <row r="56" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
         <v>107</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" t="s">
         <v>108</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
-      <c r="A57" s="1" t="s">
+    <row r="57" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
         <v>109</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" t="s">
         <v>110</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
-      <c r="A58" s="1" t="s">
+    <row r="58" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
         <v>111</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" t="s">
         <v>112</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
-      <c r="A59" s="1" t="s">
+    <row r="59" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
         <v>113</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" t="s">
         <v>114</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
-      <c r="A60" s="1" t="s">
+    <row r="60" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
         <v>115</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B60" t="s">
         <v>116</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
-      <c r="A61" s="1" t="s">
+    <row r="61" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
         <v>117</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" t="s">
         <v>118</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
-      <c r="A62" s="1" t="s">
+    <row r="62" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
         <v>119</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B62" t="s">
         <v>120</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
-      <c r="A63" s="1" t="s">
+    <row r="63" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
         <v>121</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B63" t="s">
         <v>122</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
-      <c r="A64" s="1" t="s">
+    <row r="64" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
         <v>123</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B64" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
-      <c r="A65" s="1" t="s">
+    <row r="65" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
         <v>125</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="B65" t="s">
         <v>126</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
-      <c r="A66" s="1" t="s">
+    <row r="66" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
         <v>127</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B66" t="s">
         <v>128</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
-      <c r="A67" s="1" t="s">
+    <row r="67" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
         <v>129</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B67" t="s">
         <v>130</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
-      <c r="A68" s="1" t="s">
+    <row r="68" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
         <v>131</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B68" t="s">
         <v>132</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
-      <c r="A69" s="1" t="s">
+    <row r="69" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
         <v>133</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B69" t="s">
         <v>134</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
-      <c r="A70" s="1" t="s">
+    <row r="70" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
         <v>135</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="B70" t="s">
         <v>136</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
-      <c r="A71" s="1" t="s">
+    <row r="71" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
         <v>137</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B71" t="s">
         <v>138</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
-      <c r="A72" s="1" t="s">
+    <row r="72" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
         <v>139</v>
       </c>
-      <c r="B72" s="1" t="s">
+      <c r="B72" t="s">
         <v>140</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
-      <c r="A73" s="1" t="s">
+    <row r="73" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
         <v>141</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="B73" t="s">
         <v>142</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
-      <c r="A74" s="1" t="s">
+    <row r="74" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
         <v>143</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="B74" t="s">
         <v>144</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
-      <c r="A75" s="1" t="s">
+    <row r="75" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
         <v>145</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B75" t="s">
         <v>146</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
-      <c r="A76" s="1" t="s">
+    <row r="76" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
         <v>147</v>
       </c>
-      <c r="B76" s="1" t="s">
+      <c r="B76" t="s">
         <v>148</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
-      <c r="A77" s="1" t="s">
+    <row r="77" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
         <v>149</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="B77" t="s">
         <v>150</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
-      <c r="A78" s="1" t="s">
+    <row r="78" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
         <v>151</v>
       </c>
-      <c r="B78" s="1" t="s">
+      <c r="B78" t="s">
         <v>152</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
-      <c r="A79" s="1" t="s">
+    <row r="79" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
         <v>153</v>
       </c>
-      <c r="B79" s="1" t="s">
+      <c r="B79" t="s">
         <v>154</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
-      <c r="A80" s="1" t="s">
+    <row r="80" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
         <v>155</v>
       </c>
-      <c r="B80" s="1" t="s">
+      <c r="B80" t="s">
         <v>156</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
-      <c r="A81" s="1" t="s">
+    <row r="81" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
         <v>157</v>
       </c>
-      <c r="B81" s="1" t="s">
+      <c r="B81" t="s">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
-      <c r="A82" s="1" t="s">
+    <row r="82" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
         <v>158</v>
       </c>
-      <c r="B82" s="1" t="s">
+      <c r="B82" t="s">
         <v>159</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
-      <c r="A83" s="1" t="s">
+    <row r="83" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
         <v>160</v>
       </c>
-      <c r="B83" s="1" t="s">
+      <c r="B83" t="s">
         <v>161</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
-      <c r="A84" s="1" t="s">
+    <row r="84" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
         <v>162</v>
       </c>
-      <c r="B84" s="1" t="s">
+      <c r="B84" t="s">
         <v>163</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
-      <c r="A85" s="1" t="s">
+    <row r="85" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
         <v>164</v>
       </c>
-      <c r="B85" s="1" t="s">
+      <c r="B85" t="s">
         <v>165</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
-      <c r="A86" s="1" t="s">
+    <row r="86" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
         <v>166</v>
       </c>
-      <c r="B86" s="1" t="s">
+      <c r="B86" t="s">
         <v>167</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
-      <c r="A87" s="1" t="s">
+    <row r="87" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
         <v>168</v>
       </c>
-      <c r="B87" s="1" t="s">
+      <c r="B87" t="s">
         <v>169</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
-      <c r="A88" s="1" t="s">
+    <row r="88" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
         <v>170</v>
       </c>
-      <c r="B88" s="1" t="s">
+      <c r="B88" t="s">
         <v>171</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
-      <c r="A89" s="1" t="s">
+    <row r="89" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
         <v>172</v>
       </c>
-      <c r="B89" s="1" t="s">
+      <c r="B89" t="s">
         <v>173</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
-      <c r="A90" s="1" t="s">
+    <row r="90" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
         <v>174</v>
       </c>
-      <c r="B90" s="1" t="s">
+      <c r="B90" t="s">
         <v>175</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
-      <c r="A91" s="1" t="s">
+    <row r="91" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
         <v>176</v>
       </c>
-      <c r="B91" s="1" t="s">
+      <c r="B91" t="s">
         <v>177</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
-      <c r="A92" s="1" t="s">
+    <row r="92" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
         <v>178</v>
       </c>
-      <c r="B92" s="1" t="s">
+      <c r="B92" t="s">
         <v>179</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
-      <c r="A93" s="1" t="s">
+    <row r="93" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
         <v>180</v>
       </c>
-      <c r="B93" s="1" t="s">
+      <c r="B93" t="s">
         <v>181</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
-      <c r="A94" s="1" t="s">
+    <row r="94" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
         <v>182</v>
       </c>
-      <c r="B94" s="1" t="s">
+      <c r="B94" t="s">
         <v>183</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
-      <c r="A95" s="1" t="s">
+    <row r="95" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
         <v>184</v>
       </c>
-      <c r="B95" s="1" t="s">
+      <c r="B95" t="s">
         <v>185</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
-      <c r="A96" s="1" t="s">
+    <row r="96" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
         <v>186</v>
       </c>
-      <c r="B96" s="1" t="s">
+      <c r="B96" t="s">
         <v>187</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
-      <c r="A97" s="1" t="s">
+    <row r="97" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
         <v>188</v>
       </c>
-      <c r="B97" s="1" t="s">
+      <c r="B97" t="s">
         <v>189</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
-      <c r="A98" s="1" t="s">
+    <row r="98" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
         <v>190</v>
       </c>
-      <c r="B98" s="1" t="s">
+      <c r="B98" t="s">
         <v>191</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
-      <c r="A99" s="1" t="s">
+    <row r="99" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
         <v>192</v>
       </c>
-      <c r="B99" s="1" t="s">
+      <c r="B99" t="s">
         <v>193</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
-      <c r="A100" s="1" t="s">
+    <row r="100" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
         <v>194</v>
       </c>
-      <c r="B100" s="1" t="s">
+      <c r="B100" t="s">
         <v>195</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
-      <c r="A101" s="1" t="s">
+    <row r="101" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
         <v>196</v>
       </c>
-      <c r="B101" s="1" t="s">
+      <c r="B101" t="s">
         <v>197</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
-      <c r="A102" s="1" t="s">
+    <row r="102" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
         <v>198</v>
       </c>
-      <c r="B102" s="1" t="s">
+      <c r="B102" t="s">
         <v>199</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
-      <c r="A103" s="1" t="s">
+    <row r="103" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
         <v>200</v>
       </c>
-      <c r="B103" s="1" t="s">
+      <c r="B103" t="s">
         <v>201</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
-      <c r="A104" s="1" t="s">
+    <row r="104" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
         <v>202</v>
       </c>
-      <c r="B104" s="1" t="s">
+      <c r="B104" t="s">
         <v>203</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
-      <c r="A105" s="1" t="s">
+    <row r="105" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
         <v>204</v>
       </c>
-      <c r="B105" s="1" t="s">
+      <c r="B105" t="s">
         <v>205</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
-      <c r="A106" s="1" t="s">
+    <row r="106" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
         <v>206</v>
       </c>
-      <c r="B106" s="1" t="s">
+      <c r="B106" t="s">
         <v>207</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
-      <c r="A107" s="1" t="s">
+    <row r="107" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
         <v>208</v>
       </c>
-      <c r="B107" s="1" t="s">
+      <c r="B107" t="s">
         <v>209</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75">
-      <c r="A108" s="1" t="s">
+    <row r="108" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
         <v>210</v>
       </c>
-      <c r="B108" s="1" t="s">
+      <c r="B108" t="s">
         <v>211</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75">
-      <c r="A109" s="1" t="s">
+    <row r="109" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
         <v>212</v>
       </c>
-      <c r="B109" s="1" t="s">
+      <c r="B109" t="s">
         <v>213</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
-      <c r="A110" s="1" t="s">
+    <row r="110" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
         <v>214</v>
       </c>
-      <c r="B110" s="1" t="s">
+      <c r="B110" t="s">
         <v>215</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
-      <c r="A111" s="1" t="s">
+    <row r="111" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
         <v>216</v>
       </c>
-      <c r="B111" s="1" t="s">
+      <c r="B111" t="s">
         <v>217</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
-      <c r="A112" s="1" t="s">
+    <row r="112" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
         <v>218</v>
       </c>
-      <c r="B112" s="1" t="s">
+      <c r="B112" t="s">
         <v>219</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
-      <c r="A113" s="1" t="s">
+    <row r="113" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
         <v>220</v>
       </c>
-      <c r="B113" s="1" t="s">
+      <c r="B113" t="s">
         <v>221</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
-      <c r="A114" s="1" t="s">
+    <row r="114" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
         <v>222</v>
       </c>
-      <c r="B114" s="1" t="s">
+      <c r="B114" t="s">
         <v>223</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
-      <c r="A115" s="1" t="s">
+    <row r="115" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
         <v>224</v>
       </c>
-      <c r="B115" s="1" t="s">
+      <c r="B115" t="s">
         <v>225</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
-      <c r="A116" s="1" t="s">
+    <row r="116" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
         <v>226</v>
       </c>
-      <c r="B116" s="1" t="s">
+      <c r="B116" t="s">
         <v>227</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
-      <c r="A117" s="1" t="s">
+    <row r="117" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
         <v>228</v>
       </c>
-      <c r="B117" s="1" t="s">
+      <c r="B117" t="s">
         <v>229</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
-      <c r="A118" s="1" t="s">
+    <row r="118" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
         <v>230</v>
       </c>
-      <c r="B118" s="1" t="s">
+      <c r="B118" t="s">
         <v>231</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
-      <c r="A119" s="1" t="s">
+    <row r="119" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
         <v>232</v>
       </c>
-      <c r="B119" s="1" t="s">
+      <c r="B119" t="s">
         <v>233</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
-      <c r="A120" s="1" t="s">
+    <row r="120" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
         <v>234</v>
       </c>
-      <c r="B120" s="1" t="s">
+      <c r="B120" t="s">
         <v>235</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
-      <c r="A121" s="1" t="s">
+    <row r="121" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
         <v>236</v>
       </c>
-      <c r="B121" s="1" t="s">
+      <c r="B121" t="s">
         <v>237</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
-      <c r="A122" s="1" t="s">
+    <row r="122" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
         <v>238</v>
       </c>
-      <c r="B122" s="1" t="s">
+      <c r="B122" t="s">
         <v>239</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
-      <c r="A123" s="1" t="s">
+    <row r="123" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
         <v>240</v>
       </c>
-      <c r="B123" s="1" t="s">
+      <c r="B123" t="s">
         <v>241</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
-      <c r="A124" s="1" t="s">
+    <row r="124" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
         <v>242</v>
       </c>
-      <c r="B124" s="1" t="s">
+      <c r="B124" t="s">
         <v>189</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
-      <c r="A125" s="1" t="s">
+    <row r="125" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
         <v>243</v>
       </c>
-      <c r="B125" s="1" t="s">
+      <c r="B125" t="s">
         <v>244</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
-      <c r="A126" s="1" t="s">
+    <row r="126" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
         <v>245</v>
       </c>
-      <c r="B126" s="1" t="s">
+      <c r="B126" t="s">
         <v>246</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
-      <c r="A127" s="1" t="s">
+    <row r="127" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
         <v>247</v>
       </c>
-      <c r="B127" s="1" t="s">
+      <c r="B127" t="s">
         <v>248</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
-      <c r="A128" s="1" t="s">
+    <row r="128" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
         <v>249</v>
       </c>
-      <c r="B128" s="1" t="s">
+      <c r="B128" t="s">
         <v>250</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
-      <c r="A129" s="1" t="s">
+    <row r="129" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A129" t="s">
         <v>251</v>
       </c>
-      <c r="B129" s="1" t="s">
+      <c r="B129" t="s">
         <v>252</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75">
-      <c r="A130" s="1" t="s">
+    <row r="130" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A130" t="s">
         <v>253</v>
       </c>
-      <c r="B130" s="1" t="s">
+      <c r="B130" t="s">
         <v>254</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18.75">
-      <c r="A131" s="1" t="s">
+    <row r="131" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A131" t="s">
         <v>255</v>
       </c>
-      <c r="B131" s="1" t="s">
+      <c r="B131" t="s">
         <v>256</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18.75">
-      <c r="A132" s="1" t="s">
+    <row r="132" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A132" t="s">
         <v>257</v>
       </c>
-      <c r="B132" s="1" t="s">
+      <c r="B132" t="s">
         <v>258</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="18.75">
-      <c r="A133" s="1" t="s">
+    <row r="133" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A133" t="s">
         <v>259</v>
       </c>
-      <c r="B133" s="1" t="s">
+      <c r="B133" t="s">
         <v>260</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18.75">
-      <c r="A134" s="1" t="s">
+    <row r="134" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A134" t="s">
         <v>261</v>
       </c>
-      <c r="B134" s="1" t="s">
+      <c r="B134" t="s">
         <v>262</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18.75">
-      <c r="A135" s="1" t="s">
+    <row r="135" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A135" t="s">
         <v>263</v>
       </c>
-      <c r="B135" s="1" t="s">
+      <c r="B135" t="s">
         <v>264</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18.75">
-      <c r="A136" s="1" t="s">
+    <row r="136" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A136" t="s">
         <v>265</v>
       </c>
-      <c r="B136" s="1" t="s">
+      <c r="B136" t="s">
         <v>266</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18.75">
-      <c r="A137" s="1" t="s">
+    <row r="137" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A137" t="s">
         <v>267</v>
       </c>
-      <c r="B137" s="1" t="s">
+      <c r="B137" t="s">
         <v>268</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18.75">
-      <c r="A138" s="1" t="s">
+    <row r="138" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A138" t="s">
         <v>269</v>
       </c>
-      <c r="B138" s="1" t="s">
+      <c r="B138" t="s">
         <v>270</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18.75">
-      <c r="A139" s="1" t="s">
+    <row r="139" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A139" t="s">
         <v>271</v>
       </c>
-      <c r="B139" s="1" t="s">
+      <c r="B139" t="s">
         <v>223</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18.75">
-      <c r="A140" s="1" t="s">
+    <row r="140" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A140" t="s">
         <v>272</v>
       </c>
-      <c r="B140" s="1" t="s">
+      <c r="B140" t="s">
         <v>237</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18.75">
-      <c r="A141" s="1" t="s">
+    <row r="141" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A141" t="s">
         <v>273</v>
       </c>
-      <c r="B141" s="1" t="s">
+      <c r="B141" t="s">
         <v>225</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18.75">
-      <c r="A142" s="1" t="s">
+    <row r="142" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A142" t="s">
         <v>274</v>
       </c>
-      <c r="B142" s="1" t="s">
+      <c r="B142" t="s">
         <v>275</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18.75">
-      <c r="A143" s="1" t="s">
+    <row r="143" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A143" t="s">
         <v>276</v>
       </c>
-      <c r="B143" s="1" t="s">
+      <c r="B143" t="s">
         <v>277</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="18.75">
-      <c r="A144" s="1" t="s">
+    <row r="144" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A144" t="s">
         <v>278</v>
       </c>
-      <c r="B144" s="1" t="s">
+      <c r="B144" t="s">
         <v>235</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="18.75">
-      <c r="A145" s="1" t="s">
+    <row r="145" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A145" t="s">
         <v>279</v>
       </c>
-      <c r="B145" s="1" t="s">
+      <c r="B145" t="s">
         <v>244</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="18.75">
-      <c r="A146" s="1" t="s">
+    <row r="146" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A146" t="s">
         <v>280</v>
       </c>
-      <c r="B146" s="1" t="s">
+      <c r="B146" t="s">
         <v>281</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="18.75">
-      <c r="A147" s="1" t="s">
+    <row r="147" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A147" t="s">
         <v>282</v>
       </c>
-      <c r="B147" s="1" t="s">
+      <c r="B147" t="s">
         <v>231</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="18.75">
-      <c r="A148" s="1" t="s">
+    <row r="148" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A148" t="s">
         <v>283</v>
       </c>
-      <c r="B148" s="1" t="s">
+      <c r="B148" t="s">
         <v>284</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="18.75">
-      <c r="A149" s="1" t="s">
+    <row r="149" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A149" t="s">
         <v>285</v>
       </c>
-      <c r="B149" s="1" t="s">
+      <c r="B149" t="s">
         <v>286</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18.75">
-      <c r="A150" s="1" t="s">
+    <row r="150" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A150" t="s">
         <v>287</v>
       </c>
-      <c r="B150" s="1" t="s">
+      <c r="B150" t="s">
         <v>288</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18.75">
-      <c r="A151" s="1" t="s">
+    <row r="151" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A151" t="s">
         <v>289</v>
       </c>
-      <c r="B151" s="1" t="s">
+      <c r="B151" t="s">
         <v>290</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18.75">
-      <c r="A152" s="1" t="s">
+    <row r="152" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A152" t="s">
         <v>291</v>
       </c>
-      <c r="B152" s="1" t="s">
+      <c r="B152" t="s">
         <v>292</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="18.75">
-      <c r="A153" s="1" t="s">
+    <row r="153" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A153" t="s">
         <v>293</v>
       </c>
-      <c r="B153" s="1" t="s">
+      <c r="B153" t="s">
         <v>294</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18.75">
-      <c r="A154" s="1" t="s">
+    <row r="154" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A154" t="s">
         <v>295</v>
       </c>
-      <c r="B154" s="1" t="s">
+      <c r="B154" t="s">
         <v>296</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18.75">
-      <c r="A155" s="1" t="s">
+    <row r="155" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A155" t="s">
         <v>297</v>
       </c>
-      <c r="B155" s="1" t="s">
+      <c r="B155" t="s">
         <v>241</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18.75">
-      <c r="A156" s="1" t="s">
+    <row r="156" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A156" t="s">
         <v>298</v>
       </c>
-      <c r="B156" s="1" t="s">
+      <c r="B156" t="s">
         <v>299</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18.75">
-      <c r="A157" s="1" t="s">
+    <row r="157" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A157" t="s">
         <v>300</v>
       </c>
-      <c r="B157" s="1" t="s">
+      <c r="B157" t="s">
         <v>301</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18.75">
-      <c r="A158" s="1" t="s">
+    <row r="158" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A158" t="s">
         <v>302</v>
       </c>
-      <c r="B158" s="1" t="s">
+      <c r="B158" t="s">
         <v>303</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18.75">
-      <c r="A159" s="1" t="s">
+    <row r="159" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A159" t="s">
         <v>304</v>
       </c>
-      <c r="B159" s="1" t="s">
+      <c r="B159" t="s">
         <v>305</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18.75">
-      <c r="A160" s="1" t="s">
+    <row r="160" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A160" t="s">
         <v>306</v>
       </c>
-      <c r="B160" s="1" t="s">
+      <c r="B160" t="s">
         <v>307</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18.75">
-      <c r="A161" s="1" t="s">
+    <row r="161" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A161" t="s">
         <v>308</v>
       </c>
-      <c r="B161" s="1" t="s">
+      <c r="B161" t="s">
         <v>309</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18.75">
-      <c r="A162" s="1" t="s">
+    <row r="162" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A162" t="s">
         <v>310</v>
       </c>
-      <c r="B162" s="1" t="s">
+      <c r="B162" t="s">
         <v>311</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75">
-      <c r="A163" s="1" t="s">
+    <row r="163" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A163" t="s">
         <v>312</v>
       </c>
-      <c r="B163" s="1" t="s">
+      <c r="B163" t="s">
         <v>313</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75">
-      <c r="A164" s="1" t="s">
+    <row r="164" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A164" t="s">
         <v>314</v>
       </c>
-      <c r="B164" s="1" t="s">
+      <c r="B164" t="s">
         <v>62</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75">
-      <c r="A165" s="1" t="s">
+    <row r="165" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A165" t="s">
         <v>315</v>
       </c>
-      <c r="B165" s="1" t="s">
+      <c r="B165" t="s">
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75">
-      <c r="A166" s="1" t="s">
+    <row r="166" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A166" t="s">
         <v>316</v>
       </c>
-      <c r="B166" s="1" t="s">
+      <c r="B166" t="s">
         <v>317</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75">
-      <c r="A167" s="1" t="s">
+    <row r="167" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A167" t="s">
         <v>318</v>
       </c>
-      <c r="B167" s="1" t="s">
+      <c r="B167" t="s">
         <v>319</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18.75">
-      <c r="A168" s="1" t="s">
+    <row r="168" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A168" t="s">
         <v>320</v>
       </c>
-      <c r="B168" s="1" t="s">
+      <c r="B168" t="s">
         <v>321</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="18.75">
-      <c r="A169" s="1" t="s">
+    <row r="169" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A169" t="s">
         <v>322</v>
       </c>
-      <c r="B169" s="1" t="s">
+      <c r="B169" t="s">
         <v>323</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18.75">
-      <c r="A170" s="1" t="s">
+    <row r="170" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A170" t="s">
         <v>324</v>
       </c>
-      <c r="B170" s="1" t="s">
+      <c r="B170" t="s">
         <v>325</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18.75">
-      <c r="A171" s="1" t="s">
+    <row r="171" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A171" t="s">
         <v>326</v>
       </c>
-      <c r="B171" s="1" t="s">
+      <c r="B171" t="s">
         <v>327</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="18.75">
+    <row r="172" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A173" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="B172" s="2" t="s">
+      <c r="B173" s="3" t="s">
         <v>329</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18.75">
-      <c r="A173" s="1" t="s">
-        <v>330</v>
-      </c>
-      <c r="B173" s="1" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18.75">
-      <c r="A174" s="1" t="s">
+    <row r="174" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A174" t="s">
         <v>332</v>
       </c>
-      <c r="B174" s="1" t="s">
+      <c r="B174" t="s">
         <v>333</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18.75">
-      <c r="A175" s="1" t="s">
+    <row r="175" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A175" t="s">
         <v>334</v>
       </c>
-      <c r="B175" s="1" t="s">
+      <c r="B175" t="s">
         <v>335</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18.75">
-      <c r="A176" s="1" t="s">
+    <row r="176" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A176" t="s">
         <v>336</v>
       </c>
-      <c r="B176" s="1" t="s">
+      <c r="B176" t="s">
         <v>337</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="18.75">
-      <c r="A177" s="1" t="s">
+    <row r="177" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A177" t="s">
         <v>338</v>
       </c>
-      <c r="B177" s="1" t="s">
+      <c r="B177" t="s">
         <v>339</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18.75">
-      <c r="A178" s="1" t="s">
+    <row r="178" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A178" t="s">
         <v>340</v>
       </c>
-      <c r="B178" s="1" t="s">
+      <c r="B178" t="s">
         <v>341</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18.75">
-      <c r="A179" s="1" t="s">
+    <row r="179" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A179" t="s">
         <v>342</v>
       </c>
-      <c r="B179" s="1" t="s">
+      <c r="B179" t="s">
         <v>343</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18.75">
-      <c r="A180" s="1" t="s">
+    <row r="180" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A180" t="s">
         <v>344</v>
       </c>
-      <c r="B180" s="1" t="s">
+      <c r="B180" t="s">
         <v>345</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18.75">
-      <c r="A181" s="1" t="s">
+    <row r="181" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A181" t="s">
         <v>346</v>
       </c>
-      <c r="B181" s="1" t="s">
+      <c r="B181" t="s">
         <v>347</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18.75">
-      <c r="A182" s="1" t="s">
+    <row r="182" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A182" t="s">
         <v>348</v>
       </c>
-      <c r="B182" s="1" t="s">
+      <c r="B182" t="s">
         <v>349</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18.75">
-      <c r="A183" s="1" t="s">
+    <row r="183" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A183" t="s">
         <v>350</v>
       </c>
-      <c r="B183" s="1" t="s">
+      <c r="B183" t="s">
         <v>351</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18.75">
-      <c r="A184" s="2" t="s">
+    <row r="184" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A184" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="B184" s="2" t="s">
+      <c r="B184" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18.75">
-      <c r="A185" s="1" t="s">
+    <row r="185" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A185" t="s">
         <v>354</v>
       </c>
-      <c r="B185" s="1" t="s">
+      <c r="B185" t="s">
         <v>355</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75">
-      <c r="A186" s="1" t="s">
+    <row r="186" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A186" t="s">
         <v>356</v>
       </c>
-      <c r="B186" s="1" t="s">
+      <c r="B186" t="s">
         <v>357</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18.75">
-      <c r="A187" s="1" t="s">
+    <row r="187" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A187" t="s">
         <v>358</v>
       </c>
-      <c r="B187" s="1" t="s">
+      <c r="B187" t="s">
         <v>359</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75">
-      <c r="A188" s="1" t="s">
+    <row r="188" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A188" t="s">
         <v>360</v>
       </c>
-      <c r="B188" s="1" t="s">
+      <c r="B188" t="s">
         <v>361</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75">
-      <c r="A189" s="1" t="s">
+    <row r="189" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A189" t="s">
         <v>362</v>
       </c>
-      <c r="B189" s="1" t="s">
+      <c r="B189" t="s">
         <v>363</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75">
-      <c r="A190" s="1" t="s">
+    <row r="190" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A190" t="s">
         <v>364</v>
       </c>
-      <c r="B190" s="1" t="s">
+      <c r="B190" t="s">
         <v>365</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18.75">
-      <c r="A191" s="1" t="s">
+    <row r="191" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A191" t="s">
         <v>366</v>
       </c>
-      <c r="B191" s="1" t="s">
+      <c r="B191" t="s">
         <v>367</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="18.75">
-      <c r="A192" s="2" t="s">
+    <row r="192" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A192" s="1" t="s">
         <v>368</v>
       </c>
-      <c r="B192" s="2" t="s">
+      <c r="B192" s="1" t="s">
         <v>369</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18.75">
-      <c r="A193" s="1" t="s">
+    <row r="193" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A193" t="s">
         <v>370</v>
       </c>
-      <c r="B193" s="1" t="s">
+      <c r="B193" t="s">
         <v>371</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="18.75">
-      <c r="A194" s="1" t="s">
+    <row r="194" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A194" t="s">
         <v>372</v>
       </c>
-      <c r="B194" s="1" t="s">
+      <c r="B194" t="s">
         <v>373</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18.75">
-      <c r="A195" s="1" t="s">
+    <row r="195" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A195" t="s">
         <v>374</v>
       </c>
-      <c r="B195" s="1" t="s">
+      <c r="B195" t="s">
         <v>375</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="18.75">
-      <c r="A196" s="1" t="s">
+    <row r="196" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A196" t="s">
         <v>376</v>
       </c>
-      <c r="B196" s="1" t="s">
+      <c r="B196" t="s">
         <v>377</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18.75">
-      <c r="A197" s="1" t="s">
+    <row r="197" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A197" t="s">
         <v>378</v>
       </c>
-      <c r="B197" s="1" t="s">
+      <c r="B197" t="s">
         <v>379</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="18.75">
-      <c r="A198" s="1" t="s">
+    <row r="198" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A198" t="s">
         <v>380</v>
       </c>
-      <c r="B198" s="1" t="s">
+      <c r="B198" t="s">
         <v>381</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="18.75">
-      <c r="A199" s="1" t="s">
+    <row r="199" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A199" t="s">
         <v>382</v>
       </c>
-      <c r="B199" s="1" t="s">
+      <c r="B199" t="s">
         <v>383</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="18.75">
-      <c r="A200" s="1" t="s">
+    <row r="200" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A200" t="s">
         <v>384</v>
       </c>
-      <c r="B200" s="1" t="s">
+      <c r="B200" t="s">
         <v>385</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="18.75">
-      <c r="A201" s="1" t="s">
+    <row r="201" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A201" t="s">
         <v>386</v>
       </c>
-      <c r="B201" s="1" t="s">
+      <c r="B201" t="s">
         <v>387</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="18.75">
-      <c r="A202" s="2" t="s">
+    <row r="202" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A202" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="B202" s="2" t="s">
+      <c r="B202" s="1" t="s">
         <v>389</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="18.75">
-      <c r="A203" s="1" t="s">
+    <row r="203" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A203" t="s">
         <v>390</v>
       </c>
-      <c r="B203" s="1" t="s">
+      <c r="B203" t="s">
         <v>391</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="18.75">
-      <c r="A204" s="1" t="s">
+    <row r="204" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A204" t="s">
         <v>392</v>
       </c>
-      <c r="B204" s="1" t="s">
+      <c r="B204" t="s">
         <v>393</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="18.75">
-      <c r="A205" s="1" t="s">
+    <row r="205" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A205" t="s">
         <v>394</v>
       </c>
-      <c r="B205" s="1" t="s">
+      <c r="B205" t="s">
         <v>395</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="18.75">
-      <c r="A206" s="1" t="s">
+    <row r="206" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A206" t="s">
         <v>396</v>
       </c>
-      <c r="B206" s="1" t="s">
+      <c r="B206" t="s">
         <v>397</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="18.75">
-      <c r="A207" s="1" t="s">
+    <row r="207" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A207" t="s">
         <v>398</v>
       </c>
-      <c r="B207" s="1" t="s">
+      <c r="B207" t="s">
         <v>399</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="18.75">
-      <c r="A208" s="1" t="s">
+    <row r="208" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A208" t="s">
         <v>400</v>
       </c>
-      <c r="B208" s="1" t="s">
+      <c r="B208" t="s">
         <v>401</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="209" customHeight="1" ht="18.75">
-      <c r="A209" s="1" t="s">
+    <row r="209" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A209" t="s">
         <v>402</v>
       </c>
-      <c r="B209" s="1" t="s">
+      <c r="B209" t="s">
         <v>403</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="210" customHeight="1" ht="18.75">
-      <c r="A210" s="1" t="s">
+    <row r="210" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A210" t="s">
         <v>404</v>
       </c>
-      <c r="B210" s="1" t="s">
+      <c r="B210" t="s">
         <v>405</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="211" customHeight="1" ht="18.75">
-      <c r="A211" s="1" t="s">
+    <row r="211" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A211" t="s">
         <v>406</v>
       </c>
-      <c r="B211" s="1" t="s">
+      <c r="B211" t="s">
         <v>47</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="212" customHeight="1" ht="18.75">
-      <c r="A212" s="1" t="s">
+    <row r="212" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A212" t="s">
         <v>407</v>
       </c>
-      <c r="B212" s="1" t="s">
+      <c r="B212" t="s">
         <v>49</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="213" customHeight="1" ht="18.75">
-      <c r="A213" s="1" t="s">
+    <row r="213" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A213" t="s">
         <v>408</v>
       </c>
-      <c r="B213" s="1" t="s">
+      <c r="B213" t="s">
         <v>409</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="214" customHeight="1" ht="18.75">
-      <c r="A214" s="1" t="s">
+    <row r="214" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A214" t="s">
         <v>410</v>
       </c>
-      <c r="B214" s="1" t="s">
+      <c r="B214" t="s">
         <v>411</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="215" customHeight="1" ht="18.75">
-      <c r="A215" s="1" t="s">
+    <row r="215" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A215" t="s">
         <v>412</v>
       </c>
-      <c r="B215" s="1" t="s">
+      <c r="B215" t="s">
         <v>413</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="216" customHeight="1" ht="18.75">
-      <c r="A216" s="1" t="s">
+    <row r="216" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A216" t="s">
         <v>414</v>
       </c>
-      <c r="B216" s="1" t="s">
+      <c r="B216" t="s">
         <v>415</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="217" customHeight="1" ht="18.75">
-      <c r="A217" s="1" t="s">
+    <row r="217" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A217" t="s">
         <v>416</v>
       </c>
-      <c r="B217" s="1" t="s">
+      <c r="B217" t="s">
         <v>417</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="218" customHeight="1" ht="18.75">
-      <c r="A218" s="2" t="s">
+    <row r="218" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A218" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="B218" s="2" t="s">
+      <c r="B218" s="1" t="s">
         <v>419</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="219" customHeight="1" ht="18.75">
-      <c r="A219" s="2" t="s">
+    <row r="219" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A219" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="B219" s="2" t="s">
+      <c r="B219" s="1" t="s">
         <v>421</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="220" customHeight="1" ht="18.75">
-      <c r="A220" s="1" t="s">
+    <row r="220" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A220" t="s">
         <v>422</v>
       </c>
-      <c r="B220" s="1" t="s">
+      <c r="B220" t="s">
         <v>423</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="221" customHeight="1" ht="18.75">
-      <c r="A221" s="1" t="s">
+    <row r="221" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A221" t="s">
         <v>424</v>
       </c>
-      <c r="B221" s="1" t="s">
+      <c r="B221" t="s">
         <v>425</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="222" customHeight="1" ht="18.75">
-      <c r="A222" s="1" t="s">
+    <row r="222" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A222" t="s">
         <v>426</v>
       </c>
-      <c r="B222" s="1" t="s">
+      <c r="B222" t="s">
         <v>427</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="223" customHeight="1" ht="18.75">
-      <c r="A223" s="1" t="s">
+    <row r="223" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A223" t="s">
         <v>428</v>
       </c>
-      <c r="B223" s="1" t="s">
+      <c r="B223" t="s">
         <v>429</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="224" customHeight="1" ht="18.75">
-      <c r="A224" s="1" t="s">
+    <row r="224" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A224" t="s">
         <v>430</v>
       </c>
-      <c r="B224" s="1" t="s">
+      <c r="B224" t="s">
         <v>431</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="225" customHeight="1" ht="18.75">
-      <c r="A225" s="1" t="s">
+    <row r="225" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A225" t="s">
         <v>432</v>
       </c>
-      <c r="B225" s="1" t="s">
+      <c r="B225" t="s">
         <v>433</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="226" customHeight="1" ht="18.75">
-      <c r="A226" s="1" t="s">
+    <row r="226" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A226" t="s">
         <v>434</v>
       </c>
-      <c r="B226" s="1" t="s">
+      <c r="B226" t="s">
         <v>435</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="227" customHeight="1" ht="18.75">
-      <c r="A227" s="1" t="s">
+    <row r="227" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A227" t="s">
+        <v>553</v>
+      </c>
+      <c r="B227" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A228" t="s">
+        <v>551</v>
+      </c>
+      <c r="B228" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A229" t="s">
+        <v>554</v>
+      </c>
+      <c r="B229" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A230" t="s">
         <v>436</v>
       </c>
-      <c r="B227" s="1" t="s">
+      <c r="B230" t="s">
         <v>437</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="228" customHeight="1" ht="18.75">
-      <c r="A228" s="1" t="s">
+    <row r="231" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A231" t="s">
         <v>438</v>
       </c>
-      <c r="B228" s="1" t="s">
+      <c r="B231" t="s">
         <v>439</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="229" customHeight="1" ht="18.75">
-      <c r="A229" s="1" t="s">
+    <row r="232" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A232" t="s">
         <v>440</v>
       </c>
-      <c r="B229" s="1" t="s">
+      <c r="B232" t="s">
         <v>441</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="230" customHeight="1" ht="18.75">
-      <c r="A230" s="1" t="s">
+    <row r="233" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A233" t="s">
         <v>442</v>
       </c>
-      <c r="B230" s="1" t="s">
+      <c r="B233" t="s">
         <v>443</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="231" customHeight="1" ht="18.75">
-      <c r="A231" s="1" t="s">
+    <row r="234" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A234" t="s">
         <v>444</v>
       </c>
-      <c r="B231" s="1" t="s">
+      <c r="B234" t="s">
         <v>445</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="232" customHeight="1" ht="18.75">
-      <c r="A232" s="1" t="s">
+    <row r="235" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A235" t="s">
         <v>446</v>
       </c>
-      <c r="B232" s="1" t="s">
+      <c r="B235" t="s">
         <v>447</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="233" customHeight="1" ht="18.75">
-      <c r="A233" s="1" t="s">
+    <row r="236" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A236" t="s">
         <v>448</v>
       </c>
-      <c r="B233" s="1" t="s">
+      <c r="B236" t="s">
         <v>449</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="234" customHeight="1" ht="18.75">
-      <c r="A234" s="1" t="s">
+    <row r="237" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A237" t="s">
         <v>450</v>
       </c>
-      <c r="B234" s="1" t="s">
+      <c r="B237" t="s">
         <v>451</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="235" customHeight="1" ht="18.75">
-      <c r="A235" s="1" t="s">
+    <row r="238" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A238" t="s">
         <v>452</v>
       </c>
-      <c r="B235" s="1" t="s">
+      <c r="B238" t="s">
         <v>453</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="236" customHeight="1" ht="18.75">
-      <c r="A236" s="1" t="s">
+    <row r="239" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A239" t="s">
         <v>454</v>
       </c>
-      <c r="B236" s="1" t="s">
+      <c r="B239" t="s">
         <v>455</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="237" customHeight="1" ht="18.75">
-      <c r="A237" s="1" t="s">
+    <row r="240" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A240" t="s">
         <v>456</v>
       </c>
-      <c r="B237" s="1" t="s">
+      <c r="B240" t="s">
         <v>457</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="238" customHeight="1" ht="18.75">
-      <c r="A238" s="1" t="s">
+    <row r="241" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A241" t="s">
         <v>458</v>
       </c>
-      <c r="B238" s="1" t="s">
+      <c r="B241" t="s">
         <v>459</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="239" customHeight="1" ht="18.75">
-      <c r="A239" s="1" t="s">
+    <row r="242" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A242" t="s">
         <v>460</v>
       </c>
-      <c r="B239" s="1" t="s">
+      <c r="B242" t="s">
         <v>461</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="240" customHeight="1" ht="18.75">
-      <c r="A240" s="1" t="s">
+    <row r="243" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A243" t="s">
         <v>462</v>
       </c>
-      <c r="B240" s="1" t="s">
+      <c r="B243" t="s">
         <v>463</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="241" customHeight="1" ht="18.75">
-      <c r="A241" s="1" t="s">
+    <row r="244" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A244" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="B241" s="1" t="s">
+      <c r="B244" s="2" t="s">
         <v>465</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="242" customHeight="1" ht="18.75">
-      <c r="A242" s="1" t="s">
+    <row r="245" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A245" t="s">
         <v>466</v>
       </c>
-      <c r="B242" s="1" t="s">
+      <c r="B245" t="s">
         <v>467</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="243" customHeight="1" ht="18.75">
-      <c r="A243" s="1" t="s">
+    <row r="246" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A246" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="B243" s="1" t="s">
+      <c r="B246" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="244" customHeight="1" ht="18.75">
-      <c r="A244" s="2" t="s">
+    <row r="247" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A247" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="B244" s="2" t="s">
+      <c r="B247" s="1" t="s">
         <v>470</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="245" customHeight="1" ht="18.75">
-      <c r="A245" s="1" t="s">
+    <row r="248" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A248" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="B245" s="1" t="s">
+      <c r="B248" s="2" t="s">
         <v>472</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="246" customHeight="1" ht="18.75">
-      <c r="A246" s="2" t="s">
+    <row r="249" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A249" s="4" t="s">
         <v>473</v>
       </c>
-      <c r="B246" s="2" t="s">
+      <c r="B249" s="4" t="s">
         <v>474</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="247" customHeight="1" ht="18.75">
-      <c r="A247" s="2" t="s">
+    <row r="250" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A250" s="4" t="s">
         <v>475</v>
       </c>
-      <c r="B247" s="2" t="s">
+      <c r="B250" s="4" t="s">
         <v>476</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="248" customHeight="1" ht="18.75">
-      <c r="A248" s="2" t="s">
+    <row r="251" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A251" s="3" t="s">
         <v>477</v>
       </c>
-      <c r="B248" s="2" t="s">
+      <c r="B251" s="3" t="s">
         <v>478</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="249" customHeight="1" ht="18.75">
-      <c r="A249" s="1" t="s">
+    <row r="252" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A252" t="s">
         <v>479</v>
       </c>
-      <c r="B249" s="1" t="s">
+      <c r="B252" t="s">
         <v>480</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="250" customHeight="1" ht="18.75">
-      <c r="A250" s="1" t="s">
+    <row r="253" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A253" t="s">
         <v>481</v>
       </c>
-      <c r="B250" s="1" t="s">
+      <c r="B253" t="s">
         <v>482</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="251" customHeight="1" ht="18.75">
-      <c r="A251" s="1" t="s">
+    <row r="254" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A254" t="s">
         <v>483</v>
       </c>
-      <c r="B251" s="1" t="s">
+      <c r="B254" t="s">
         <v>484</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="252" customHeight="1" ht="18.75">
-      <c r="A252" s="1" t="s">
+    <row r="255" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A255" t="s">
         <v>485</v>
       </c>
-      <c r="B252" s="1" t="s">
+      <c r="B255" t="s">
         <v>486</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="253" customHeight="1" ht="18.75">
-      <c r="A253" s="1" t="s">
+    <row r="256" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A256" s="2" t="s">
         <v>487</v>
       </c>
-      <c r="B253" s="1" t="s">
+      <c r="B256" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="254" customHeight="1" ht="18.75">
-      <c r="A254" s="1" t="s">
+    <row r="257" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A257" t="s">
         <v>488</v>
       </c>
-      <c r="B254" s="1" t="s">
+      <c r="B257" t="s">
         <v>489</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="255" customHeight="1" ht="18.75">
-      <c r="A255" s="1" t="s">
+    <row r="258" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A258" s="5" t="s">
         <v>490</v>
       </c>
-      <c r="B255" s="1" t="s">
+      <c r="B258" s="5" t="s">
         <v>491</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="256" customHeight="1" ht="18.75">
-      <c r="A256" s="2" t="s">
+    <row r="259" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A259" s="3" t="s">
         <v>492</v>
       </c>
-      <c r="B256" s="2" t="s">
+      <c r="B259" s="3" t="s">
         <v>493</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="257" customHeight="1" ht="18.75">
-      <c r="A257" s="1" t="s">
+    <row r="260" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A260" t="s">
         <v>494</v>
       </c>
-      <c r="B257" s="1" t="s">
+      <c r="B260" t="s">
         <v>495</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="258" customHeight="1" ht="18.75">
-      <c r="A258" s="1" t="s">
+    <row r="261" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A261" t="s">
         <v>496</v>
       </c>
-      <c r="B258" s="1" t="s">
+      <c r="B261" t="s">
         <v>497</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="259" customHeight="1" ht="18.75">
-      <c r="A259" s="1" t="s">
+    <row r="262" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A262" t="s">
         <v>498</v>
       </c>
-      <c r="B259" s="1" t="s">
+      <c r="B262" t="s">
         <v>277</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="260" customHeight="1" ht="18.75">
-      <c r="A260" s="1" t="s">
+    <row r="263" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A263" t="s">
         <v>499</v>
       </c>
-      <c r="B260" s="1" t="s">
+      <c r="B263" t="s">
         <v>500</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="18.75">
-      <c r="A261" s="1" t="s">
+    <row r="264" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A264" t="s">
         <v>501</v>
       </c>
-      <c r="B261" s="1" t="s">
+      <c r="B264" t="s">
         <v>502</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="18.75">
-      <c r="A262" s="1" t="s">
+    <row r="265" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A265" t="s">
         <v>503</v>
       </c>
-      <c r="B262" s="1" t="s">
+      <c r="B265" t="s">
         <v>504</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="263" customHeight="1" ht="18.75">
-      <c r="A263" s="1" t="s">
+    <row r="266" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A266" t="s">
         <v>505</v>
       </c>
-      <c r="B263" s="1" t="s">
+      <c r="B266" t="s">
         <v>506</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="264" customHeight="1" ht="18.75">
-      <c r="A264" s="1" t="s">
+    <row r="267" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A267" t="s">
         <v>507</v>
       </c>
-      <c r="B264" s="1" t="s">
+      <c r="B267" t="s">
         <v>508</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="265" customHeight="1" ht="18.75">
-      <c r="A265" s="1" t="s">
+    <row r="268" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A268" t="s">
         <v>509</v>
       </c>
-      <c r="B265" s="1" t="s">
+      <c r="B268" t="s">
         <v>510</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="266" customHeight="1" ht="18.75">
-      <c r="A266" s="1" t="s">
+    <row r="269" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A269" t="s">
         <v>511</v>
       </c>
-      <c r="B266" s="1" t="s">
+      <c r="B269" t="s">
         <v>512</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="267" customHeight="1" ht="18.75">
-      <c r="A267" s="1" t="s">
+    <row r="270" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A270" t="s">
         <v>513</v>
       </c>
-      <c r="B267" s="1" t="s">
+      <c r="B270" t="s">
         <v>514</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="268" customHeight="1" ht="18.75">
-      <c r="A268" s="1" t="s">
+    <row r="271" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A271" t="s">
         <v>515</v>
       </c>
-      <c r="B268" s="1" t="s">
+      <c r="B271" t="s">
         <v>516</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="269" customHeight="1" ht="18.75">
-      <c r="A269" s="1" t="s">
+    <row r="272" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A272" s="2" t="s">
         <v>517</v>
       </c>
-      <c r="B269" s="1" t="s">
+      <c r="B272" s="2" t="s">
         <v>518</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="270" customHeight="1" ht="18.75">
-      <c r="A270" s="1" t="s">
+    <row r="273" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A273" t="s">
         <v>519</v>
       </c>
-      <c r="B270" s="1" t="s">
+      <c r="B273" t="s">
         <v>520</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="271" customHeight="1" ht="18.75">
-      <c r="A271" s="1" t="s">
+    <row r="274" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A274" s="5" t="s">
         <v>521</v>
       </c>
-      <c r="B271" s="1" t="s">
+      <c r="B274" s="5" t="s">
         <v>522</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="18.75">
-      <c r="A272" s="2" t="s">
+    <row r="275" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A275" s="3" t="s">
         <v>523</v>
       </c>
-      <c r="B272" s="2" t="s">
+      <c r="B275" s="3" t="s">
         <v>524</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="273" customHeight="1" ht="18.75">
-      <c r="A273" s="1" t="s">
+    <row r="276" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A276" s="2" t="s">
         <v>525</v>
       </c>
-      <c r="B273" s="1" t="s">
+      <c r="B276" s="2" t="s">
         <v>526</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="18.75">
-      <c r="A274" s="1" t="s">
+    <row r="277" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A277" t="s">
         <v>527</v>
       </c>
-      <c r="B274" s="1" t="s">
+      <c r="B277" t="s">
         <v>528</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="275" customHeight="1" ht="18.75">
-      <c r="A275" s="1" t="s">
+    <row r="278" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A278" s="5" t="s">
         <v>529</v>
       </c>
-      <c r="B275" s="1" t="s">
+      <c r="B278" s="5" t="s">
         <v>530</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="276" customHeight="1" ht="18.75">
-      <c r="A276" s="2" t="s">
+    <row r="279" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A279" s="3" t="s">
         <v>531</v>
       </c>
-      <c r="B276" s="2" t="s">
+      <c r="B279" s="3" t="s">
         <v>532</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="277" customHeight="1" ht="18.75">
-      <c r="A277" s="1" t="s">
+    <row r="280" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A280" t="s">
         <v>533</v>
       </c>
-      <c r="B277" s="1" t="s">
+      <c r="B280" t="s">
         <v>534</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="18.75">
-      <c r="A278" s="1" t="s">
+    <row r="281" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A281" t="s">
         <v>535</v>
       </c>
-      <c r="B278" s="1" t="s">
+      <c r="B281" t="s">
         <v>536</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="279" customHeight="1" ht="18.75">
-      <c r="A279" s="1" t="s">
+    <row r="282" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A282" t="s">
         <v>537</v>
       </c>
-      <c r="B279" s="1" t="s">
+      <c r="B282" t="s">
         <v>538</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="280" customHeight="1" ht="18.75">
-      <c r="A280" s="1" t="s">
+    <row r="283" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A283" t="s">
         <v>539</v>
       </c>
-      <c r="B280" s="1" t="s">
+      <c r="B283" t="s">
         <v>540</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="281" customHeight="1" ht="18.75">
-      <c r="A281" s="1" t="s">
+    <row r="284" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A284" t="s">
         <v>541</v>
       </c>
-      <c r="B281" s="1" t="s">
+      <c r="B284" t="s">
         <v>542</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="282" customHeight="1" ht="18.75">
-      <c r="A282" s="1" t="s">
+    <row r="285" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A285" t="s">
         <v>543</v>
       </c>
-      <c r="B282" s="1" t="s">
+      <c r="B285" t="s">
         <v>544</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="283" customHeight="1" ht="18.75">
-      <c r="A283" s="1" t="s">
+    <row r="286" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A286" t="s">
         <v>545</v>
       </c>
-      <c r="B283" s="1" t="s">
+      <c r="B286" t="s">
         <v>546</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="284" customHeight="1" ht="18.75">
-      <c r="A284" s="1" t="s">
+    <row r="287" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A287" t="s">
         <v>547</v>
       </c>
-      <c r="B284" s="1" t="s">
+      <c r="B287" t="s">
         <v>548</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="285" customHeight="1" ht="18.75">
-      <c r="A285" s="1" t="s">
+    <row r="288" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A288" t="s">
         <v>549</v>
       </c>
-      <c r="B285" s="1" t="s">
+      <c r="B288" t="s">
         <v>550</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B288" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B288">
+      <sortCondition ref="A1:A288"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Generic Medication Dispensed Report (#242)
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -1,23 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10921"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/salmanraza/Documents/GitHub/tamanu-source-dbt/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C960FFE9-82F0-894D-A44C-58483C095E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Translated String"/>
+    <sheet name="Translated String" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Translated String'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Translated String'!$A$1:$B$1</definedName>
   </definedNames>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="561">
   <si>
     <t>stringId</t>
   </si>
@@ -1682,13 +1688,30 @@
   </si>
   <si>
     <t>Schedule</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedication</t>
+  </si>
+  <si>
+    <t>Medication</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedicationCode</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionQuantity</t>
+  </si>
+  <si>
+    <t>Quantity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1732,25 +1755,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1761,10 +1785,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -1802,71 +1826,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1894,7 +1918,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1917,11 +1941,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1930,13 +1954,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1946,7 +1970,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1955,7 +1979,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1964,7 +1988,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1972,10 +1996,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -2040,2314 +2064,2343 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B287"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B290"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" style="3" width="58.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="58.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>27</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>33</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="1" t="s">
+    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>35</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="1" t="s">
+    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>37</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="1" t="s">
+    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="1" t="s">
+    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>41</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="1" t="s">
+    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>43</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="1" t="s">
+    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>45</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="1" t="s">
+    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="1" t="s">
+    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" t="s">
         <v>49</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="1" t="s">
+    <row r="26" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" t="s">
         <v>51</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
-      <c r="A27" s="1" t="s">
+    <row r="27" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
         <v>53</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
-      <c r="A28" s="1" t="s">
+    <row r="28" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>55</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
-      <c r="A29" s="1" t="s">
+    <row r="29" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" t="s">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
-      <c r="A30" s="1" t="s">
+    <row r="30" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" t="s">
         <v>58</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
-      <c r="A31" s="1" t="s">
+    <row r="31" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
         <v>59</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>60</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
-      <c r="A32" s="1" t="s">
+    <row r="32" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>61</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
         <v>62</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="1" t="s">
+    <row r="33" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
         <v>63</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" t="s">
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
-      <c r="A34" s="1" t="s">
+    <row r="34" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
         <v>64</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" t="s">
         <v>65</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
-      <c r="A35" s="1" t="s">
+    <row r="35" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
         <v>66</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" t="s">
         <v>67</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
-      <c r="A36" s="1" t="s">
+    <row r="36" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" t="s">
         <v>69</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
-      <c r="A37" s="1" t="s">
+    <row r="37" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
         <v>70</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" t="s">
         <v>71</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
-      <c r="A38" s="1" t="s">
+    <row r="38" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
         <v>72</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" t="s">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
-      <c r="A39" s="1" t="s">
+    <row r="39" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
         <v>73</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" t="s">
         <v>74</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
-      <c r="A40" s="1" t="s">
+    <row r="40" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
         <v>75</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" t="s">
         <v>76</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
-      <c r="A41" s="1" t="s">
+    <row r="41" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
         <v>77</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" t="s">
         <v>78</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
-      <c r="A42" s="1" t="s">
+    <row r="42" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
         <v>79</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" t="s">
         <v>80</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
-      <c r="A43" s="1" t="s">
+    <row r="43" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
         <v>81</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" t="s">
         <v>82</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
-      <c r="A44" s="1" t="s">
+    <row r="44" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
         <v>83</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" t="s">
         <v>84</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
-      <c r="A45" s="1" t="s">
+    <row r="45" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
         <v>85</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" t="s">
         <v>86</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
-      <c r="A46" s="1" t="s">
+    <row r="46" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
         <v>87</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" t="s">
         <v>88</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
-      <c r="A47" s="1" t="s">
+    <row r="47" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>89</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" t="s">
         <v>90</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
-      <c r="A48" s="1" t="s">
+    <row r="48" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
         <v>91</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" t="s">
         <v>92</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
-      <c r="A49" s="1" t="s">
+    <row r="49" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
         <v>93</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" t="s">
         <v>94</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
-      <c r="A50" s="1" t="s">
+    <row r="50" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
         <v>95</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" t="s">
         <v>96</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
-      <c r="A51" s="1" t="s">
+    <row r="51" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
         <v>97</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" t="s">
         <v>98</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
-      <c r="A52" s="1" t="s">
+    <row r="52" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
         <v>99</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" t="s">
         <v>100</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
-      <c r="A53" s="1" t="s">
+    <row r="53" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
         <v>101</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" t="s">
         <v>102</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
-      <c r="A54" s="1" t="s">
+    <row r="54" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
         <v>103</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" t="s">
         <v>104</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
-      <c r="A55" s="1" t="s">
+    <row r="55" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
         <v>105</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" t="s">
         <v>106</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
-      <c r="A56" s="1" t="s">
+    <row r="56" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
         <v>107</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" t="s">
         <v>108</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
-      <c r="A57" s="1" t="s">
+    <row r="57" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
         <v>109</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" t="s">
         <v>110</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
-      <c r="A58" s="1" t="s">
+    <row r="58" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
         <v>111</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" t="s">
         <v>112</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
-      <c r="A59" s="1" t="s">
+    <row r="59" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
         <v>113</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" t="s">
         <v>114</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
-      <c r="A60" s="1" t="s">
+    <row r="60" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
         <v>115</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B60" t="s">
         <v>116</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
-      <c r="A61" s="1" t="s">
+    <row r="61" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
         <v>117</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" t="s">
         <v>118</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
-      <c r="A62" s="1" t="s">
+    <row r="62" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
         <v>119</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B62" t="s">
         <v>120</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
-      <c r="A63" s="1" t="s">
+    <row r="63" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
         <v>121</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B63" t="s">
         <v>122</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
-      <c r="A64" s="1" t="s">
+    <row r="64" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
         <v>123</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B64" t="s">
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
-      <c r="A65" s="1" t="s">
+    <row r="65" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
         <v>125</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="B65" t="s">
         <v>126</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
-      <c r="A66" s="1" t="s">
+    <row r="66" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
         <v>127</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B66" t="s">
         <v>128</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
-      <c r="A67" s="1" t="s">
+    <row r="67" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
         <v>129</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B67" t="s">
         <v>130</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
-      <c r="A68" s="1" t="s">
+    <row r="68" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
         <v>131</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B68" t="s">
         <v>132</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
-      <c r="A69" s="1" t="s">
+    <row r="69" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
         <v>133</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B69" t="s">
         <v>134</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
-      <c r="A70" s="1" t="s">
+    <row r="70" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
         <v>135</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="B70" t="s">
         <v>136</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
-      <c r="A71" s="1" t="s">
+    <row r="71" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
         <v>137</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B71" t="s">
         <v>138</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
-      <c r="A72" s="1" t="s">
+    <row r="72" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
         <v>139</v>
       </c>
-      <c r="B72" s="1" t="s">
+      <c r="B72" t="s">
         <v>140</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
-      <c r="A73" s="1" t="s">
+    <row r="73" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
         <v>141</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="B73" t="s">
         <v>142</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
-      <c r="A74" s="1" t="s">
+    <row r="74" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
         <v>143</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="B74" t="s">
         <v>144</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
-      <c r="A75" s="1" t="s">
+    <row r="75" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
         <v>145</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B75" t="s">
         <v>146</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
-      <c r="A76" s="1" t="s">
+    <row r="76" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
         <v>147</v>
       </c>
-      <c r="B76" s="1" t="s">
+      <c r="B76" t="s">
         <v>148</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
-      <c r="A77" s="1" t="s">
+    <row r="77" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
         <v>149</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="B77" t="s">
         <v>150</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
-      <c r="A78" s="1" t="s">
+    <row r="78" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
         <v>151</v>
       </c>
-      <c r="B78" s="1" t="s">
+      <c r="B78" t="s">
         <v>152</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
-      <c r="A79" s="1" t="s">
+    <row r="79" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
         <v>153</v>
       </c>
-      <c r="B79" s="1" t="s">
+      <c r="B79" t="s">
         <v>154</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
-      <c r="A80" s="1" t="s">
+    <row r="80" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
         <v>155</v>
       </c>
-      <c r="B80" s="1" t="s">
+      <c r="B80" t="s">
         <v>156</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
-      <c r="A81" s="1" t="s">
+    <row r="81" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
         <v>157</v>
       </c>
-      <c r="B81" s="1" t="s">
+      <c r="B81" t="s">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
-      <c r="A82" s="1" t="s">
+    <row r="82" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
         <v>158</v>
       </c>
-      <c r="B82" s="1" t="s">
+      <c r="B82" t="s">
         <v>159</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
-      <c r="A83" s="1" t="s">
+    <row r="83" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
         <v>160</v>
       </c>
-      <c r="B83" s="1" t="s">
+      <c r="B83" t="s">
         <v>161</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
-      <c r="A84" s="1" t="s">
+    <row r="84" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
         <v>162</v>
       </c>
-      <c r="B84" s="1" t="s">
+      <c r="B84" t="s">
         <v>163</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
-      <c r="A85" s="1" t="s">
+    <row r="85" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
         <v>164</v>
       </c>
-      <c r="B85" s="1" t="s">
+      <c r="B85" t="s">
         <v>165</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
-      <c r="A86" s="1" t="s">
+    <row r="86" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
         <v>166</v>
       </c>
-      <c r="B86" s="1" t="s">
+      <c r="B86" t="s">
         <v>167</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
-      <c r="A87" s="1" t="s">
+    <row r="87" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
         <v>168</v>
       </c>
-      <c r="B87" s="1" t="s">
+      <c r="B87" t="s">
         <v>169</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
-      <c r="A88" s="1" t="s">
+    <row r="88" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
         <v>170</v>
       </c>
-      <c r="B88" s="1" t="s">
+      <c r="B88" t="s">
         <v>171</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
-      <c r="A89" s="1" t="s">
+    <row r="89" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
         <v>172</v>
       </c>
-      <c r="B89" s="1" t="s">
+      <c r="B89" t="s">
         <v>173</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
-      <c r="A90" s="1" t="s">
+    <row r="90" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
         <v>174</v>
       </c>
-      <c r="B90" s="1" t="s">
+      <c r="B90" t="s">
         <v>175</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
-      <c r="A91" s="1" t="s">
+    <row r="91" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
         <v>176</v>
       </c>
-      <c r="B91" s="1" t="s">
+      <c r="B91" t="s">
         <v>177</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
-      <c r="A92" s="1" t="s">
+    <row r="92" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
         <v>178</v>
       </c>
-      <c r="B92" s="1" t="s">
+      <c r="B92" t="s">
         <v>179</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
-      <c r="A93" s="1" t="s">
+    <row r="93" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
         <v>180</v>
       </c>
-      <c r="B93" s="1" t="s">
+      <c r="B93" t="s">
         <v>181</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
-      <c r="A94" s="1" t="s">
+    <row r="94" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
         <v>182</v>
       </c>
-      <c r="B94" s="1" t="s">
+      <c r="B94" t="s">
         <v>183</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
-      <c r="A95" s="1" t="s">
+    <row r="95" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
         <v>184</v>
       </c>
-      <c r="B95" s="1" t="s">
+      <c r="B95" t="s">
         <v>185</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
-      <c r="A96" s="1" t="s">
+    <row r="96" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
         <v>186</v>
       </c>
-      <c r="B96" s="1" t="s">
+      <c r="B96" t="s">
         <v>187</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
-      <c r="A97" s="1" t="s">
+    <row r="97" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
         <v>188</v>
       </c>
-      <c r="B97" s="1" t="s">
+      <c r="B97" t="s">
         <v>189</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
-      <c r="A98" s="1" t="s">
+    <row r="98" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
         <v>190</v>
       </c>
-      <c r="B98" s="1" t="s">
+      <c r="B98" t="s">
         <v>191</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
-      <c r="A99" s="1" t="s">
+    <row r="99" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
         <v>192</v>
       </c>
-      <c r="B99" s="1" t="s">
+      <c r="B99" t="s">
         <v>193</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
-      <c r="A100" s="1" t="s">
+    <row r="100" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
         <v>194</v>
       </c>
-      <c r="B100" s="1" t="s">
+      <c r="B100" t="s">
         <v>195</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
-      <c r="A101" s="1" t="s">
+    <row r="101" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
         <v>196</v>
       </c>
-      <c r="B101" s="1" t="s">
+      <c r="B101" t="s">
         <v>197</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
-      <c r="A102" s="1" t="s">
+    <row r="102" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
         <v>198</v>
       </c>
-      <c r="B102" s="1" t="s">
+      <c r="B102" t="s">
         <v>199</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
-      <c r="A103" s="1" t="s">
+    <row r="103" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
         <v>200</v>
       </c>
-      <c r="B103" s="1" t="s">
+      <c r="B103" t="s">
         <v>201</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
-      <c r="A104" s="1" t="s">
+    <row r="104" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
         <v>202</v>
       </c>
-      <c r="B104" s="1" t="s">
+      <c r="B104" t="s">
         <v>203</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
-      <c r="A105" s="1" t="s">
+    <row r="105" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
         <v>204</v>
       </c>
-      <c r="B105" s="1" t="s">
+      <c r="B105" t="s">
         <v>205</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
-      <c r="A106" s="1" t="s">
+    <row r="106" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
         <v>206</v>
       </c>
-      <c r="B106" s="1" t="s">
+      <c r="B106" t="s">
         <v>207</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
-      <c r="A107" s="1" t="s">
+    <row r="107" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
         <v>208</v>
       </c>
-      <c r="B107" s="1" t="s">
+      <c r="B107" t="s">
         <v>209</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75">
-      <c r="A108" s="1" t="s">
+    <row r="108" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
         <v>210</v>
       </c>
-      <c r="B108" s="1" t="s">
+      <c r="B108" t="s">
         <v>211</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75">
-      <c r="A109" s="1" t="s">
+    <row r="109" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
         <v>212</v>
       </c>
-      <c r="B109" s="1" t="s">
+      <c r="B109" t="s">
         <v>213</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
-      <c r="A110" s="1" t="s">
+    <row r="110" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
         <v>214</v>
       </c>
-      <c r="B110" s="1" t="s">
+      <c r="B110" t="s">
         <v>215</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
-      <c r="A111" s="1" t="s">
+    <row r="111" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
         <v>216</v>
       </c>
-      <c r="B111" s="1" t="s">
+      <c r="B111" t="s">
         <v>217</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
-      <c r="A112" s="1" t="s">
+    <row r="112" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
         <v>218</v>
       </c>
-      <c r="B112" s="1" t="s">
+      <c r="B112" t="s">
         <v>219</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
-      <c r="A113" s="1" t="s">
+    <row r="113" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
         <v>220</v>
       </c>
-      <c r="B113" s="1" t="s">
+      <c r="B113" t="s">
         <v>221</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
-      <c r="A114" s="1" t="s">
+    <row r="114" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
         <v>222</v>
       </c>
-      <c r="B114" s="1" t="s">
+      <c r="B114" t="s">
         <v>223</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
-      <c r="A115" s="1" t="s">
+    <row r="115" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
         <v>224</v>
       </c>
-      <c r="B115" s="1" t="s">
+      <c r="B115" t="s">
         <v>225</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
-      <c r="A116" s="1" t="s">
+    <row r="116" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
         <v>226</v>
       </c>
-      <c r="B116" s="1" t="s">
+      <c r="B116" t="s">
         <v>227</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
-      <c r="A117" s="1" t="s">
+    <row r="117" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
         <v>228</v>
       </c>
-      <c r="B117" s="1" t="s">
+      <c r="B117" t="s">
         <v>229</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
-      <c r="A118" s="1" t="s">
+    <row r="118" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
         <v>230</v>
       </c>
-      <c r="B118" s="1" t="s">
+      <c r="B118" t="s">
         <v>231</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
-      <c r="A119" s="1" t="s">
+    <row r="119" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
         <v>232</v>
       </c>
-      <c r="B119" s="1" t="s">
+      <c r="B119" t="s">
         <v>233</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
-      <c r="A120" s="1" t="s">
+    <row r="120" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
         <v>234</v>
       </c>
-      <c r="B120" s="1" t="s">
+      <c r="B120" t="s">
         <v>235</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
-      <c r="A121" s="1" t="s">
+    <row r="121" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
         <v>236</v>
       </c>
-      <c r="B121" s="1" t="s">
+      <c r="B121" t="s">
         <v>237</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
-      <c r="A122" s="1" t="s">
+    <row r="122" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
         <v>238</v>
       </c>
-      <c r="B122" s="1" t="s">
+      <c r="B122" t="s">
         <v>239</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
-      <c r="A123" s="1" t="s">
+    <row r="123" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
         <v>240</v>
       </c>
-      <c r="B123" s="1" t="s">
+      <c r="B123" t="s">
         <v>241</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
-      <c r="A124" s="1" t="s">
+    <row r="124" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
         <v>242</v>
       </c>
-      <c r="B124" s="1" t="s">
+      <c r="B124" t="s">
         <v>189</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
-      <c r="A125" s="1" t="s">
+    <row r="125" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
         <v>243</v>
       </c>
-      <c r="B125" s="1" t="s">
+      <c r="B125" t="s">
         <v>244</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
-      <c r="A126" s="1" t="s">
+    <row r="126" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
         <v>245</v>
       </c>
-      <c r="B126" s="1" t="s">
+      <c r="B126" t="s">
         <v>246</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
-      <c r="A127" s="1" t="s">
+    <row r="127" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
         <v>247</v>
       </c>
-      <c r="B127" s="1" t="s">
+      <c r="B127" t="s">
         <v>248</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
-      <c r="A128" s="1" t="s">
+    <row r="128" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
         <v>249</v>
       </c>
-      <c r="B128" s="1" t="s">
+      <c r="B128" t="s">
         <v>250</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
-      <c r="A129" s="1" t="s">
+    <row r="129" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A129" t="s">
         <v>251</v>
       </c>
-      <c r="B129" s="1" t="s">
+      <c r="B129" t="s">
         <v>252</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75">
-      <c r="A130" s="1" t="s">
+    <row r="130" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A130" t="s">
         <v>253</v>
       </c>
-      <c r="B130" s="1" t="s">
+      <c r="B130" t="s">
         <v>254</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18.75">
-      <c r="A131" s="1" t="s">
+    <row r="131" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A131" t="s">
         <v>255</v>
       </c>
-      <c r="B131" s="1" t="s">
+      <c r="B131" t="s">
         <v>256</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18.75">
-      <c r="A132" s="1" t="s">
+    <row r="132" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A132" t="s">
         <v>257</v>
       </c>
-      <c r="B132" s="1" t="s">
+      <c r="B132" t="s">
         <v>258</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="18.75">
-      <c r="A133" s="1" t="s">
+    <row r="133" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A133" t="s">
         <v>259</v>
       </c>
-      <c r="B133" s="1" t="s">
+      <c r="B133" t="s">
         <v>260</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18.75">
-      <c r="A134" s="1" t="s">
+    <row r="134" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A134" t="s">
         <v>261</v>
       </c>
-      <c r="B134" s="1" t="s">
+      <c r="B134" t="s">
         <v>262</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18.75">
-      <c r="A135" s="1" t="s">
+    <row r="135" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A135" t="s">
         <v>263</v>
       </c>
-      <c r="B135" s="1" t="s">
+      <c r="B135" t="s">
         <v>264</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18.75">
-      <c r="A136" s="1" t="s">
+    <row r="136" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A136" t="s">
         <v>265</v>
       </c>
-      <c r="B136" s="1" t="s">
+      <c r="B136" t="s">
         <v>266</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18.75">
-      <c r="A137" s="1" t="s">
+    <row r="137" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A137" t="s">
         <v>267</v>
       </c>
-      <c r="B137" s="1" t="s">
+      <c r="B137" t="s">
         <v>268</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18.75">
-      <c r="A138" s="1" t="s">
+    <row r="138" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A138" t="s">
         <v>269</v>
       </c>
-      <c r="B138" s="1" t="s">
+      <c r="B138" t="s">
         <v>270</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18.75">
-      <c r="A139" s="1" t="s">
+    <row r="139" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A139" t="s">
         <v>271</v>
       </c>
-      <c r="B139" s="1" t="s">
+      <c r="B139" t="s">
         <v>223</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18.75">
-      <c r="A140" s="1" t="s">
+    <row r="140" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A140" t="s">
         <v>272</v>
       </c>
-      <c r="B140" s="1" t="s">
+      <c r="B140" t="s">
         <v>237</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18.75">
-      <c r="A141" s="1" t="s">
+    <row r="141" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A141" t="s">
         <v>273</v>
       </c>
-      <c r="B141" s="1" t="s">
+      <c r="B141" t="s">
         <v>225</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18.75">
-      <c r="A142" s="1" t="s">
+    <row r="142" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A142" t="s">
         <v>274</v>
       </c>
-      <c r="B142" s="1" t="s">
+      <c r="B142" t="s">
         <v>275</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18.75">
-      <c r="A143" s="1" t="s">
+    <row r="143" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A143" t="s">
         <v>276</v>
       </c>
-      <c r="B143" s="1" t="s">
+      <c r="B143" t="s">
         <v>277</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="18.75">
-      <c r="A144" s="1" t="s">
+    <row r="144" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A144" t="s">
         <v>278</v>
       </c>
-      <c r="B144" s="1" t="s">
+      <c r="B144" t="s">
         <v>235</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="18.75">
-      <c r="A145" s="1" t="s">
+    <row r="145" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A145" t="s">
         <v>279</v>
       </c>
-      <c r="B145" s="1" t="s">
+      <c r="B145" t="s">
         <v>244</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="18.75">
-      <c r="A146" s="1" t="s">
+    <row r="146" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A146" t="s">
         <v>280</v>
       </c>
-      <c r="B146" s="1" t="s">
+      <c r="B146" t="s">
         <v>281</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="18.75">
-      <c r="A147" s="1" t="s">
+    <row r="147" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A147" t="s">
         <v>282</v>
       </c>
-      <c r="B147" s="1" t="s">
+      <c r="B147" t="s">
         <v>231</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="18.75">
-      <c r="A148" s="1" t="s">
+    <row r="148" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A148" t="s">
         <v>283</v>
       </c>
-      <c r="B148" s="1" t="s">
+      <c r="B148" t="s">
         <v>284</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="18.75">
-      <c r="A149" s="1" t="s">
+    <row r="149" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A149" t="s">
         <v>285</v>
       </c>
-      <c r="B149" s="1" t="s">
+      <c r="B149" t="s">
         <v>286</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18.75">
-      <c r="A150" s="1" t="s">
+    <row r="150" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A150" t="s">
         <v>287</v>
       </c>
-      <c r="B150" s="1" t="s">
+      <c r="B150" t="s">
         <v>288</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18.75">
-      <c r="A151" s="1" t="s">
+    <row r="151" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A151" t="s">
         <v>289</v>
       </c>
-      <c r="B151" s="1" t="s">
+      <c r="B151" t="s">
         <v>290</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18.75">
-      <c r="A152" s="1" t="s">
+    <row r="152" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A152" t="s">
         <v>291</v>
       </c>
-      <c r="B152" s="1" t="s">
+      <c r="B152" t="s">
         <v>292</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="18.75">
-      <c r="A153" s="1" t="s">
+    <row r="153" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A153" t="s">
         <v>293</v>
       </c>
-      <c r="B153" s="1" t="s">
+      <c r="B153" t="s">
         <v>294</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18.75">
-      <c r="A154" s="1" t="s">
+    <row r="154" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A154" t="s">
         <v>295</v>
       </c>
-      <c r="B154" s="1" t="s">
+      <c r="B154" t="s">
         <v>296</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18.75">
-      <c r="A155" s="1" t="s">
+    <row r="155" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A155" t="s">
         <v>297</v>
       </c>
-      <c r="B155" s="1" t="s">
+      <c r="B155" t="s">
         <v>241</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18.75">
-      <c r="A156" s="1" t="s">
+    <row r="156" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A156" t="s">
         <v>298</v>
       </c>
-      <c r="B156" s="1" t="s">
+      <c r="B156" t="s">
         <v>299</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18.75">
-      <c r="A157" s="1" t="s">
+    <row r="157" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A157" t="s">
         <v>300</v>
       </c>
-      <c r="B157" s="1" t="s">
+      <c r="B157" t="s">
         <v>301</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18.75">
-      <c r="A158" s="1" t="s">
+    <row r="158" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A158" t="s">
         <v>302</v>
       </c>
-      <c r="B158" s="1" t="s">
+      <c r="B158" t="s">
         <v>303</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18.75">
-      <c r="A159" s="1" t="s">
+    <row r="159" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A159" t="s">
         <v>304</v>
       </c>
-      <c r="B159" s="1" t="s">
+      <c r="B159" t="s">
         <v>305</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18.75">
-      <c r="A160" s="1" t="s">
+    <row r="160" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A160" t="s">
         <v>306</v>
       </c>
-      <c r="B160" s="1" t="s">
+      <c r="B160" t="s">
         <v>307</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18.75">
-      <c r="A161" s="1" t="s">
+    <row r="161" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A161" t="s">
         <v>308</v>
       </c>
-      <c r="B161" s="1" t="s">
+      <c r="B161" t="s">
         <v>309</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18.75">
-      <c r="A162" s="1" t="s">
+    <row r="162" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A162" t="s">
         <v>310</v>
       </c>
-      <c r="B162" s="1" t="s">
+      <c r="B162" t="s">
         <v>311</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75">
-      <c r="A163" s="1" t="s">
+    <row r="163" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A163" t="s">
         <v>312</v>
       </c>
-      <c r="B163" s="1" t="s">
+      <c r="B163" t="s">
         <v>313</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75">
-      <c r="A164" s="1" t="s">
+    <row r="164" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A164" t="s">
         <v>314</v>
       </c>
-      <c r="B164" s="1" t="s">
+      <c r="B164" t="s">
         <v>62</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75">
-      <c r="A165" s="1" t="s">
+    <row r="165" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A165" t="s">
         <v>315</v>
       </c>
-      <c r="B165" s="1" t="s">
+      <c r="B165" t="s">
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75">
-      <c r="A166" s="1" t="s">
+    <row r="166" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A166" t="s">
         <v>316</v>
       </c>
-      <c r="B166" s="1" t="s">
+      <c r="B166" t="s">
         <v>317</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75">
-      <c r="A167" s="1" t="s">
+    <row r="167" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A167" t="s">
         <v>318</v>
       </c>
-      <c r="B167" s="1" t="s">
+      <c r="B167" t="s">
         <v>319</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18.75">
-      <c r="A168" s="1" t="s">
+    <row r="168" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A168" t="s">
         <v>320</v>
       </c>
-      <c r="B168" s="1" t="s">
+      <c r="B168" t="s">
         <v>321</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="18.75">
-      <c r="A169" s="1" t="s">
+    <row r="169" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A169" t="s">
         <v>322</v>
       </c>
-      <c r="B169" s="1" t="s">
+      <c r="B169" t="s">
         <v>323</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18.75">
-      <c r="A170" s="1" t="s">
+    <row r="170" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A170" t="s">
         <v>324</v>
       </c>
-      <c r="B170" s="1" t="s">
+      <c r="B170" t="s">
         <v>325</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18.75">
-      <c r="A171" s="1" t="s">
+    <row r="171" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A171" t="s">
         <v>326</v>
       </c>
-      <c r="B171" s="1" t="s">
+      <c r="B171" t="s">
         <v>327</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="19.5">
+    <row r="172" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A173" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="B172" s="2" t="s">
+      <c r="B173" s="3" t="s">
         <v>329</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18.75">
-      <c r="A173" s="1" t="s">
-        <v>330</v>
-      </c>
-      <c r="B173" s="1" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18.75">
-      <c r="A174" s="1" t="s">
+    <row r="174" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A174" t="s">
         <v>332</v>
       </c>
-      <c r="B174" s="1" t="s">
+      <c r="B174" t="s">
         <v>333</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18.75">
-      <c r="A175" s="1" t="s">
+    <row r="175" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A175" t="s">
         <v>334</v>
       </c>
-      <c r="B175" s="1" t="s">
+      <c r="B175" t="s">
         <v>335</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18.75">
-      <c r="A176" s="1" t="s">
+    <row r="176" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A176" t="s">
         <v>336</v>
       </c>
-      <c r="B176" s="1" t="s">
+      <c r="B176" t="s">
         <v>337</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="18.75">
-      <c r="A177" s="1" t="s">
+    <row r="177" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A177" t="s">
         <v>338</v>
       </c>
-      <c r="B177" s="1" t="s">
+      <c r="B177" t="s">
         <v>339</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18.75">
-      <c r="A178" s="1" t="s">
+    <row r="178" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A178" t="s">
         <v>340</v>
       </c>
-      <c r="B178" s="1" t="s">
+      <c r="B178" t="s">
         <v>341</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18.75">
-      <c r="A179" s="1" t="s">
+    <row r="179" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A179" t="s">
         <v>342</v>
       </c>
-      <c r="B179" s="1" t="s">
+      <c r="B179" t="s">
         <v>343</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18.75">
-      <c r="A180" s="1" t="s">
+    <row r="180" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A180" t="s">
         <v>344</v>
       </c>
-      <c r="B180" s="1" t="s">
+      <c r="B180" t="s">
         <v>345</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18.75">
-      <c r="A181" s="1" t="s">
+    <row r="181" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A181" t="s">
         <v>346</v>
       </c>
-      <c r="B181" s="1" t="s">
+      <c r="B181" t="s">
         <v>347</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18.75">
-      <c r="A182" s="1" t="s">
+    <row r="182" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A182" t="s">
         <v>348</v>
       </c>
-      <c r="B182" s="1" t="s">
+      <c r="B182" t="s">
         <v>349</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18.75">
-      <c r="A183" s="1" t="s">
+    <row r="183" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A183" t="s">
         <v>350</v>
       </c>
-      <c r="B183" s="1" t="s">
+      <c r="B183" t="s">
         <v>351</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18.75">
-      <c r="A184" s="2" t="s">
+    <row r="184" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A184" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="B184" s="2" t="s">
+      <c r="B184" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18.75">
-      <c r="A185" s="1" t="s">
+    <row r="185" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A185" t="s">
         <v>354</v>
       </c>
-      <c r="B185" s="1" t="s">
+      <c r="B185" t="s">
         <v>355</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75">
-      <c r="A186" s="1" t="s">
+    <row r="186" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A186" t="s">
         <v>356</v>
       </c>
-      <c r="B186" s="1" t="s">
+      <c r="B186" t="s">
         <v>357</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18.75">
-      <c r="A187" s="1" t="s">
+    <row r="187" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A187" t="s">
         <v>358</v>
       </c>
-      <c r="B187" s="1" t="s">
+      <c r="B187" t="s">
         <v>359</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75">
-      <c r="A188" s="1" t="s">
+    <row r="188" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A188" t="s">
         <v>360</v>
       </c>
-      <c r="B188" s="1" t="s">
+      <c r="B188" t="s">
         <v>361</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75">
-      <c r="A189" s="1" t="s">
+    <row r="189" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A189" t="s">
         <v>362</v>
       </c>
-      <c r="B189" s="1" t="s">
+      <c r="B189" t="s">
         <v>363</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75">
-      <c r="A190" s="1" t="s">
+    <row r="190" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A190" t="s">
         <v>364</v>
       </c>
-      <c r="B190" s="1" t="s">
+      <c r="B190" t="s">
         <v>365</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18.75">
-      <c r="A191" s="1" t="s">
+    <row r="191" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A191" t="s">
         <v>366</v>
       </c>
-      <c r="B191" s="1" t="s">
+      <c r="B191" t="s">
         <v>367</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="18.75">
-      <c r="A192" s="2" t="s">
+    <row r="192" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A192" s="1" t="s">
         <v>368</v>
       </c>
-      <c r="B192" s="2" t="s">
+      <c r="B192" s="1" t="s">
         <v>369</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18.75">
-      <c r="A193" s="1" t="s">
+    <row r="193" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A193" t="s">
         <v>370</v>
       </c>
-      <c r="B193" s="1" t="s">
+      <c r="B193" t="s">
         <v>371</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="18.75">
-      <c r="A194" s="1" t="s">
+    <row r="194" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A194" t="s">
         <v>372</v>
       </c>
-      <c r="B194" s="1" t="s">
+      <c r="B194" t="s">
         <v>373</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18.75">
-      <c r="A195" s="1" t="s">
+    <row r="195" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A195" t="s">
         <v>374</v>
       </c>
-      <c r="B195" s="1" t="s">
+      <c r="B195" t="s">
         <v>375</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="18.75">
-      <c r="A196" s="1" t="s">
+    <row r="196" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A196" t="s">
         <v>376</v>
       </c>
-      <c r="B196" s="1" t="s">
+      <c r="B196" t="s">
         <v>377</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18.75">
-      <c r="A197" s="1" t="s">
+    <row r="197" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A197" t="s">
         <v>378</v>
       </c>
-      <c r="B197" s="1" t="s">
+      <c r="B197" t="s">
         <v>379</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="18.75">
-      <c r="A198" s="1" t="s">
+    <row r="198" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A198" t="s">
         <v>380</v>
       </c>
-      <c r="B198" s="1" t="s">
+      <c r="B198" t="s">
         <v>381</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="18.75">
-      <c r="A199" s="1" t="s">
+    <row r="199" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A199" t="s">
         <v>382</v>
       </c>
-      <c r="B199" s="1" t="s">
+      <c r="B199" t="s">
         <v>383</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="18.75">
-      <c r="A200" s="1" t="s">
+    <row r="200" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A200" t="s">
         <v>384</v>
       </c>
-      <c r="B200" s="1" t="s">
+      <c r="B200" t="s">
         <v>385</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="18.75">
-      <c r="A201" s="1" t="s">
+    <row r="201" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A201" t="s">
         <v>386</v>
       </c>
-      <c r="B201" s="1" t="s">
+      <c r="B201" t="s">
         <v>387</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="18.75">
-      <c r="A202" s="2" t="s">
+    <row r="202" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A202" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="B202" s="2" t="s">
+      <c r="B202" s="1" t="s">
         <v>389</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="18.75">
-      <c r="A203" s="1" t="s">
+    <row r="203" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A203" t="s">
         <v>390</v>
       </c>
-      <c r="B203" s="1" t="s">
+      <c r="B203" t="s">
         <v>391</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="18.75">
-      <c r="A204" s="1" t="s">
+    <row r="204" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A204" t="s">
         <v>392</v>
       </c>
-      <c r="B204" s="1" t="s">
+      <c r="B204" t="s">
         <v>393</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="18.75">
-      <c r="A205" s="1" t="s">
+    <row r="205" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A205" t="s">
         <v>394</v>
       </c>
-      <c r="B205" s="1" t="s">
+      <c r="B205" t="s">
         <v>395</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="18.75">
-      <c r="A206" s="1" t="s">
+    <row r="206" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A206" t="s">
         <v>396</v>
       </c>
-      <c r="B206" s="1" t="s">
+      <c r="B206" t="s">
         <v>397</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="18.75">
-      <c r="A207" s="1" t="s">
+    <row r="207" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A207" t="s">
         <v>398</v>
       </c>
-      <c r="B207" s="1" t="s">
+      <c r="B207" t="s">
         <v>399</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="18.75">
-      <c r="A208" s="1" t="s">
+    <row r="208" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A208" t="s">
         <v>400</v>
       </c>
-      <c r="B208" s="1" t="s">
+      <c r="B208" t="s">
         <v>401</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="209" customHeight="1" ht="18.75">
-      <c r="A209" s="1" t="s">
+    <row r="209" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A209" t="s">
         <v>402</v>
       </c>
-      <c r="B209" s="1" t="s">
+      <c r="B209" t="s">
         <v>403</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="210" customHeight="1" ht="18.75">
-      <c r="A210" s="1" t="s">
+    <row r="210" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A210" t="s">
         <v>404</v>
       </c>
-      <c r="B210" s="1" t="s">
+      <c r="B210" t="s">
         <v>405</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="211" customHeight="1" ht="18.75">
-      <c r="A211" s="1" t="s">
+    <row r="211" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A211" t="s">
         <v>406</v>
       </c>
-      <c r="B211" s="1" t="s">
+      <c r="B211" t="s">
         <v>47</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="212" customHeight="1" ht="18.75">
-      <c r="A212" s="1" t="s">
+    <row r="212" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A212" t="s">
         <v>407</v>
       </c>
-      <c r="B212" s="1" t="s">
+      <c r="B212" t="s">
         <v>49</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="213" customHeight="1" ht="18.75">
-      <c r="A213" s="1" t="s">
+    <row r="213" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A213" t="s">
         <v>408</v>
       </c>
-      <c r="B213" s="1" t="s">
+      <c r="B213" t="s">
         <v>409</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="214" customHeight="1" ht="18.75">
-      <c r="A214" s="1" t="s">
+    <row r="214" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A214" t="s">
         <v>410</v>
       </c>
-      <c r="B214" s="1" t="s">
+      <c r="B214" t="s">
         <v>411</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="215" customHeight="1" ht="18.75">
-      <c r="A215" s="1" t="s">
+    <row r="215" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A215" t="s">
         <v>412</v>
       </c>
-      <c r="B215" s="1" t="s">
+      <c r="B215" t="s">
         <v>413</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="216" customHeight="1" ht="18.75">
-      <c r="A216" s="1" t="s">
+    <row r="216" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A216" t="s">
         <v>414</v>
       </c>
-      <c r="B216" s="1" t="s">
+      <c r="B216" t="s">
         <v>415</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="217" customHeight="1" ht="18.75">
-      <c r="A217" s="1" t="s">
+    <row r="217" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A217" t="s">
         <v>416</v>
       </c>
-      <c r="B217" s="1" t="s">
+      <c r="B217" t="s">
         <v>417</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="218" customHeight="1" ht="18.75">
-      <c r="A218" s="2" t="s">
+    <row r="218" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A218" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="B218" s="2" t="s">
+      <c r="B218" s="1" t="s">
         <v>419</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="219" customHeight="1" ht="18.75">
-      <c r="A219" s="2" t="s">
+    <row r="219" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A219" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="B219" s="2" t="s">
+      <c r="B219" s="1" t="s">
         <v>421</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="220" customHeight="1" ht="18.75">
-      <c r="A220" s="1" t="s">
+    <row r="220" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A220" t="s">
         <v>422</v>
       </c>
-      <c r="B220" s="1" t="s">
+      <c r="B220" t="s">
         <v>423</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="221" customHeight="1" ht="18.75">
-      <c r="A221" s="1" t="s">
+    <row r="221" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A221" t="s">
         <v>424</v>
       </c>
-      <c r="B221" s="1" t="s">
+      <c r="B221" t="s">
         <v>425</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="222" customHeight="1" ht="18.75">
-      <c r="A222" s="1" t="s">
+    <row r="222" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A222" t="s">
         <v>426</v>
       </c>
-      <c r="B222" s="1" t="s">
+      <c r="B222" t="s">
         <v>427</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="223" customHeight="1" ht="18.75">
-      <c r="A223" s="1" t="s">
+    <row r="223" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A223" t="s">
         <v>428</v>
       </c>
-      <c r="B223" s="1" t="s">
+      <c r="B223" t="s">
         <v>429</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="224" customHeight="1" ht="18.75">
-      <c r="A224" s="1" t="s">
+    <row r="224" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A224" t="s">
         <v>430</v>
       </c>
-      <c r="B224" s="1" t="s">
+      <c r="B224" t="s">
         <v>431</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="225" customHeight="1" ht="18.75">
-      <c r="A225" s="1" t="s">
+    <row r="225" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A225" t="s">
         <v>432</v>
       </c>
-      <c r="B225" s="1" t="s">
+      <c r="B225" t="s">
         <v>433</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="226" customHeight="1" ht="18.75">
-      <c r="A226" s="1" t="s">
+    <row r="226" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A226" t="s">
         <v>434</v>
       </c>
-      <c r="B226" s="1" t="s">
+      <c r="B226" t="s">
         <v>435</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="227" customHeight="1" ht="18.75">
-      <c r="A227" s="1" t="s">
+    <row r="227" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A227" t="s">
+        <v>555</v>
+      </c>
+      <c r="B227" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A228" t="s">
+        <v>557</v>
+      </c>
+      <c r="B228" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A229" t="s">
+        <v>559</v>
+      </c>
+      <c r="B229" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A230" t="s">
         <v>436</v>
       </c>
-      <c r="B227" s="1" t="s">
+      <c r="B230" t="s">
         <v>437</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="228" customHeight="1" ht="18.75">
-      <c r="A228" s="1" t="s">
+    <row r="231" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A231" t="s">
         <v>438</v>
       </c>
-      <c r="B228" s="1" t="s">
+      <c r="B231" t="s">
         <v>439</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="229" customHeight="1" ht="18.75">
-      <c r="A229" s="1" t="s">
+    <row r="232" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A232" t="s">
         <v>440</v>
       </c>
-      <c r="B229" s="1" t="s">
+      <c r="B232" t="s">
         <v>441</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="230" customHeight="1" ht="18.75">
-      <c r="A230" s="1" t="s">
+    <row r="233" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A233" t="s">
         <v>442</v>
       </c>
-      <c r="B230" s="1" t="s">
+      <c r="B233" t="s">
         <v>443</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="231" customHeight="1" ht="18.75">
-      <c r="A231" s="1" t="s">
+    <row r="234" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A234" t="s">
         <v>444</v>
       </c>
-      <c r="B231" s="1" t="s">
+      <c r="B234" t="s">
         <v>445</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="232" customHeight="1" ht="18.75">
-      <c r="A232" s="1" t="s">
+    <row r="235" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A235" t="s">
         <v>446</v>
       </c>
-      <c r="B232" s="1" t="s">
+      <c r="B235" t="s">
         <v>447</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="233" customHeight="1" ht="18.75">
-      <c r="A233" s="1" t="s">
+    <row r="236" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A236" t="s">
         <v>448</v>
       </c>
-      <c r="B233" s="1" t="s">
+      <c r="B236" t="s">
         <v>449</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="234" customHeight="1" ht="18.75">
-      <c r="A234" s="1" t="s">
+    <row r="237" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A237" t="s">
         <v>450</v>
       </c>
-      <c r="B234" s="1" t="s">
+      <c r="B237" t="s">
         <v>451</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="235" customHeight="1" ht="18.75">
-      <c r="A235" s="1" t="s">
+    <row r="238" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A238" t="s">
         <v>452</v>
       </c>
-      <c r="B235" s="1" t="s">
+      <c r="B238" t="s">
         <v>453</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="236" customHeight="1" ht="18.75">
-      <c r="A236" s="1" t="s">
+    <row r="239" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A239" t="s">
         <v>454</v>
       </c>
-      <c r="B236" s="1" t="s">
+      <c r="B239" t="s">
         <v>455</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="237" customHeight="1" ht="18.75">
-      <c r="A237" s="1" t="s">
+    <row r="240" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A240" t="s">
         <v>456</v>
       </c>
-      <c r="B237" s="1" t="s">
+      <c r="B240" t="s">
         <v>457</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="238" customHeight="1" ht="18.75">
-      <c r="A238" s="1" t="s">
+    <row r="241" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A241" t="s">
         <v>458</v>
       </c>
-      <c r="B238" s="1" t="s">
+      <c r="B241" t="s">
         <v>459</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="239" customHeight="1" ht="18.75">
-      <c r="A239" s="1" t="s">
+    <row r="242" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A242" t="s">
         <v>460</v>
       </c>
-      <c r="B239" s="1" t="s">
+      <c r="B242" t="s">
         <v>461</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="240" customHeight="1" ht="18.75">
-      <c r="A240" s="1" t="s">
+    <row r="243" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A243" t="s">
         <v>462</v>
       </c>
-      <c r="B240" s="1" t="s">
+      <c r="B243" t="s">
         <v>463</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="241" customHeight="1" ht="18.75">
-      <c r="A241" s="1" t="s">
+    <row r="244" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A244" t="s">
         <v>464</v>
       </c>
-      <c r="B241" s="1" t="s">
+      <c r="B244" t="s">
         <v>465</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="242" customHeight="1" ht="18.75">
-      <c r="A242" s="1" t="s">
+    <row r="245" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A245" t="s">
         <v>466</v>
       </c>
-      <c r="B242" s="1" t="s">
+      <c r="B245" t="s">
         <v>467</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="243" customHeight="1" ht="18.75">
-      <c r="A243" s="1" t="s">
+    <row r="246" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A246" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="B243" s="1" t="s">
+      <c r="B246" s="2" t="s">
         <v>469</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="244" customHeight="1" ht="18.75">
-      <c r="A244" s="1" t="s">
+    <row r="247" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A247" t="s">
         <v>470</v>
       </c>
-      <c r="B244" s="1" t="s">
+      <c r="B247" t="s">
         <v>471</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="245" customHeight="1" ht="18.75">
-      <c r="A245" s="1" t="s">
+    <row r="248" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A248" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="B245" s="1" t="s">
+      <c r="B248" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="246" customHeight="1" ht="18.75">
-      <c r="A246" s="2" t="s">
+    <row r="249" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A249" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="B246" s="2" t="s">
+      <c r="B249" s="1" t="s">
         <v>474</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="247" customHeight="1" ht="18.75">
-      <c r="A247" s="1" t="s">
+    <row r="250" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A250" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="B247" s="1" t="s">
+      <c r="B250" s="2" t="s">
         <v>476</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="248" customHeight="1" ht="18.75">
-      <c r="A248" s="2" t="s">
+    <row r="251" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A251" s="3" t="s">
         <v>477</v>
       </c>
-      <c r="B248" s="2" t="s">
+      <c r="B251" s="3" t="s">
         <v>478</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="249" customHeight="1" ht="18.75">
-      <c r="A249" s="2" t="s">
+    <row r="252" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A252" s="3" t="s">
         <v>479</v>
       </c>
-      <c r="B249" s="2" t="s">
+      <c r="B252" s="3" t="s">
         <v>480</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="250" customHeight="1" ht="18.75">
-      <c r="A250" s="2" t="s">
+    <row r="253" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A253" s="3" t="s">
         <v>481</v>
       </c>
-      <c r="B250" s="2" t="s">
+      <c r="B253" s="3" t="s">
         <v>482</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="251" customHeight="1" ht="18.75">
-      <c r="A251" s="1" t="s">
+    <row r="254" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A254" t="s">
         <v>483</v>
       </c>
-      <c r="B251" s="1" t="s">
+      <c r="B254" t="s">
         <v>484</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="252" customHeight="1" ht="18.75">
-      <c r="A252" s="1" t="s">
+    <row r="255" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A255" t="s">
         <v>485</v>
       </c>
-      <c r="B252" s="1" t="s">
+      <c r="B255" t="s">
         <v>486</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="253" customHeight="1" ht="18.75">
-      <c r="A253" s="1" t="s">
+    <row r="256" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A256" t="s">
         <v>487</v>
       </c>
-      <c r="B253" s="1" t="s">
+      <c r="B256" t="s">
         <v>488</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="254" customHeight="1" ht="18.75">
-      <c r="A254" s="1" t="s">
+    <row r="257" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A257" t="s">
         <v>489</v>
       </c>
-      <c r="B254" s="1" t="s">
+      <c r="B257" t="s">
         <v>490</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="255" customHeight="1" ht="18.75">
-      <c r="A255" s="1" t="s">
+    <row r="258" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A258" s="2" t="s">
         <v>491</v>
       </c>
-      <c r="B255" s="1" t="s">
+      <c r="B258" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="256" customHeight="1" ht="18.75">
-      <c r="A256" s="1" t="s">
+    <row r="259" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A259" t="s">
         <v>492</v>
       </c>
-      <c r="B256" s="1" t="s">
+      <c r="B259" t="s">
         <v>493</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="257" customHeight="1" ht="18.75">
-      <c r="A257" s="1" t="s">
+    <row r="260" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A260" t="s">
         <v>494</v>
       </c>
-      <c r="B257" s="1" t="s">
+      <c r="B260" t="s">
         <v>495</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="258" customHeight="1" ht="18.75">
-      <c r="A258" s="2" t="s">
+    <row r="261" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A261" s="3" t="s">
         <v>496</v>
       </c>
-      <c r="B258" s="2" t="s">
+      <c r="B261" s="3" t="s">
         <v>497</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="259" customHeight="1" ht="18.75">
-      <c r="A259" s="1" t="s">
+    <row r="262" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A262" t="s">
         <v>498</v>
       </c>
-      <c r="B259" s="1" t="s">
+      <c r="B262" t="s">
         <v>499</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="260" customHeight="1" ht="18.75">
-      <c r="A260" s="1" t="s">
+    <row r="263" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A263" t="s">
         <v>500</v>
       </c>
-      <c r="B260" s="1" t="s">
+      <c r="B263" t="s">
         <v>501</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="18.75">
-      <c r="A261" s="1" t="s">
+    <row r="264" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A264" t="s">
         <v>502</v>
       </c>
-      <c r="B261" s="1" t="s">
+      <c r="B264" t="s">
         <v>277</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="18.75">
-      <c r="A262" s="1" t="s">
+    <row r="265" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A265" t="s">
         <v>503</v>
       </c>
-      <c r="B262" s="1" t="s">
+      <c r="B265" t="s">
         <v>504</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="263" customHeight="1" ht="18.75">
-      <c r="A263" s="1" t="s">
+    <row r="266" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A266" t="s">
         <v>505</v>
       </c>
-      <c r="B263" s="1" t="s">
+      <c r="B266" t="s">
         <v>506</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="264" customHeight="1" ht="18.75">
-      <c r="A264" s="1" t="s">
+    <row r="267" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A267" t="s">
         <v>507</v>
       </c>
-      <c r="B264" s="1" t="s">
+      <c r="B267" t="s">
         <v>508</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="265" customHeight="1" ht="18.75">
-      <c r="A265" s="1" t="s">
+    <row r="268" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A268" t="s">
         <v>509</v>
       </c>
-      <c r="B265" s="1" t="s">
+      <c r="B268" t="s">
         <v>510</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="266" customHeight="1" ht="18.75">
-      <c r="A266" s="1" t="s">
+    <row r="269" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A269" t="s">
         <v>511</v>
       </c>
-      <c r="B266" s="1" t="s">
+      <c r="B269" t="s">
         <v>512</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="267" customHeight="1" ht="18.75">
-      <c r="A267" s="1" t="s">
+    <row r="270" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A270" t="s">
         <v>513</v>
       </c>
-      <c r="B267" s="1" t="s">
+      <c r="B270" t="s">
         <v>514</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="268" customHeight="1" ht="18.75">
-      <c r="A268" s="1" t="s">
+    <row r="271" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A271" t="s">
         <v>515</v>
       </c>
-      <c r="B268" s="1" t="s">
+      <c r="B271" t="s">
         <v>516</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="269" customHeight="1" ht="18.75">
-      <c r="A269" s="1" t="s">
+    <row r="272" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A272" t="s">
         <v>517</v>
       </c>
-      <c r="B269" s="1" t="s">
+      <c r="B272" t="s">
         <v>518</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="270" customHeight="1" ht="18.75">
-      <c r="A270" s="1" t="s">
+    <row r="273" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A273" t="s">
         <v>519</v>
       </c>
-      <c r="B270" s="1" t="s">
+      <c r="B273" t="s">
         <v>520</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="271" customHeight="1" ht="18.75">
-      <c r="A271" s="1" t="s">
+    <row r="274" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A274" s="2" t="s">
         <v>521</v>
       </c>
-      <c r="B271" s="1" t="s">
+      <c r="B274" s="2" t="s">
         <v>522</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="18.75">
-      <c r="A272" s="1" t="s">
+    <row r="275" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A275" t="s">
         <v>523</v>
       </c>
-      <c r="B272" s="1" t="s">
+      <c r="B275" t="s">
         <v>524</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="273" customHeight="1" ht="18.75">
-      <c r="A273" s="1" t="s">
+    <row r="276" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A276" t="s">
         <v>525</v>
       </c>
-      <c r="B273" s="1" t="s">
+      <c r="B276" t="s">
         <v>526</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="18.75">
-      <c r="A274" s="2" t="s">
+    <row r="277" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A277" s="3" t="s">
         <v>527</v>
       </c>
-      <c r="B274" s="2" t="s">
+      <c r="B277" s="3" t="s">
         <v>528</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="275" customHeight="1" ht="18.75">
-      <c r="A275" s="1" t="s">
+    <row r="278" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A278" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="B275" s="1" t="s">
+      <c r="B278" s="2" t="s">
         <v>530</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="276" customHeight="1" ht="18.75">
-      <c r="A276" s="1" t="s">
+    <row r="279" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A279" t="s">
         <v>531</v>
       </c>
-      <c r="B276" s="1" t="s">
+      <c r="B279" t="s">
         <v>532</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="277" customHeight="1" ht="18.75">
-      <c r="A277" s="1" t="s">
+    <row r="280" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A280" t="s">
         <v>533</v>
       </c>
-      <c r="B277" s="1" t="s">
+      <c r="B280" t="s">
         <v>534</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="18.75">
-      <c r="A278" s="2" t="s">
+    <row r="281" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A281" s="3" t="s">
         <v>535</v>
       </c>
-      <c r="B278" s="2" t="s">
+      <c r="B281" s="3" t="s">
         <v>536</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="279" customHeight="1" ht="18.75">
-      <c r="A279" s="1" t="s">
+    <row r="282" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A282" t="s">
         <v>537</v>
       </c>
-      <c r="B279" s="1" t="s">
+      <c r="B282" t="s">
         <v>538</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="280" customHeight="1" ht="18.75">
-      <c r="A280" s="1" t="s">
+    <row r="283" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A283" t="s">
         <v>539</v>
       </c>
-      <c r="B280" s="1" t="s">
+      <c r="B283" t="s">
         <v>540</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="281" customHeight="1" ht="18.75">
-      <c r="A281" s="1" t="s">
+    <row r="284" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A284" t="s">
         <v>541</v>
       </c>
-      <c r="B281" s="1" t="s">
+      <c r="B284" t="s">
         <v>542</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="282" customHeight="1" ht="18.75">
-      <c r="A282" s="1" t="s">
+    <row r="285" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A285" t="s">
         <v>543</v>
       </c>
-      <c r="B282" s="1" t="s">
+      <c r="B285" t="s">
         <v>544</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="283" customHeight="1" ht="18.75">
-      <c r="A283" s="1" t="s">
+    <row r="286" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A286" t="s">
         <v>545</v>
       </c>
-      <c r="B283" s="1" t="s">
+      <c r="B286" t="s">
         <v>546</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="284" customHeight="1" ht="18.75">
-      <c r="A284" s="1" t="s">
+    <row r="287" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A287" t="s">
         <v>547</v>
       </c>
-      <c r="B284" s="1" t="s">
+      <c r="B287" t="s">
         <v>548</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="285" customHeight="1" ht="18.75">
-      <c r="A285" s="1" t="s">
+    <row r="288" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A288" t="s">
         <v>549</v>
       </c>
-      <c r="B285" s="1" t="s">
+      <c r="B288" t="s">
         <v>550</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="286" customHeight="1" ht="18.75">
-      <c r="A286" s="1" t="s">
+    <row r="289" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A289" t="s">
         <v>551</v>
       </c>
-      <c r="B286" s="1" t="s">
+      <c r="B289" t="s">
         <v>552</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="287" customHeight="1" ht="18.75">
-      <c r="A287" s="1" t="s">
+    <row r="290" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A290" t="s">
         <v>553</v>
       </c>
-      <c r="B287" s="1" t="s">
+      <c r="B290" t="s">
         <v>554</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B1" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B290">
+      <sortCondition ref="A1:A290"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MAUI-5749 Usage quality metrics on patients (#241)
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/salmanraza/Documents/GitHub/tamanu-source-dbt/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia\Documents\GitHub\tamanu-source-dbt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C960FFE9-82F0-894D-A44C-58483C095E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74409AB8-E8B9-4DE4-AACE-7B87B9E1ADBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14390" yWindow="-10" windowWidth="14420" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Translated String" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Translated String'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Translated String'!$A$1:$B$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="561">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="581">
   <si>
     <t>stringId</t>
   </si>
@@ -1277,6 +1277,66 @@
   </si>
   <si>
     <t>Social security number</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotal</t>
+  </si>
+  <si>
+    <t>Total patients</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalBirthRegistrations</t>
+  </si>
+  <si>
+    <t>Total birth registrations</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalIncorrectRegistrationsForAgedUnder6Months</t>
+  </si>
+  <si>
+    <t>Total incorrect registrations for aged under 6 months</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalMerged</t>
+  </si>
+  <si>
+    <t>Total patients merged</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalPatientRegistrations</t>
+  </si>
+  <si>
+    <t>Total patient registrations</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithIncompleteName</t>
+  </si>
+  <si>
+    <t>Total patients with incomplete name</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithInvalidDateOfBirth</t>
+  </si>
+  <si>
+    <t>Total patients with invalid date of birth</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithMissingContact</t>
+  </si>
+  <si>
+    <t>Total patients with missing contact</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithMissingDateOfBirth</t>
+  </si>
+  <si>
+    <t>Total patients with missing date of birth</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithMissingLocation</t>
+  </si>
+  <si>
+    <t>Total patients with missing location</t>
   </si>
   <si>
     <t>report.reporting.patientStreetVillage</t>
@@ -1754,15 +1814,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2068,14 +2125,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B290"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B300"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="58.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="64.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2083,7 +2140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -2091,7 +2148,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -2099,7 +2156,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2107,7 +2164,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2115,7 +2172,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -2123,7 +2180,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -2131,7 +2188,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -2139,7 +2196,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2147,7 +2204,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -2155,7 +2212,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -2163,7 +2220,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -2171,7 +2228,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -2179,7 +2236,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -2187,7 +2244,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -2195,7 +2252,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -2203,7 +2260,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -2211,7 +2268,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -2219,7 +2276,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -2227,7 +2284,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -2235,7 +2292,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>40</v>
       </c>
@@ -2243,7 +2300,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>42</v>
       </c>
@@ -2251,7 +2308,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>44</v>
       </c>
@@ -2259,7 +2316,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>46</v>
       </c>
@@ -2267,7 +2324,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>48</v>
       </c>
@@ -2275,7 +2332,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>50</v>
       </c>
@@ -2283,7 +2340,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>52</v>
       </c>
@@ -2291,7 +2348,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>54</v>
       </c>
@@ -2299,7 +2356,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>56</v>
       </c>
@@ -2307,7 +2364,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>57</v>
       </c>
@@ -2315,7 +2372,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>59</v>
       </c>
@@ -2323,7 +2380,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>61</v>
       </c>
@@ -2331,7 +2388,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>63</v>
       </c>
@@ -2339,7 +2396,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>64</v>
       </c>
@@ -2347,7 +2404,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>66</v>
       </c>
@@ -2355,7 +2412,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>68</v>
       </c>
@@ -2363,7 +2420,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>70</v>
       </c>
@@ -2371,7 +2428,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>72</v>
       </c>
@@ -2379,7 +2436,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>73</v>
       </c>
@@ -2387,7 +2444,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>75</v>
       </c>
@@ -2395,7 +2452,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>77</v>
       </c>
@@ -2403,7 +2460,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>79</v>
       </c>
@@ -2411,7 +2468,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>81</v>
       </c>
@@ -2419,7 +2476,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>83</v>
       </c>
@@ -2427,7 +2484,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>85</v>
       </c>
@@ -2435,7 +2492,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>87</v>
       </c>
@@ -2443,7 +2500,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>89</v>
       </c>
@@ -2451,7 +2508,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>91</v>
       </c>
@@ -2459,7 +2516,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>93</v>
       </c>
@@ -2467,7 +2524,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>95</v>
       </c>
@@ -2475,7 +2532,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>97</v>
       </c>
@@ -2483,7 +2540,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>99</v>
       </c>
@@ -2491,7 +2548,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>101</v>
       </c>
@@ -2499,7 +2556,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>103</v>
       </c>
@@ -2507,7 +2564,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>105</v>
       </c>
@@ -2515,7 +2572,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>107</v>
       </c>
@@ -2523,7 +2580,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>109</v>
       </c>
@@ -2531,7 +2588,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>111</v>
       </c>
@@ -2539,7 +2596,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>113</v>
       </c>
@@ -2547,7 +2604,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>115</v>
       </c>
@@ -2555,7 +2612,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>117</v>
       </c>
@@ -2563,7 +2620,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>119</v>
       </c>
@@ -2571,7 +2628,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>121</v>
       </c>
@@ -2579,7 +2636,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>123</v>
       </c>
@@ -2587,7 +2644,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
         <v>125</v>
       </c>
@@ -2595,7 +2652,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
         <v>127</v>
       </c>
@@ -2603,7 +2660,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
         <v>129</v>
       </c>
@@ -2611,7 +2668,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
         <v>131</v>
       </c>
@@ -2619,7 +2676,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
         <v>133</v>
       </c>
@@ -2627,7 +2684,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
         <v>135</v>
       </c>
@@ -2635,7 +2692,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
         <v>137</v>
       </c>
@@ -2643,7 +2700,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
         <v>139</v>
       </c>
@@ -2651,7 +2708,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
         <v>141</v>
       </c>
@@ -2659,7 +2716,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
         <v>143</v>
       </c>
@@ -2667,7 +2724,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
         <v>145</v>
       </c>
@@ -2675,7 +2732,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
         <v>147</v>
       </c>
@@ -2683,7 +2740,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
         <v>149</v>
       </c>
@@ -2691,7 +2748,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
         <v>151</v>
       </c>
@@ -2699,7 +2756,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
         <v>153</v>
       </c>
@@ -2707,7 +2764,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
         <v>155</v>
       </c>
@@ -2715,7 +2772,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="81" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
         <v>157</v>
       </c>
@@ -2723,7 +2780,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="82" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
         <v>158</v>
       </c>
@@ -2731,7 +2788,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="83" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
         <v>160</v>
       </c>
@@ -2739,7 +2796,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="84" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
         <v>162</v>
       </c>
@@ -2747,7 +2804,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="85" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
         <v>164</v>
       </c>
@@ -2755,7 +2812,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="86" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
         <v>166</v>
       </c>
@@ -2763,7 +2820,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="87" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
         <v>168</v>
       </c>
@@ -2771,7 +2828,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="88" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
         <v>170</v>
       </c>
@@ -2779,7 +2836,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="89" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
         <v>172</v>
       </c>
@@ -2787,7 +2844,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="90" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
         <v>174</v>
       </c>
@@ -2795,7 +2852,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="91" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
         <v>176</v>
       </c>
@@ -2803,7 +2860,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="92" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
         <v>178</v>
       </c>
@@ -2811,7 +2868,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="93" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
         <v>180</v>
       </c>
@@ -2819,7 +2876,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="94" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
         <v>182</v>
       </c>
@@ -2827,7 +2884,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="95" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
         <v>184</v>
       </c>
@@ -2835,7 +2892,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="96" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
         <v>186</v>
       </c>
@@ -2843,7 +2900,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="97" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
         <v>188</v>
       </c>
@@ -2851,7 +2908,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="98" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
         <v>190</v>
       </c>
@@ -2859,7 +2916,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="99" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
         <v>192</v>
       </c>
@@ -2867,7 +2924,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="100" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
         <v>194</v>
       </c>
@@ -2875,7 +2932,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="101" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
         <v>196</v>
       </c>
@@ -2883,7 +2940,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="102" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
         <v>198</v>
       </c>
@@ -2891,7 +2948,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="103" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
         <v>200</v>
       </c>
@@ -2899,7 +2956,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="104" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
         <v>202</v>
       </c>
@@ -2907,7 +2964,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="105" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
         <v>204</v>
       </c>
@@ -2915,7 +2972,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="106" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
         <v>206</v>
       </c>
@@ -2923,7 +2980,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="107" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
         <v>208</v>
       </c>
@@ -2931,7 +2988,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="108" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
         <v>210</v>
       </c>
@@ -2939,7 +2996,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="109" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
         <v>212</v>
       </c>
@@ -2947,7 +3004,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="110" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
         <v>214</v>
       </c>
@@ -2955,7 +3012,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="111" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
         <v>216</v>
       </c>
@@ -2963,7 +3020,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="112" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
         <v>218</v>
       </c>
@@ -2971,7 +3028,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="113" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
         <v>220</v>
       </c>
@@ -2979,7 +3036,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="114" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
         <v>222</v>
       </c>
@@ -2987,7 +3044,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="115" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
         <v>224</v>
       </c>
@@ -2995,7 +3052,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="116" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
         <v>226</v>
       </c>
@@ -3003,7 +3060,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="117" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
         <v>228</v>
       </c>
@@ -3011,7 +3068,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="118" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
         <v>230</v>
       </c>
@@ -3019,7 +3076,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="119" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
         <v>232</v>
       </c>
@@ -3027,7 +3084,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="120" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
         <v>234</v>
       </c>
@@ -3035,7 +3092,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="121" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
         <v>236</v>
       </c>
@@ -3043,7 +3100,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="122" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
         <v>238</v>
       </c>
@@ -3051,7 +3108,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="123" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
         <v>240</v>
       </c>
@@ -3059,7 +3116,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="124" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
         <v>242</v>
       </c>
@@ -3067,7 +3124,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="125" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
         <v>243</v>
       </c>
@@ -3075,7 +3132,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="126" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
         <v>245</v>
       </c>
@@ -3083,7 +3140,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="127" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
         <v>247</v>
       </c>
@@ -3091,7 +3148,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="128" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
         <v>249</v>
       </c>
@@ -3099,7 +3156,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="129" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
         <v>251</v>
       </c>
@@ -3107,7 +3164,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="130" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
         <v>253</v>
       </c>
@@ -3115,7 +3172,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="131" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
         <v>255</v>
       </c>
@@ -3123,7 +3180,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="132" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
         <v>257</v>
       </c>
@@ -3131,7 +3188,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="133" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
         <v>259</v>
       </c>
@@ -3139,7 +3196,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="134" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
         <v>261</v>
       </c>
@@ -3147,7 +3204,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="135" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
         <v>263</v>
       </c>
@@ -3155,7 +3212,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="136" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
         <v>265</v>
       </c>
@@ -3163,7 +3220,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="137" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
         <v>267</v>
       </c>
@@ -3171,7 +3228,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="138" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
         <v>269</v>
       </c>
@@ -3179,7 +3236,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="139" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
         <v>271</v>
       </c>
@@ -3187,7 +3244,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="140" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
         <v>272</v>
       </c>
@@ -3195,7 +3252,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="141" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
         <v>273</v>
       </c>
@@ -3203,7 +3260,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="142" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
         <v>274</v>
       </c>
@@ -3211,7 +3268,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="143" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
         <v>276</v>
       </c>
@@ -3219,7 +3276,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="144" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
         <v>278</v>
       </c>
@@ -3227,7 +3284,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="145" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>279</v>
       </c>
@@ -3235,7 +3292,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="146" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>280</v>
       </c>
@@ -3243,7 +3300,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="147" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>282</v>
       </c>
@@ -3251,7 +3308,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="148" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>283</v>
       </c>
@@ -3259,7 +3316,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="149" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>285</v>
       </c>
@@ -3267,7 +3324,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="150" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
         <v>287</v>
       </c>
@@ -3275,7 +3332,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="151" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>289</v>
       </c>
@@ -3283,7 +3340,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="152" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
         <v>291</v>
       </c>
@@ -3291,7 +3348,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="153" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
         <v>293</v>
       </c>
@@ -3299,7 +3356,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="154" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
         <v>295</v>
       </c>
@@ -3307,7 +3364,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="155" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
         <v>297</v>
       </c>
@@ -3315,7 +3372,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="156" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
         <v>298</v>
       </c>
@@ -3323,7 +3380,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="157" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
         <v>300</v>
       </c>
@@ -3331,7 +3388,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="158" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
         <v>302</v>
       </c>
@@ -3339,7 +3396,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="159" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
         <v>304</v>
       </c>
@@ -3347,7 +3404,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="160" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
         <v>306</v>
       </c>
@@ -3355,7 +3412,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="161" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
         <v>308</v>
       </c>
@@ -3363,7 +3420,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="162" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
         <v>310</v>
       </c>
@@ -3371,7 +3428,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="163" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
         <v>312</v>
       </c>
@@ -3379,7 +3436,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="164" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A164" t="s">
         <v>314</v>
       </c>
@@ -3387,7 +3444,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="165" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A165" t="s">
         <v>315</v>
       </c>
@@ -3395,7 +3452,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="166" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A166" t="s">
         <v>316</v>
       </c>
@@ -3403,7 +3460,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="167" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A167" t="s">
         <v>318</v>
       </c>
@@ -3411,7 +3468,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="168" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A168" t="s">
         <v>320</v>
       </c>
@@ -3419,7 +3476,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="169" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A169" t="s">
         <v>322</v>
       </c>
@@ -3427,7 +3484,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="170" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A170" t="s">
         <v>324</v>
       </c>
@@ -3435,7 +3492,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="171" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A171" t="s">
         <v>326</v>
       </c>
@@ -3443,7 +3500,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="172" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A172" s="2" t="s">
         <v>330</v>
       </c>
@@ -3451,15 +3508,15 @@
         <v>331</v>
       </c>
     </row>
-    <row r="173" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A173" s="3" t="s">
+    <row r="173" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A173" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="B173" s="3" t="s">
+      <c r="B173" s="1" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="174" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A174" t="s">
         <v>332</v>
       </c>
@@ -3467,7 +3524,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="175" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A175" t="s">
         <v>334</v>
       </c>
@@ -3475,7 +3532,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="176" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A176" t="s">
         <v>336</v>
       </c>
@@ -3483,7 +3540,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="177" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A177" t="s">
         <v>338</v>
       </c>
@@ -3491,7 +3548,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="178" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A178" t="s">
         <v>340</v>
       </c>
@@ -3499,7 +3556,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="179" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A179" t="s">
         <v>342</v>
       </c>
@@ -3507,7 +3564,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="180" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A180" t="s">
         <v>344</v>
       </c>
@@ -3515,7 +3572,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="181" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A181" t="s">
         <v>346</v>
       </c>
@@ -3523,7 +3580,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="182" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A182" t="s">
         <v>348</v>
       </c>
@@ -3531,7 +3588,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="183" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A183" t="s">
         <v>350</v>
       </c>
@@ -3539,7 +3596,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="184" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A184" s="1" t="s">
         <v>352</v>
       </c>
@@ -3547,7 +3604,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="185" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A185" t="s">
         <v>354</v>
       </c>
@@ -3555,7 +3612,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="186" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A186" t="s">
         <v>356</v>
       </c>
@@ -3563,7 +3620,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="187" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A187" t="s">
         <v>358</v>
       </c>
@@ -3571,7 +3628,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="188" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A188" t="s">
         <v>360</v>
       </c>
@@ -3579,7 +3636,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="189" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A189" t="s">
         <v>362</v>
       </c>
@@ -3587,7 +3644,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="190" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A190" t="s">
         <v>364</v>
       </c>
@@ -3595,7 +3652,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="191" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A191" t="s">
         <v>366</v>
       </c>
@@ -3603,7 +3660,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="192" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A192" s="1" t="s">
         <v>368</v>
       </c>
@@ -3611,7 +3668,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="193" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A193" t="s">
         <v>370</v>
       </c>
@@ -3619,7 +3676,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="194" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A194" t="s">
         <v>372</v>
       </c>
@@ -3627,7 +3684,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="195" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A195" t="s">
         <v>374</v>
       </c>
@@ -3635,7 +3692,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="196" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A196" t="s">
         <v>376</v>
       </c>
@@ -3643,7 +3700,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="197" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A197" t="s">
         <v>378</v>
       </c>
@@ -3651,7 +3708,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="198" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A198" t="s">
         <v>380</v>
       </c>
@@ -3659,7 +3716,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="199" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A199" t="s">
         <v>382</v>
       </c>
@@ -3667,7 +3724,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="200" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A200" t="s">
         <v>384</v>
       </c>
@@ -3675,7 +3732,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="201" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A201" t="s">
         <v>386</v>
       </c>
@@ -3683,7 +3740,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="202" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A202" s="1" t="s">
         <v>388</v>
       </c>
@@ -3691,7 +3748,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="203" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A203" t="s">
         <v>390</v>
       </c>
@@ -3699,7 +3756,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="204" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A204" t="s">
         <v>392</v>
       </c>
@@ -3707,7 +3764,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="205" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A205" t="s">
         <v>394</v>
       </c>
@@ -3715,7 +3772,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="206" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A206" t="s">
         <v>396</v>
       </c>
@@ -3723,7 +3780,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="207" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A207" t="s">
         <v>398</v>
       </c>
@@ -3731,7 +3788,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="208" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A208" t="s">
         <v>400</v>
       </c>
@@ -3739,7 +3796,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="209" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A209" t="s">
         <v>402</v>
       </c>
@@ -3747,7 +3804,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="210" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A210" t="s">
         <v>404</v>
       </c>
@@ -3755,7 +3812,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="211" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A211" t="s">
         <v>406</v>
       </c>
@@ -3763,7 +3820,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="212" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A212" t="s">
         <v>407</v>
       </c>
@@ -3771,7 +3828,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="213" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A213" t="s">
         <v>408</v>
       </c>
@@ -3779,7 +3836,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="214" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A214" t="s">
         <v>410</v>
       </c>
@@ -3787,7 +3844,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="215" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A215" t="s">
         <v>412</v>
       </c>
@@ -3795,7 +3852,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="216" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A216" t="s">
         <v>414</v>
       </c>
@@ -3803,7 +3860,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="217" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A217" t="s">
         <v>416</v>
       </c>
@@ -3811,103 +3868,103 @@
         <v>417</v>
       </c>
     </row>
-    <row r="218" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A218" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="B218" s="1" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A219" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="B219" s="1" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A220" t="s">
+        <v>442</v>
+      </c>
+      <c r="B220" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A221" t="s">
         <v>418</v>
       </c>
-      <c r="B218" s="1" t="s">
+      <c r="B221" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="219" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A219" s="1" t="s">
+    <row r="222" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A222" t="s">
         <v>420</v>
       </c>
-      <c r="B219" s="1" t="s">
+      <c r="B222" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="220" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A220" t="s">
+    <row r="223" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A223" t="s">
         <v>422</v>
       </c>
-      <c r="B220" t="s">
+      <c r="B223" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="221" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A221" t="s">
+    <row r="224" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A224" t="s">
         <v>424</v>
       </c>
-      <c r="B221" t="s">
+      <c r="B224" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="222" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A222" t="s">
+    <row r="225" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A225" t="s">
         <v>426</v>
       </c>
-      <c r="B222" t="s">
+      <c r="B225" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="223" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A223" t="s">
+    <row r="226" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A226" t="s">
         <v>428</v>
       </c>
-      <c r="B223" t="s">
+      <c r="B226" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="224" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A224" t="s">
+    <row r="227" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A227" t="s">
         <v>430</v>
       </c>
-      <c r="B224" t="s">
+      <c r="B227" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="225" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A225" t="s">
+    <row r="228" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A228" t="s">
         <v>432</v>
       </c>
-      <c r="B225" t="s">
+      <c r="B228" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="226" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A226" t="s">
+    <row r="229" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A229" t="s">
         <v>434</v>
       </c>
-      <c r="B226" t="s">
+      <c r="B229" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="227" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A227" t="s">
-        <v>555</v>
-      </c>
-      <c r="B227" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="228" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A228" t="s">
-        <v>557</v>
-      </c>
-      <c r="B228" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="229" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A229" t="s">
-        <v>559</v>
-      </c>
-      <c r="B229" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="230" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A230" t="s">
         <v>436</v>
       </c>
@@ -3915,79 +3972,79 @@
         <v>437</v>
       </c>
     </row>
-    <row r="231" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A231" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="B231" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="232" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A232" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="B232" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="233" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A233" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
       <c r="B233" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="234" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A234" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
       <c r="B234" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="235" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A235" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
       <c r="B235" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="236" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A236" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
       <c r="B236" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="237" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A237" t="s">
-        <v>450</v>
+        <v>575</v>
       </c>
       <c r="B237" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="238" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A238" t="s">
-        <v>452</v>
+        <v>577</v>
       </c>
       <c r="B238" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="239" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A239" t="s">
-        <v>454</v>
+        <v>579</v>
       </c>
       <c r="B239" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="240" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A240" t="s">
         <v>456</v>
       </c>
@@ -3995,7 +4052,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="241" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A241" t="s">
         <v>458</v>
       </c>
@@ -4003,7 +4060,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="242" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A242" t="s">
         <v>460</v>
       </c>
@@ -4011,7 +4068,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="243" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A243" t="s">
         <v>462</v>
       </c>
@@ -4019,7 +4076,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="244" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A244" t="s">
         <v>464</v>
       </c>
@@ -4027,7 +4084,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="245" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A245" t="s">
         <v>466</v>
       </c>
@@ -4035,15 +4092,15 @@
         <v>467</v>
       </c>
     </row>
-    <row r="246" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A246" s="2" t="s">
+    <row r="246" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A246" t="s">
         <v>468</v>
       </c>
-      <c r="B246" s="2" t="s">
+      <c r="B246" t="s">
         <v>469</v>
       </c>
     </row>
-    <row r="247" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A247" t="s">
         <v>470</v>
       </c>
@@ -4051,223 +4108,223 @@
         <v>471</v>
       </c>
     </row>
-    <row r="248" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A248" s="2" t="s">
+    <row r="248" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A248" t="s">
         <v>472</v>
       </c>
-      <c r="B248" s="2" t="s">
+      <c r="B248" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A249" t="s">
+        <v>474</v>
+      </c>
+      <c r="B249" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A250" t="s">
+        <v>476</v>
+      </c>
+      <c r="B250" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A251" t="s">
+        <v>478</v>
+      </c>
+      <c r="B251" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A252" t="s">
+        <v>480</v>
+      </c>
+      <c r="B252" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A253" t="s">
+        <v>482</v>
+      </c>
+      <c r="B253" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A254" t="s">
+        <v>484</v>
+      </c>
+      <c r="B254" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A255" t="s">
+        <v>486</v>
+      </c>
+      <c r="B255" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A256" t="s">
+        <v>488</v>
+      </c>
+      <c r="B256" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A257" t="s">
+        <v>490</v>
+      </c>
+      <c r="B257" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A258" t="s">
+        <v>492</v>
+      </c>
+      <c r="B258" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="249" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A249" s="1" t="s">
-        <v>473</v>
-      </c>
-      <c r="B249" s="1" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="250" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A250" s="2" t="s">
-        <v>475</v>
-      </c>
-      <c r="B250" s="2" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="251" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A251" s="3" t="s">
-        <v>477</v>
-      </c>
-      <c r="B251" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="252" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A252" s="3" t="s">
-        <v>479</v>
-      </c>
-      <c r="B252" s="3" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="253" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A253" s="3" t="s">
-        <v>481</v>
-      </c>
-      <c r="B253" s="3" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="254" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A254" t="s">
-        <v>483</v>
-      </c>
-      <c r="B254" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="255" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A255" t="s">
-        <v>485</v>
-      </c>
-      <c r="B255" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="256" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A256" t="s">
-        <v>487</v>
-      </c>
-      <c r="B256" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="257" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A257" t="s">
-        <v>489</v>
-      </c>
-      <c r="B257" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="258" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A258" s="2" t="s">
-        <v>491</v>
-      </c>
-      <c r="B258" s="2" t="s">
+    <row r="259" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A259" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="B259" s="1" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A260" t="s">
+        <v>495</v>
+      </c>
+      <c r="B260" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A261" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="B261" s="1" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A262" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="B262" s="1" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A263" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="B263" s="1" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A264" t="s">
+        <v>503</v>
+      </c>
+      <c r="B264" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A265" t="s">
+        <v>505</v>
+      </c>
+      <c r="B265" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A266" t="s">
+        <v>507</v>
+      </c>
+      <c r="B266" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A267" t="s">
+        <v>509</v>
+      </c>
+      <c r="B267" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A268" t="s">
+        <v>511</v>
+      </c>
+      <c r="B268" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="259" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A259" t="s">
-        <v>492</v>
-      </c>
-      <c r="B259" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="260" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A260" t="s">
-        <v>494</v>
-      </c>
-      <c r="B260" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="261" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A261" s="3" t="s">
-        <v>496</v>
-      </c>
-      <c r="B261" s="3" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="262" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A262" t="s">
-        <v>498</v>
-      </c>
-      <c r="B262" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="263" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A263" t="s">
-        <v>500</v>
-      </c>
-      <c r="B263" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="264" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A264" t="s">
-        <v>502</v>
-      </c>
-      <c r="B264" t="s">
+    <row r="269" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A269" t="s">
+        <v>512</v>
+      </c>
+      <c r="B269" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A270" t="s">
+        <v>514</v>
+      </c>
+      <c r="B270" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A271" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="B271" s="1" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A272" t="s">
+        <v>518</v>
+      </c>
+      <c r="B272" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A273" t="s">
+        <v>520</v>
+      </c>
+      <c r="B273" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A274" t="s">
+        <v>522</v>
+      </c>
+      <c r="B274" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="265" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A265" t="s">
-        <v>503</v>
-      </c>
-      <c r="B265" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="266" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A266" t="s">
-        <v>505</v>
-      </c>
-      <c r="B266" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="267" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A267" t="s">
-        <v>507</v>
-      </c>
-      <c r="B267" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="268" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A268" t="s">
-        <v>509</v>
-      </c>
-      <c r="B268" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="269" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A269" t="s">
-        <v>511</v>
-      </c>
-      <c r="B269" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="270" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A270" t="s">
-        <v>513</v>
-      </c>
-      <c r="B270" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="271" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A271" t="s">
-        <v>515</v>
-      </c>
-      <c r="B271" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="272" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A272" t="s">
-        <v>517</v>
-      </c>
-      <c r="B272" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="273" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A273" t="s">
-        <v>519</v>
-      </c>
-      <c r="B273" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="274" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A274" s="2" t="s">
-        <v>521</v>
-      </c>
-      <c r="B274" s="2" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="275" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A275" t="s">
         <v>523</v>
       </c>
@@ -4275,7 +4332,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="276" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A276" t="s">
         <v>525</v>
       </c>
@@ -4283,23 +4340,23 @@
         <v>526</v>
       </c>
     </row>
-    <row r="277" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A277" s="3" t="s">
+    <row r="277" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A277" t="s">
         <v>527</v>
       </c>
-      <c r="B277" s="3" t="s">
+      <c r="B277" t="s">
         <v>528</v>
       </c>
     </row>
-    <row r="278" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A278" s="2" t="s">
+    <row r="278" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A278" t="s">
         <v>529</v>
       </c>
-      <c r="B278" s="2" t="s">
+      <c r="B278" t="s">
         <v>530</v>
       </c>
     </row>
-    <row r="279" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A279" t="s">
         <v>531</v>
       </c>
@@ -4307,7 +4364,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="280" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A280" t="s">
         <v>533</v>
       </c>
@@ -4315,15 +4372,15 @@
         <v>534</v>
       </c>
     </row>
-    <row r="281" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A281" s="3" t="s">
+    <row r="281" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A281" t="s">
         <v>535</v>
       </c>
-      <c r="B281" s="3" t="s">
+      <c r="B281" t="s">
         <v>536</v>
       </c>
     </row>
-    <row r="282" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A282" t="s">
         <v>537</v>
       </c>
@@ -4331,7 +4388,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="283" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A283" t="s">
         <v>539</v>
       </c>
@@ -4339,7 +4396,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="284" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A284" t="s">
         <v>541</v>
       </c>
@@ -4347,7 +4404,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="285" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A285" t="s">
         <v>543</v>
       </c>
@@ -4355,7 +4412,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="286" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A286" t="s">
         <v>545</v>
       </c>
@@ -4363,15 +4420,15 @@
         <v>546</v>
       </c>
     </row>
-    <row r="287" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A287" t="s">
+    <row r="287" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A287" s="1" t="s">
         <v>547</v>
       </c>
-      <c r="B287" t="s">
+      <c r="B287" s="1" t="s">
         <v>548</v>
       </c>
     </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A288" t="s">
         <v>549</v>
       </c>
@@ -4379,7 +4436,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="289" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A289" t="s">
         <v>551</v>
       </c>
@@ -4387,7 +4444,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="290" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A290" t="s">
         <v>553</v>
       </c>
@@ -4395,12 +4452,87 @@
         <v>554</v>
       </c>
     </row>
+    <row r="291" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A291" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="B291" s="1" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A292" t="s">
+        <v>557</v>
+      </c>
+      <c r="B292" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A293" t="s">
+        <v>559</v>
+      </c>
+      <c r="B293" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A294" t="s">
+        <v>561</v>
+      </c>
+      <c r="B294" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A295" t="s">
+        <v>563</v>
+      </c>
+      <c r="B295" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A296" t="s">
+        <v>565</v>
+      </c>
+      <c r="B296" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A297" t="s">
+        <v>567</v>
+      </c>
+      <c r="B297" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A298" t="s">
+        <v>569</v>
+      </c>
+      <c r="B298" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A299" t="s">
+        <v>571</v>
+      </c>
+      <c r="B299" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A300" t="s">
+        <v>573</v>
+      </c>
+      <c r="B300" t="s">
+        <v>574</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B1" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B290">
-      <sortCondition ref="A1:A290"/>
-    </sortState>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MAUI 5749 patient metrics v8 (#244)
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -1,29 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10921"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/salmanraza/Documents/GitHub/tamanu-source-dbt/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD87B249-52E5-194F-AD43-9BBE9D9AB31D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Translated String" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Translated String"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Translated String'!$A$1:$B$288</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Translated String'!$A$1:$B$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="583">
   <si>
     <t>stringId</t>
   </si>
@@ -1279,6 +1273,66 @@
     <t>Social security number</t>
   </si>
   <si>
+    <t>report.reporting.patientTotal</t>
+  </si>
+  <si>
+    <t>Total patients</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalBirthRegistrations</t>
+  </si>
+  <si>
+    <t>Total birth registrations</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalIncorrectRegistrationsForAgedUnder6Months</t>
+  </si>
+  <si>
+    <t>Total incorrect registrations for aged under 6 months</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalMerged</t>
+  </si>
+  <si>
+    <t>Total patients merged</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalPatientRegistrations</t>
+  </si>
+  <si>
+    <t>Total patient registrations</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithIncompleteName</t>
+  </si>
+  <si>
+    <t>Total patients with incomplete name</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithInvalidDateOfBirth</t>
+  </si>
+  <si>
+    <t>Total patients with invalid date of birth</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithMissingContact</t>
+  </si>
+  <si>
+    <t>Total patients with missing contact</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithMissingDateOfBirth</t>
+  </si>
+  <si>
+    <t>Total patients with missing date of birth</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithMissingLocation</t>
+  </si>
+  <si>
+    <t>Total patients with missing location</t>
+  </si>
+  <si>
     <t>report.reporting.patientStreetVillage</t>
   </si>
   <si>
@@ -1333,6 +1387,24 @@
     <t>Tamanu user name</t>
   </si>
   <si>
+    <t>report.reporting.prescriptionMedication</t>
+  </si>
+  <si>
+    <t>Medication</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedicationCode</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionQuantity</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
     <t>report.reporting.procedure</t>
   </si>
   <si>
@@ -1351,6 +1423,12 @@
     <t>Procedure assistant</t>
   </si>
   <si>
+    <t>report.reporting.procedureAssistantAnaesthetist</t>
+  </si>
+  <si>
+    <t>Procedure assistant anesthetist</t>
+  </si>
+  <si>
     <t>report.reporting.procedureClinician</t>
   </si>
   <si>
@@ -1411,6 +1489,18 @@
     <t>Procedure start (date and time)</t>
   </si>
   <si>
+    <t>report.reporting.procedureTimeIn</t>
+  </si>
+  <si>
+    <t>Procedure time in</t>
+  </si>
+  <si>
+    <t>report.reporting.procedureTimeOut</t>
+  </si>
+  <si>
+    <t>Procedure time out</t>
+  </si>
+  <si>
     <t>report.reporting.referralCompletedBy</t>
   </si>
   <si>
@@ -1676,30 +1766,13 @@
   </si>
   <si>
     <t>Schedule</t>
-  </si>
-  <si>
-    <t>report.reporting.prescriptionMedicationCode</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>report.reporting.prescriptionMedication</t>
-  </si>
-  <si>
-    <t>report.reporting.prescriptionQuantity</t>
-  </si>
-  <si>
-    <t>Medication</t>
-  </si>
-  <si>
-    <t>Quantity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1742,31 +1815,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="4">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1777,10 +1845,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -1818,71 +1886,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1910,7 +1978,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1933,11 +2001,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1946,13 +2014,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1962,7 +2030,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1971,7 +2039,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1980,7 +2048,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1988,10 +2056,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -2056,1754 +2124,1754 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B288"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B301"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="58.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="3" width="64.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="3" width="35.71928571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+      <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+      <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+      <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+      <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+      <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+      <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+      <c r="A22" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+      <c r="A23" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+      <c r="A24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+      <c r="A25" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+      <c r="A26" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+      <c r="A27" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+      <c r="A28" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+      <c r="A29" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+      <c r="A30" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+      <c r="A31" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
+      <c r="A32" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
+      <c r="A33" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
+      <c r="A34" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
+      <c r="A35" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
+      <c r="A36" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
+      <c r="A37" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
+      <c r="A38" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
+      <c r="A39" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
+      <c r="A40" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
+      <c r="A41" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
+      <c r="A42" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
+      <c r="A43" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
+      <c r="A44" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
+      <c r="A45" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
+      <c r="A46" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
+      <c r="A47" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
+      <c r="A48" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
+      <c r="A49" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
+      <c r="A50" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
+      <c r="A51" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
+      <c r="A52" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
+      <c r="A53" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
+      <c r="A54" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
+      <c r="A55" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
+      <c r="A56" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
+      <c r="A57" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="1" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
+      <c r="A58" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
+      <c r="A59" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
+      <c r="A60" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
+      <c r="A61" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B61" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
+      <c r="A62" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B62" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
+      <c r="A63" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B63" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
+      <c r="A64" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B64" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
+      <c r="A65" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
+      <c r="A66" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
+      <c r="A67" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B67" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
+      <c r="A68" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
+      <c r="A69" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
+      <c r="A70" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B70" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
+      <c r="A71" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
+      <c r="A72" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
+      <c r="A73" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
+      <c r="A74" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B74" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
+      <c r="A75" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B75" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
+      <c r="A76" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B76" s="1" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
+      <c r="A77" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B77" s="1" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
+    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
+      <c r="A78" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B78" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
+    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
+      <c r="A79" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B79" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
+    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
+      <c r="A80" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B80" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="81" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
+    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
+      <c r="A81" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B81" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="82" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
+    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
+      <c r="A82" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B82" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="83" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
+    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
+      <c r="A83" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B83" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="84" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
+    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
+      <c r="A84" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B84" s="1" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="85" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
+    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
+      <c r="A85" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B85" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="86" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
+      <c r="A86" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B86" s="1" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="87" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
+      <c r="A87" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B87" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="88" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
+      <c r="A88" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B88" s="1" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="89" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
+    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
+      <c r="A89" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B89" s="1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="90" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
+    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
+      <c r="A90" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="91" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
+    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
+      <c r="A91" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B91" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="92" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
+    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
+      <c r="A92" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B92" s="1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="93" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
+    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
+      <c r="A93" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B93" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="94" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
+    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
+      <c r="A94" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B94" s="1" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="95" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
+    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
+      <c r="A95" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B95" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="96" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
+    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
+      <c r="A96" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B96" s="1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="97" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
+    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
+      <c r="A97" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B97" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="98" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
+    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
+      <c r="A98" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B98" s="1" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="99" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
+    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
+      <c r="A99" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B99" s="1" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="100" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
+    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
+      <c r="A100" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B100" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="101" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
+    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
+      <c r="A101" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B101" s="1" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="102" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
+    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
+      <c r="A102" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B102" s="1" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="103" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A103" t="s">
+    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
+      <c r="A103" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="B103" t="s">
+      <c r="B103" s="1" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="104" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A104" t="s">
+    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
+      <c r="A104" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B104" s="1" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="105" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A105" t="s">
+    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
+      <c r="A105" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B105" s="1" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="106" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
+    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
+      <c r="A106" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B106" s="1" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="107" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A107" t="s">
+    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
+      <c r="A107" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B107" s="1" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="108" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A108" t="s">
+    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75">
+      <c r="A108" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B108" s="1" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="109" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A109" t="s">
+    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75">
+      <c r="A109" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B109" s="1" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="110" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A110" t="s">
+    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
+      <c r="A110" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B110" s="1" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="111" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
+    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
+      <c r="A111" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B111" s="1" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="112" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A112" t="s">
+    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
+      <c r="A112" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="B112" t="s">
+      <c r="B112" s="1" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="113" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A113" t="s">
+    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
+      <c r="A113" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="B113" t="s">
+      <c r="B113" s="1" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="114" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
+    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
+      <c r="A114" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="B114" t="s">
+      <c r="B114" s="1" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="115" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
+    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
+      <c r="A115" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B115" s="1" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="116" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A116" t="s">
+    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
+      <c r="A116" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B116" s="1" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="117" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A117" t="s">
+    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
+      <c r="A117" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B117" t="s">
+      <c r="B117" s="1" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="118" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A118" t="s">
+    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
+      <c r="A118" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="B118" t="s">
+      <c r="B118" s="1" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="119" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A119" t="s">
+    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
+      <c r="A119" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="B119" t="s">
+      <c r="B119" s="1" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="120" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A120" t="s">
+    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
+      <c r="A120" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="B120" t="s">
+      <c r="B120" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="121" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A121" t="s">
+    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
+      <c r="A121" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B121" s="1" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="122" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A122" t="s">
+    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
+      <c r="A122" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="B122" t="s">
+      <c r="B122" s="1" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="123" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A123" t="s">
+    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
+      <c r="A123" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="B123" t="s">
+      <c r="B123" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="124" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A124" t="s">
+    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
+      <c r="A124" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B124" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="125" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A125" t="s">
+    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
+      <c r="A125" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="B125" t="s">
+      <c r="B125" s="1" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="126" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A126" t="s">
+    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
+      <c r="A126" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="B126" t="s">
+      <c r="B126" s="1" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="127" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A127" t="s">
+    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
+      <c r="A127" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B127" t="s">
+      <c r="B127" s="1" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="128" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A128" t="s">
+    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
+      <c r="A128" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="B128" t="s">
+      <c r="B128" s="1" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="129" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A129" t="s">
+    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
+      <c r="A129" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="B129" t="s">
+      <c r="B129" s="1" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="130" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A130" t="s">
+    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75">
+      <c r="A130" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B130" s="1" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="131" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A131" t="s">
+    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18.75">
+      <c r="A131" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="B131" t="s">
+      <c r="B131" s="1" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="132" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A132" t="s">
+    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18.75">
+      <c r="A132" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="B132" t="s">
+      <c r="B132" s="1" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="133" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A133" t="s">
+    <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="18.75">
+      <c r="A133" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B133" s="1" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="134" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A134" t="s">
+    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18.75">
+      <c r="A134" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="B134" t="s">
+      <c r="B134" s="1" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="135" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A135" t="s">
+    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18.75">
+      <c r="A135" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B135" s="1" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="136" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A136" t="s">
+    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18.75">
+      <c r="A136" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="B136" t="s">
+      <c r="B136" s="1" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="137" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A137" t="s">
+    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18.75">
+      <c r="A137" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="B137" t="s">
+      <c r="B137" s="1" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="138" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A138" t="s">
+    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18.75">
+      <c r="A138" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B138" s="1" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="139" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A139" t="s">
+    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18.75">
+      <c r="A139" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B139" t="s">
+      <c r="B139" s="1" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="140" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A140" t="s">
+    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18.75">
+      <c r="A140" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="B140" t="s">
+      <c r="B140" s="1" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="141" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A141" t="s">
+    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18.75">
+      <c r="A141" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B141" t="s">
+      <c r="B141" s="1" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="142" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A142" t="s">
+    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18.75">
+      <c r="A142" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="B142" t="s">
+      <c r="B142" s="1" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="143" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A143" t="s">
+    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18.75">
+      <c r="A143" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="B143" t="s">
+      <c r="B143" s="1" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="144" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A144" t="s">
+    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="18.75">
+      <c r="A144" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="B144" t="s">
+      <c r="B144" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="145" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A145" t="s">
+    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="18.75">
+      <c r="A145" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="B145" t="s">
+      <c r="B145" s="1" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="146" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A146" t="s">
+    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="18.75">
+      <c r="A146" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="B146" t="s">
+      <c r="B146" s="1" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="147" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A147" t="s">
+    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="18.75">
+      <c r="A147" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="B147" t="s">
+      <c r="B147" s="1" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="148" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A148" t="s">
+    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="18.75">
+      <c r="A148" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="B148" t="s">
+      <c r="B148" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="149" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A149" t="s">
+    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="18.75">
+      <c r="A149" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="B149" t="s">
+      <c r="B149" s="1" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="150" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A150" t="s">
+    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18.75">
+      <c r="A150" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="B150" t="s">
+      <c r="B150" s="1" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="151" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A151" t="s">
+    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18.75">
+      <c r="A151" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="B151" t="s">
+      <c r="B151" s="1" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="152" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A152" t="s">
+    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18.75">
+      <c r="A152" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="B152" t="s">
+      <c r="B152" s="1" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="153" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A153" t="s">
+    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="18.75">
+      <c r="A153" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="B153" t="s">
+      <c r="B153" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="154" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A154" t="s">
+    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18.75">
+      <c r="A154" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="B154" t="s">
+      <c r="B154" s="1" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="155" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A155" t="s">
+    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18.75">
+      <c r="A155" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="B155" t="s">
+      <c r="B155" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="156" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A156" t="s">
+    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18.75">
+      <c r="A156" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="B156" t="s">
+      <c r="B156" s="1" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="157" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A157" t="s">
+    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18.75">
+      <c r="A157" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="B157" t="s">
+      <c r="B157" s="1" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="158" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A158" t="s">
+    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18.75">
+      <c r="A158" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="B158" t="s">
+      <c r="B158" s="1" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="159" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A159" t="s">
+    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18.75">
+      <c r="A159" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="B159" t="s">
+      <c r="B159" s="1" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="160" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A160" t="s">
+    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18.75">
+      <c r="A160" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="B160" t="s">
+      <c r="B160" s="1" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="161" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A161" t="s">
+    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18.75">
+      <c r="A161" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="B161" t="s">
+      <c r="B161" s="1" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="162" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A162" t="s">
+    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18.75">
+      <c r="A162" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="B162" t="s">
+      <c r="B162" s="1" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="163" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A163" t="s">
+    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75">
+      <c r="A163" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="B163" t="s">
+      <c r="B163" s="1" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="164" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A164" t="s">
+    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75">
+      <c r="A164" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="B164" t="s">
+      <c r="B164" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="165" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A165" t="s">
+    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75">
+      <c r="A165" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B165" t="s">
+      <c r="B165" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="166" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A166" t="s">
+    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75">
+      <c r="A166" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="B166" t="s">
+      <c r="B166" s="1" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="167" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A167" t="s">
+    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75">
+      <c r="A167" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="B167" t="s">
+      <c r="B167" s="1" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="168" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A168" t="s">
+    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="19.5">
+      <c r="A168" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B168" t="s">
+      <c r="B168" s="1" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="169" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A169" t="s">
+    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="18.75">
+      <c r="A169" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="B169" t="s">
+      <c r="B169" s="1" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="170" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A170" t="s">
+    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18.75">
+      <c r="A170" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="B170" t="s">
+      <c r="B170" s="1" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="171" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A171" t="s">
+    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18.75">
+      <c r="A171" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="B171" t="s">
+      <c r="B171" s="1" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="172" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="19.5">
       <c r="A172" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18.75">
+      <c r="A173" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="B172" s="2" t="s">
+      <c r="B173" s="1" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="173" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A173" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="B173" s="3" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A174" t="s">
+    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18.75">
+      <c r="A174" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="B174" t="s">
+      <c r="B174" s="1" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="175" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A175" t="s">
+    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18.75">
+      <c r="A175" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="B175" t="s">
+      <c r="B175" s="1" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="176" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A176" t="s">
+    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18.75">
+      <c r="A176" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="B176" t="s">
+      <c r="B176" s="1" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="177" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A177" t="s">
+    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="18.75">
+      <c r="A177" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B177" t="s">
+      <c r="B177" s="1" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="178" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A178" t="s">
+    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18.75">
+      <c r="A178" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="B178" t="s">
+      <c r="B178" s="1" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="179" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A179" t="s">
+    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18.75">
+      <c r="A179" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="B179" t="s">
+      <c r="B179" s="1" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="180" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A180" t="s">
+    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18.75">
+      <c r="A180" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="B180" t="s">
+      <c r="B180" s="1" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="181" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A181" t="s">
+    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18.75">
+      <c r="A181" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="B181" t="s">
+      <c r="B181" s="1" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="182" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A182" t="s">
+    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18.75">
+      <c r="A182" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="B182" t="s">
+      <c r="B182" s="1" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="183" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A183" t="s">
+    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18.75">
+      <c r="A183" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="B183" t="s">
+      <c r="B183" s="1" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="184" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A184" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="19.5">
+      <c r="A184" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="B184" s="1" t="s">
+      <c r="B184" s="2" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="185" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A185" t="s">
+    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18.75">
+      <c r="A185" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="B185" t="s">
+      <c r="B185" s="1" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="186" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A186" t="s">
+    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75">
+      <c r="A186" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="B186" t="s">
+      <c r="B186" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="187" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A187" t="s">
+    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18.75">
+      <c r="A187" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="B187" t="s">
+      <c r="B187" s="1" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="188" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A188" t="s">
+    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75">
+      <c r="A188" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="B188" t="s">
+      <c r="B188" s="1" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="189" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A189" t="s">
+    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75">
+      <c r="A189" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="B189" t="s">
+      <c r="B189" s="1" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="190" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A190" t="s">
+    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75">
+      <c r="A190" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="B190" t="s">
+      <c r="B190" s="1" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="191" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A191" t="s">
+    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18.75">
+      <c r="A191" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="B191" t="s">
+      <c r="B191" s="1" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="192" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A192" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="19.5">
+      <c r="A192" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="B192" s="1" t="s">
+      <c r="B192" s="2" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="193" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A193" t="s">
+    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18.75">
+      <c r="A193" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="B193" t="s">
+      <c r="B193" s="1" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="194" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A194" t="s">
+    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="18.75">
+      <c r="A194" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="B194" t="s">
+      <c r="B194" s="1" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="195" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A195" t="s">
+    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18.75">
+      <c r="A195" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="B195" t="s">
+      <c r="B195" s="1" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="196" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A196" t="s">
+    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="18.75">
+      <c r="A196" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="B196" t="s">
+      <c r="B196" s="1" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="197" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A197" t="s">
+    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18.75">
+      <c r="A197" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="B197" t="s">
+      <c r="B197" s="1" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="198" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A198" t="s">
+    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="18.75">
+      <c r="A198" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="B198" t="s">
+      <c r="B198" s="1" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="199" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A199" t="s">
+    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="18.75">
+      <c r="A199" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="B199" t="s">
+      <c r="B199" s="1" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="200" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A200" t="s">
+    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="18.75">
+      <c r="A200" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="B200" t="s">
+      <c r="B200" s="1" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="201" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A201" t="s">
+    <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="18.75">
+      <c r="A201" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B201" t="s">
+      <c r="B201" s="1" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="202" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A202" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="20.25">
+      <c r="A202" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="B202" s="1" t="s">
+      <c r="B202" s="2" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="203" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A203" t="s">
+    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="19.5">
+      <c r="A203" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="B203" t="s">
+      <c r="B203" s="1" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="204" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A204" t="s">
+    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="19.5">
+      <c r="A204" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="B204" t="s">
+      <c r="B204" s="1" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="205" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A205" t="s">
+    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="19.5">
+      <c r="A205" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="B205" t="s">
+      <c r="B205" s="1" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="206" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A206" t="s">
+    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="19.5">
+      <c r="A206" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="B206" t="s">
+      <c r="B206" s="1" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="207" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A207" t="s">
+    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="19.5">
+      <c r="A207" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="B207" t="s">
+      <c r="B207" s="1" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="208" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A208" t="s">
+    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="19.5">
+      <c r="A208" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="B208" t="s">
+      <c r="B208" s="1" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="209" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A209" t="s">
+    <row x14ac:dyDescent="0.25" r="209" customHeight="1" ht="18.75">
+      <c r="A209" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="B209" t="s">
+      <c r="B209" s="1" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="210" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A210" t="s">
+    <row x14ac:dyDescent="0.25" r="210" customHeight="1" ht="18.75">
+      <c r="A210" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="B210" t="s">
+      <c r="B210" s="1" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="211" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A211" t="s">
+    <row x14ac:dyDescent="0.25" r="211" customHeight="1" ht="18.75">
+      <c r="A211" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="B211" t="s">
+      <c r="B211" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="212" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A212" t="s">
+    <row x14ac:dyDescent="0.25" r="212" customHeight="1" ht="18.75">
+      <c r="A212" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="B212" t="s">
+      <c r="B212" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="213" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A213" t="s">
+    <row x14ac:dyDescent="0.25" r="213" customHeight="1" ht="18.75">
+      <c r="A213" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="B213" t="s">
+      <c r="B213" s="1" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="214" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A214" t="s">
+    <row x14ac:dyDescent="0.25" r="214" customHeight="1" ht="18.75">
+      <c r="A214" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="B214" t="s">
+      <c r="B214" s="1" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="215" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A215" t="s">
+    <row x14ac:dyDescent="0.25" r="215" customHeight="1" ht="18.75">
+      <c r="A215" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="B215" t="s">
+      <c r="B215" s="1" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="216" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A216" t="s">
+    <row x14ac:dyDescent="0.25" r="216" customHeight="1" ht="18.75">
+      <c r="A216" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="B216" t="s">
+      <c r="B216" s="1" t="s">
         <v>415</v>
       </c>
     </row>
-    <row r="217" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A217" t="s">
+    <row x14ac:dyDescent="0.25" r="217" customHeight="1" ht="18.75">
+      <c r="A217" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="B217" t="s">
+      <c r="B217" s="1" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="218" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="218" customHeight="1" ht="19.5">
       <c r="A218" s="1" t="s">
         <v>418</v>
       </c>
@@ -3811,7 +3879,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="219" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row x14ac:dyDescent="0.25" r="219" customHeight="1" ht="19.5">
       <c r="A219" s="1" t="s">
         <v>420</v>
       </c>
@@ -3819,564 +3887,663 @@
         <v>421</v>
       </c>
     </row>
-    <row r="220" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A220" t="s">
+    <row x14ac:dyDescent="0.25" r="220" customHeight="1" ht="19.5">
+      <c r="A220" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="B220" t="s">
+      <c r="B220" s="1" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="221" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A221" t="s">
+    <row x14ac:dyDescent="0.25" r="221" customHeight="1" ht="19.5">
+      <c r="A221" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="B221" t="s">
+      <c r="B221" s="1" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="222" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A222" t="s">
+    <row x14ac:dyDescent="0.25" r="222" customHeight="1" ht="19.5">
+      <c r="A222" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="B222" t="s">
+      <c r="B222" s="1" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="223" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A223" t="s">
+    <row x14ac:dyDescent="0.25" r="223" customHeight="1" ht="19.5">
+      <c r="A223" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="B223" t="s">
+      <c r="B223" s="1" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="224" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A224" t="s">
+    <row x14ac:dyDescent="0.25" r="224" customHeight="1" ht="19.5">
+      <c r="A224" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="B224" t="s">
+      <c r="B224" s="1" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="225" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A225" t="s">
+    <row x14ac:dyDescent="0.25" r="225" customHeight="1" ht="19.5">
+      <c r="A225" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="B225" t="s">
+      <c r="B225" s="1" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="226" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A226" t="s">
+    <row x14ac:dyDescent="0.25" r="226" customHeight="1" ht="19.5">
+      <c r="A226" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="B226" t="s">
+      <c r="B226" s="1" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="227" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A227" t="s">
+    <row x14ac:dyDescent="0.25" r="227" customHeight="1" ht="19.5">
+      <c r="A227" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="B227" s="1" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="228" customHeight="1" ht="18.75">
+      <c r="A228" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="B228" s="2" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="229" customHeight="1" ht="18.75">
+      <c r="A229" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="B229" s="2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="230" customHeight="1" ht="18.75">
+      <c r="A230" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="B230" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="231" customHeight="1" ht="18.75">
+      <c r="A231" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="B231" s="1" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="232" customHeight="1" ht="18.75">
+      <c r="A232" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="B232" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="233" customHeight="1" ht="18.75">
+      <c r="A233" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="B233" s="1" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="234" customHeight="1" ht="18.75">
+      <c r="A234" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="B234" s="1" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="235" customHeight="1" ht="18.75">
+      <c r="A235" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="B235" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="236" customHeight="1" ht="18.75">
+      <c r="A236" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="B236" s="1" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="237" customHeight="1" ht="18.75">
+      <c r="A237" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="B237" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="238" customHeight="1" ht="18.75">
+      <c r="A238" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B238" s="1" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="239" customHeight="1" ht="18.75">
+      <c r="A239" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B239" s="1" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="240" customHeight="1" ht="18.75">
+      <c r="A240" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="B240" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="241" customHeight="1" ht="18.75">
+      <c r="A241" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="B241" s="1" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="242" customHeight="1" ht="18.75">
+      <c r="A242" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="B242" s="1" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="243" customHeight="1" ht="18.75">
+      <c r="A243" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B243" s="1" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="244" customHeight="1" ht="18.75">
+      <c r="A244" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="245" customHeight="1" ht="18.75">
+      <c r="A245" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="B245" s="1" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="246" customHeight="1" ht="18.75">
+      <c r="A246" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="B246" s="1" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="247" customHeight="1" ht="18.75">
+      <c r="A247" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="B247" s="1" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="248" customHeight="1" ht="18.75">
+      <c r="A248" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="B248" s="1" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="249" customHeight="1" ht="18.75">
+      <c r="A249" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="B249" s="1" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="250" customHeight="1" ht="18.75">
+      <c r="A250" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="B250" s="1" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="251" customHeight="1" ht="18.75">
+      <c r="A251" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B251" s="1" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="252" customHeight="1" ht="18.75">
+      <c r="A252" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="B252" s="1" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="253" customHeight="1" ht="18.75">
+      <c r="A253" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B253" s="1" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="254" customHeight="1" ht="18.75">
+      <c r="A254" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="B254" s="1" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="255" customHeight="1" ht="18.75">
+      <c r="A255" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="B255" s="1" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="256" customHeight="1" ht="18.75">
+      <c r="A256" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="B256" s="1" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="257" customHeight="1" ht="18.75">
+      <c r="A257" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B257" s="1" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="258" customHeight="1" ht="18.75">
+      <c r="A258" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="B258" s="1" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="259" customHeight="1" ht="18.75">
+      <c r="A259" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="B259" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="260" customHeight="1" ht="18.75">
+      <c r="A260" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="B260" s="2" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="18.75">
+      <c r="A261" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="B261" s="1" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="18.75">
+      <c r="A262" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="B262" s="2" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="263" customHeight="1" ht="18.75">
+      <c r="A263" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="B263" s="2" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="264" customHeight="1" ht="18.75">
+      <c r="A264" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="B264" s="2" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="265" customHeight="1" ht="18.75">
+      <c r="A265" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="B265" s="1" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="266" customHeight="1" ht="18.75">
+      <c r="A266" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="B266" s="1" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="267" customHeight="1" ht="18.75">
+      <c r="A267" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="B267" s="1" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="268" customHeight="1" ht="18.75">
+      <c r="A268" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="B268" s="1" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="269" customHeight="1" ht="18.75">
+      <c r="A269" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="B269" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="270" customHeight="1" ht="18.75">
+      <c r="A270" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="B270" s="1" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="271" customHeight="1" ht="18.75">
+      <c r="A271" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="B271" s="1" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="18.75">
+      <c r="A272" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="B272" s="2" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="273" customHeight="1" ht="18.75">
+      <c r="A273" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="B273" s="1" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="18.75">
+      <c r="A274" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="B274" s="1" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="275" customHeight="1" ht="18.75">
+      <c r="A275" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="B275" s="1" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="276" customHeight="1" ht="18.75">
+      <c r="A276" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="B276" s="1" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="277" customHeight="1" ht="18.75">
+      <c r="A277" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="B277" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="18.75">
+      <c r="A278" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="B278" s="1" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="279" customHeight="1" ht="18.75">
+      <c r="A279" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="B279" s="1" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="280" customHeight="1" ht="18.75">
+      <c r="A280" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="B280" s="1" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="281" customHeight="1" ht="18.75">
+      <c r="A281" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="B281" s="1" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="282" customHeight="1" ht="18.75">
+      <c r="A282" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="B282" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="283" customHeight="1" ht="18.75">
+      <c r="A283" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="B283" s="1" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="284" customHeight="1" ht="18.75">
+      <c r="A284" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="B284" s="1" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="285" customHeight="1" ht="18.75">
+      <c r="A285" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="B285" s="1" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="286" customHeight="1" ht="18.75">
+      <c r="A286" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="B286" s="1" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="287" customHeight="1" ht="18.75">
+      <c r="A287" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="B227" t="s">
+      <c r="B287" s="1" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="288" customHeight="1" ht="18.75">
+      <c r="A288" s="2" t="s">
         <v>555</v>
       </c>
-    </row>
-    <row r="228" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A228" t="s">
-        <v>551</v>
-      </c>
-      <c r="B228" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="229" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A229" t="s">
-        <v>554</v>
-      </c>
-      <c r="B229" t="s">
+      <c r="B288" s="2" t="s">
         <v>556</v>
       </c>
     </row>
-    <row r="230" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A230" t="s">
-        <v>436</v>
-      </c>
-      <c r="B230" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="231" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A231" t="s">
-        <v>438</v>
-      </c>
-      <c r="B231" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="232" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A232" t="s">
-        <v>440</v>
-      </c>
-      <c r="B232" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="233" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A233" t="s">
-        <v>442</v>
-      </c>
-      <c r="B233" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="234" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A234" t="s">
-        <v>444</v>
-      </c>
-      <c r="B234" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="235" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A235" t="s">
-        <v>446</v>
-      </c>
-      <c r="B235" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="236" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A236" t="s">
-        <v>448</v>
-      </c>
-      <c r="B236" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="237" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A237" t="s">
-        <v>450</v>
-      </c>
-      <c r="B237" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="238" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A238" t="s">
-        <v>452</v>
-      </c>
-      <c r="B238" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="239" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A239" t="s">
-        <v>454</v>
-      </c>
-      <c r="B239" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="240" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A240" t="s">
-        <v>456</v>
-      </c>
-      <c r="B240" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="241" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A241" t="s">
-        <v>458</v>
-      </c>
-      <c r="B241" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="242" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A242" t="s">
-        <v>460</v>
-      </c>
-      <c r="B242" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="243" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A243" t="s">
-        <v>462</v>
-      </c>
-      <c r="B243" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="244" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A244" s="2" t="s">
-        <v>464</v>
-      </c>
-      <c r="B244" s="2" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="245" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A245" t="s">
-        <v>466</v>
-      </c>
-      <c r="B245" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="246" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A246" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="B246" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="247" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A247" s="1" t="s">
-        <v>469</v>
-      </c>
-      <c r="B247" s="1" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="248" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A248" s="2" t="s">
-        <v>471</v>
-      </c>
-      <c r="B248" s="2" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="249" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A249" s="4" t="s">
-        <v>473</v>
-      </c>
-      <c r="B249" s="4" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="250" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A250" s="4" t="s">
-        <v>475</v>
-      </c>
-      <c r="B250" s="4" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="251" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A251" s="3" t="s">
-        <v>477</v>
-      </c>
-      <c r="B251" s="3" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="252" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A252" t="s">
-        <v>479</v>
-      </c>
-      <c r="B252" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="253" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A253" t="s">
-        <v>481</v>
-      </c>
-      <c r="B253" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="254" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A254" t="s">
-        <v>483</v>
-      </c>
-      <c r="B254" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="255" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A255" t="s">
-        <v>485</v>
-      </c>
-      <c r="B255" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="256" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A256" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="B256" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="257" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A257" t="s">
-        <v>488</v>
-      </c>
-      <c r="B257" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="258" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A258" s="5" t="s">
-        <v>490</v>
-      </c>
-      <c r="B258" s="5" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="259" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A259" s="3" t="s">
-        <v>492</v>
-      </c>
-      <c r="B259" s="3" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="260" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A260" t="s">
-        <v>494</v>
-      </c>
-      <c r="B260" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="261" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A261" t="s">
-        <v>496</v>
-      </c>
-      <c r="B261" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="262" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A262" t="s">
-        <v>498</v>
-      </c>
-      <c r="B262" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="263" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A263" t="s">
-        <v>499</v>
-      </c>
-      <c r="B263" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="264" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A264" t="s">
-        <v>501</v>
-      </c>
-      <c r="B264" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="265" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A265" t="s">
-        <v>503</v>
-      </c>
-      <c r="B265" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="266" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A266" t="s">
-        <v>505</v>
-      </c>
-      <c r="B266" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="267" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A267" t="s">
-        <v>507</v>
-      </c>
-      <c r="B267" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="268" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A268" t="s">
-        <v>509</v>
-      </c>
-      <c r="B268" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="269" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A269" t="s">
-        <v>511</v>
-      </c>
-      <c r="B269" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="270" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A270" t="s">
-        <v>513</v>
-      </c>
-      <c r="B270" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="271" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A271" t="s">
-        <v>515</v>
-      </c>
-      <c r="B271" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="272" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A272" s="2" t="s">
-        <v>517</v>
-      </c>
-      <c r="B272" s="2" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="273" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A273" t="s">
-        <v>519</v>
-      </c>
-      <c r="B273" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="274" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A274" s="5" t="s">
-        <v>521</v>
-      </c>
-      <c r="B274" s="5" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="275" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A275" s="3" t="s">
-        <v>523</v>
-      </c>
-      <c r="B275" s="3" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="276" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A276" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="B276" s="2" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="277" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A277" t="s">
-        <v>527</v>
-      </c>
-      <c r="B277" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="278" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A278" s="5" t="s">
-        <v>529</v>
-      </c>
-      <c r="B278" s="5" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="279" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A279" s="3" t="s">
-        <v>531</v>
-      </c>
-      <c r="B279" s="3" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="280" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A280" t="s">
-        <v>533</v>
-      </c>
-      <c r="B280" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="281" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A281" t="s">
-        <v>535</v>
-      </c>
-      <c r="B281" t="s">
-        <v>536</v>
-      </c>
-    </row>
-    <row r="282" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A282" t="s">
-        <v>537</v>
-      </c>
-      <c r="B282" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="283" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A283" t="s">
-        <v>539</v>
-      </c>
-      <c r="B283" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A284" t="s">
-        <v>541</v>
-      </c>
-      <c r="B284" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="285" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A285" t="s">
-        <v>543</v>
-      </c>
-      <c r="B285" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="286" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A286" t="s">
-        <v>545</v>
-      </c>
-      <c r="B286" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A287" t="s">
-        <v>547</v>
-      </c>
-      <c r="B287" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A288" t="s">
-        <v>549</v>
-      </c>
-      <c r="B288" t="s">
-        <v>550</v>
+    <row x14ac:dyDescent="0.25" r="289" customHeight="1" ht="18.75">
+      <c r="A289" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="B289" s="1" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="290" customHeight="1" ht="18.75">
+      <c r="A290" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="291" customHeight="1" ht="18.75">
+      <c r="A291" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="B291" s="1" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="292" customHeight="1" ht="18.75">
+      <c r="A292" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B292" s="2" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="293" customHeight="1" ht="18.75">
+      <c r="A293" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="B293" s="1" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="294" customHeight="1" ht="18.75">
+      <c r="A294" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="B294" s="1" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="295" customHeight="1" ht="18.75">
+      <c r="A295" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="B295" s="1" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="296" customHeight="1" ht="18.75">
+      <c r="A296" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="B296" s="1" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="297" customHeight="1" ht="18.75">
+      <c r="A297" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="B297" s="1" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="298" customHeight="1" ht="18.75">
+      <c r="A298" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="B298" s="1" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="299" customHeight="1" ht="18.75">
+      <c r="A299" s="1" t="s">
+        <v>577</v>
+      </c>
+      <c r="B299" s="1" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="300" customHeight="1" ht="18.75">
+      <c r="A300" s="1" t="s">
+        <v>579</v>
+      </c>
+      <c r="B300" s="1" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="301" customHeight="1" ht="18.75">
+      <c r="A301" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="B301" s="1" t="s">
+        <v>582</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B288" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B288">
-      <sortCondition ref="A1:A288"/>
-    </sortState>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add prescription line list
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -1,29 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia\Documents\GitHub\tamanu-source-dbt\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74409AB8-E8B9-4DE4-AACE-7B87B9E1ADBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14390" yWindow="-10" windowWidth="14420" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Translated String" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Translated String"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Translated String'!$A$1:$B$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="585">
   <si>
     <t>stringId</t>
   </si>
@@ -1009,18 +1003,18 @@
     <t>Edited by user</t>
   </si>
   <si>
+    <t>report.reporting.logChangeDateTime</t>
+  </si>
+  <si>
+    <t>Date and time edited</t>
+  </si>
+  <si>
     <t>report.reporting.logChangeRecordCreatedDateTime</t>
   </si>
   <si>
     <t>Date and time created</t>
   </si>
   <si>
-    <t>report.reporting.logChangeDateTime</t>
-  </si>
-  <si>
-    <t>Date and time edited</t>
-  </si>
-  <si>
     <t>report.reporting.medications</t>
   </si>
   <si>
@@ -1279,6 +1273,24 @@
     <t>Social security number</t>
   </si>
   <si>
+    <t>report.reporting.patientStreetVillage</t>
+  </si>
+  <si>
+    <t>Street / Village</t>
+  </si>
+  <si>
+    <t>report.reporting.patientSubDivision</t>
+  </si>
+  <si>
+    <t>Sub-division</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTitle</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
     <t>report.reporting.patientTotal</t>
   </si>
   <si>
@@ -1339,24 +1351,6 @@
     <t>Total patients with missing location</t>
   </si>
   <si>
-    <t>report.reporting.patientStreetVillage</t>
-  </si>
-  <si>
-    <t>Street / Village</t>
-  </si>
-  <si>
-    <t>report.reporting.patientSubDivision</t>
-  </si>
-  <si>
-    <t>Sub-division</t>
-  </si>
-  <si>
-    <t>report.reporting.patientTitle</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
     <t>report.reporting.patientVillage</t>
   </si>
   <si>
@@ -1393,6 +1387,36 @@
     <t>Tamanu user name</t>
   </si>
   <si>
+    <t>report.reporting.prescriptionDate</t>
+  </si>
+  <si>
+    <t>Prescription date</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedication</t>
+  </si>
+  <si>
+    <t>Medication</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedicationCode</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionQuantity</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionSelectedForDischarge</t>
+  </si>
+  <si>
+    <t>Prescription selected for discharge</t>
+  </si>
+  <si>
     <t>report.reporting.procedure</t>
   </si>
   <si>
@@ -1748,37 +1772,26 @@
   </si>
   <si>
     <t>Schedule</t>
-  </si>
-  <si>
-    <t>report.reporting.prescriptionMedication</t>
-  </si>
-  <si>
-    <t>Medication</t>
-  </si>
-  <si>
-    <t>report.reporting.prescriptionMedicationCode</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>report.reporting.prescriptionQuantity</t>
-  </si>
-  <si>
-    <t>Quantity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1814,24 +1827,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="5">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1842,10 +1860,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -1883,71 +1901,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1975,7 +1993,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1998,11 +2016,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -2011,13 +2029,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -2027,7 +2045,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -2036,7 +2054,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -2045,7 +2063,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -2053,10 +2071,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -2121,2415 +2139,2431 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B300"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:B302"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="64.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="4" width="64.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="35.71928571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+      <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+      <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+      <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+      <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+      <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+      <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+      <c r="A22" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+      <c r="A23" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+      <c r="A24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+      <c r="A25" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+      <c r="A26" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" t="s">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+      <c r="A27" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A28" t="s">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+      <c r="A28" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" t="s">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+      <c r="A29" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" t="s">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+      <c r="A30" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" t="s">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+      <c r="A31" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
+      <c r="A32" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" t="s">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
+      <c r="A33" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" t="s">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
+      <c r="A34" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
+      <c r="A35" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" t="s">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
+      <c r="A36" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" t="s">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
+      <c r="A37" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A38" t="s">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
+      <c r="A38" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A39" t="s">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
+      <c r="A39" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" t="s">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
+      <c r="A40" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" t="s">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
+      <c r="A41" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A42" t="s">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
+      <c r="A42" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A43" t="s">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
+      <c r="A43" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A44" t="s">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
+      <c r="A44" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A45" t="s">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
+      <c r="A45" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A46" t="s">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
+      <c r="A46" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A47" t="s">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
+      <c r="A47" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A48" t="s">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
+      <c r="A48" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A49" t="s">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
+      <c r="A49" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A50" t="s">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
+      <c r="A50" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A51" t="s">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
+      <c r="A51" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A52" t="s">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
+      <c r="A52" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A53" t="s">
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
+      <c r="A53" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A54" t="s">
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
+      <c r="A54" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A55" t="s">
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
+      <c r="A55" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A56" t="s">
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
+      <c r="A56" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A57" t="s">
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
+      <c r="A57" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="1" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A58" t="s">
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
+      <c r="A58" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A59" t="s">
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
+      <c r="A59" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A60" t="s">
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
+      <c r="A60" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A61" t="s">
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
+      <c r="A61" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B61" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A62" t="s">
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
+      <c r="A62" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B62" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A63" t="s">
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
+      <c r="A63" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B63" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A64" t="s">
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
+      <c r="A64" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B64" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A65" t="s">
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
+      <c r="A65" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A66" t="s">
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
+      <c r="A66" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A67" t="s">
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
+      <c r="A67" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B67" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A68" t="s">
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
+      <c r="A68" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A69" t="s">
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
+      <c r="A69" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A70" t="s">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
+      <c r="A70" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B70" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A71" t="s">
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
+      <c r="A71" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A72" t="s">
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
+      <c r="A72" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A73" t="s">
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
+      <c r="A73" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A74" t="s">
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
+      <c r="A74" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B74" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A75" t="s">
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
+      <c r="A75" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B75" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A76" t="s">
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
+      <c r="A76" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B76" s="1" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A77" t="s">
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
+      <c r="A77" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B77" s="1" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A78" t="s">
+    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
+      <c r="A78" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B78" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A79" t="s">
+    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
+      <c r="A79" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B79" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A80" t="s">
+    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
+      <c r="A80" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B80" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="81" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A81" t="s">
+    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
+      <c r="A81" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B81" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="82" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A82" t="s">
+    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
+      <c r="A82" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B82" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="83" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A83" t="s">
+    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
+      <c r="A83" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B83" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="84" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A84" t="s">
+    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
+      <c r="A84" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B84" s="1" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="85" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A85" t="s">
+    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
+      <c r="A85" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B85" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="86" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A86" t="s">
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
+      <c r="A86" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B86" s="1" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="87" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A87" t="s">
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
+      <c r="A87" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B87" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="88" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A88" t="s">
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
+      <c r="A88" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B88" s="1" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="89" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A89" t="s">
+    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
+      <c r="A89" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B89" s="1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="90" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A90" t="s">
+    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
+      <c r="A90" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="91" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A91" t="s">
+    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
+      <c r="A91" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B91" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="92" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A92" t="s">
+    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
+      <c r="A92" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B92" s="1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="93" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A93" t="s">
+    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
+      <c r="A93" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B93" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="94" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A94" t="s">
+    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
+      <c r="A94" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B94" s="1" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="95" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A95" t="s">
+    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
+      <c r="A95" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B95" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="96" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A96" t="s">
+    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
+      <c r="A96" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B96" s="1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="97" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A97" t="s">
+    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
+      <c r="A97" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B97" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="98" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A98" t="s">
+    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
+      <c r="A98" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B98" s="1" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="99" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A99" t="s">
+    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
+      <c r="A99" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B99" s="1" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="100" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A100" t="s">
+    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
+      <c r="A100" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B100" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="101" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A101" t="s">
+    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
+      <c r="A101" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B101" s="1" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="102" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A102" t="s">
+    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
+      <c r="A102" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B102" s="1" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="103" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A103" t="s">
+    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
+      <c r="A103" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="B103" t="s">
+      <c r="B103" s="1" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="104" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A104" t="s">
+    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
+      <c r="A104" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B104" s="1" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="105" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A105" t="s">
+    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
+      <c r="A105" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B105" s="1" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="106" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A106" t="s">
+    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
+      <c r="A106" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B106" s="1" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="107" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A107" t="s">
+    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
+      <c r="A107" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B107" s="1" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="108" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A108" t="s">
+    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75">
+      <c r="A108" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B108" s="1" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="109" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A109" t="s">
+    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75">
+      <c r="A109" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B109" s="1" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="110" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A110" t="s">
+    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
+      <c r="A110" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B110" s="1" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="111" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A111" t="s">
+    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
+      <c r="A111" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B111" s="1" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="112" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A112" t="s">
+    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
+      <c r="A112" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="B112" t="s">
+      <c r="B112" s="1" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="113" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A113" t="s">
+    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
+      <c r="A113" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="B113" t="s">
+      <c r="B113" s="1" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="114" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A114" t="s">
+    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
+      <c r="A114" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="B114" t="s">
+      <c r="B114" s="1" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="115" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A115" t="s">
+    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
+      <c r="A115" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B115" s="1" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="116" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A116" t="s">
+    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
+      <c r="A116" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B116" s="1" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="117" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A117" t="s">
+    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
+      <c r="A117" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B117" t="s">
+      <c r="B117" s="1" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="118" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A118" t="s">
+    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
+      <c r="A118" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="B118" t="s">
+      <c r="B118" s="1" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="119" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A119" t="s">
+    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
+      <c r="A119" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="B119" t="s">
+      <c r="B119" s="1" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="120" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A120" t="s">
+    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
+      <c r="A120" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="B120" t="s">
+      <c r="B120" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="121" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A121" t="s">
+    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
+      <c r="A121" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B121" s="1" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="122" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A122" t="s">
+    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
+      <c r="A122" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="B122" t="s">
+      <c r="B122" s="1" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="123" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A123" t="s">
+    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
+      <c r="A123" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="B123" t="s">
+      <c r="B123" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="124" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A124" t="s">
+    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
+      <c r="A124" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B124" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="125" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A125" t="s">
+    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
+      <c r="A125" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="B125" t="s">
+      <c r="B125" s="1" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="126" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A126" t="s">
+    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
+      <c r="A126" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="B126" t="s">
+      <c r="B126" s="1" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="127" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A127" t="s">
+    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
+      <c r="A127" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B127" t="s">
+      <c r="B127" s="1" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="128" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A128" t="s">
+    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
+      <c r="A128" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="B128" t="s">
+      <c r="B128" s="1" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="129" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A129" t="s">
+    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
+      <c r="A129" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="B129" t="s">
+      <c r="B129" s="1" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="130" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A130" t="s">
+    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75">
+      <c r="A130" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B130" s="1" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="131" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A131" t="s">
+    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18.75">
+      <c r="A131" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="B131" t="s">
+      <c r="B131" s="1" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="132" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A132" t="s">
+    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18.75">
+      <c r="A132" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="B132" t="s">
+      <c r="B132" s="1" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="133" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A133" t="s">
+    <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="18.75">
+      <c r="A133" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B133" s="1" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="134" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A134" t="s">
+    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18.75">
+      <c r="A134" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="B134" t="s">
+      <c r="B134" s="1" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="135" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A135" t="s">
+    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18.75">
+      <c r="A135" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B135" s="1" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="136" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A136" t="s">
+    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18.75">
+      <c r="A136" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="B136" t="s">
+      <c r="B136" s="1" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="137" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A137" t="s">
+    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18.75">
+      <c r="A137" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="B137" t="s">
+      <c r="B137" s="1" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="138" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A138" t="s">
+    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18.75">
+      <c r="A138" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B138" s="1" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="139" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A139" t="s">
+    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18.75">
+      <c r="A139" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B139" t="s">
+      <c r="B139" s="1" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="140" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A140" t="s">
+    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18.75">
+      <c r="A140" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="B140" t="s">
+      <c r="B140" s="1" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="141" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A141" t="s">
+    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18.75">
+      <c r="A141" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B141" t="s">
+      <c r="B141" s="1" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="142" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A142" t="s">
+    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18.75">
+      <c r="A142" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="B142" t="s">
+      <c r="B142" s="1" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="143" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A143" t="s">
+    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18.75">
+      <c r="A143" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="B143" t="s">
+      <c r="B143" s="1" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="144" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A144" t="s">
+    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="18.75">
+      <c r="A144" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="B144" t="s">
+      <c r="B144" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="145" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A145" t="s">
+    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="18.75">
+      <c r="A145" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="B145" t="s">
+      <c r="B145" s="1" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="146" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A146" t="s">
+    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="18.75">
+      <c r="A146" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="B146" t="s">
+      <c r="B146" s="1" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="147" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A147" t="s">
+    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="18.75">
+      <c r="A147" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="B147" t="s">
+      <c r="B147" s="1" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="148" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A148" t="s">
+    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="18.75">
+      <c r="A148" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="B148" t="s">
+      <c r="B148" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="149" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A149" t="s">
+    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="18.75">
+      <c r="A149" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="B149" t="s">
+      <c r="B149" s="1" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="150" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A150" t="s">
+    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18.75">
+      <c r="A150" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="B150" t="s">
+      <c r="B150" s="1" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="151" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A151" t="s">
+    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18.75">
+      <c r="A151" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="B151" t="s">
+      <c r="B151" s="1" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="152" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A152" t="s">
+    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18.75">
+      <c r="A152" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="B152" t="s">
+      <c r="B152" s="1" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="153" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A153" t="s">
+    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="18.75">
+      <c r="A153" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="B153" t="s">
+      <c r="B153" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="154" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A154" t="s">
+    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18.75">
+      <c r="A154" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="B154" t="s">
+      <c r="B154" s="1" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="155" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A155" t="s">
+    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18.75">
+      <c r="A155" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="B155" t="s">
+      <c r="B155" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="156" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A156" t="s">
+    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18.75">
+      <c r="A156" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="B156" t="s">
+      <c r="B156" s="1" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="157" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A157" t="s">
+    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18.75">
+      <c r="A157" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="B157" t="s">
+      <c r="B157" s="1" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="158" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A158" t="s">
+    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18.75">
+      <c r="A158" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="B158" t="s">
+      <c r="B158" s="1" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="159" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A159" t="s">
+    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18.75">
+      <c r="A159" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="B159" t="s">
+      <c r="B159" s="1" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="160" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A160" t="s">
+    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18.75">
+      <c r="A160" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="B160" t="s">
+      <c r="B160" s="1" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="161" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A161" t="s">
+    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18.75">
+      <c r="A161" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="B161" t="s">
+      <c r="B161" s="1" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="162" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A162" t="s">
+    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18.75">
+      <c r="A162" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="B162" t="s">
+      <c r="B162" s="1" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="163" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A163" t="s">
+    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75">
+      <c r="A163" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="B163" t="s">
+      <c r="B163" s="1" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="164" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A164" t="s">
+    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75">
+      <c r="A164" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="B164" t="s">
+      <c r="B164" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="165" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A165" t="s">
+    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75">
+      <c r="A165" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B165" t="s">
+      <c r="B165" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="166" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A166" t="s">
+    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75">
+      <c r="A166" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="B166" t="s">
+      <c r="B166" s="1" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="167" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A167" t="s">
+    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75">
+      <c r="A167" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="B167" t="s">
+      <c r="B167" s="1" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="168" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A168" t="s">
+    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="19.5">
+      <c r="A168" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B168" t="s">
+      <c r="B168" s="1" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="169" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A169" t="s">
+    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="19.5">
+      <c r="A169" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="B169" t="s">
+      <c r="B169" s="1" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="170" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A170" t="s">
+    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="19.5">
+      <c r="A170" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="B170" t="s">
+      <c r="B170" s="1" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="171" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A171" t="s">
+    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="19.5">
+      <c r="A171" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="B171" t="s">
+      <c r="B171" s="1" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="172" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="19.5">
       <c r="A172" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="20.25">
+      <c r="A173" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="B172" s="2" t="s">
+      <c r="B173" s="3" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="173" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A173" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="B173" s="1" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A174" t="s">
+    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="19.5">
+      <c r="A174" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="B174" t="s">
+      <c r="B174" s="1" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="175" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A175" t="s">
+    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="19.5">
+      <c r="A175" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="B175" t="s">
+      <c r="B175" s="1" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="176" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A176" t="s">
+    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="19.5">
+      <c r="A176" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="B176" t="s">
+      <c r="B176" s="1" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="177" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A177" t="s">
+    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="19.5">
+      <c r="A177" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B177" t="s">
+      <c r="B177" s="1" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="178" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A178" t="s">
+    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="19.5">
+      <c r="A178" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="B178" t="s">
+      <c r="B178" s="1" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="179" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A179" t="s">
+    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="19.5">
+      <c r="A179" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="B179" t="s">
+      <c r="B179" s="1" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="180" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A180" t="s">
+    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="19.5">
+      <c r="A180" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="B180" t="s">
+      <c r="B180" s="1" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="181" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A181" t="s">
+    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="19.5">
+      <c r="A181" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="B181" t="s">
+      <c r="B181" s="1" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="182" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A182" t="s">
+    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="19.5">
+      <c r="A182" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="B182" t="s">
+      <c r="B182" s="1" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="183" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A183" t="s">
+    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="19.5">
+      <c r="A183" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="B183" t="s">
+      <c r="B183" s="1" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="184" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A184" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="20.25">
+      <c r="A184" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="B184" s="1" t="s">
+      <c r="B184" s="3" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="185" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A185" t="s">
+    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="19.5">
+      <c r="A185" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="B185" t="s">
+      <c r="B185" s="1" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="186" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A186" t="s">
+    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="19.5">
+      <c r="A186" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="B186" t="s">
+      <c r="B186" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="187" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A187" t="s">
+    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="19.5">
+      <c r="A187" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="B187" t="s">
+      <c r="B187" s="1" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="188" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A188" t="s">
+    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="19.5">
+      <c r="A188" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="B188" t="s">
+      <c r="B188" s="1" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="189" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A189" t="s">
+    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="19.5">
+      <c r="A189" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="B189" t="s">
+      <c r="B189" s="1" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="190" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A190" t="s">
+    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="19.5">
+      <c r="A190" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="B190" t="s">
+      <c r="B190" s="1" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="191" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A191" t="s">
+    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="19.5">
+      <c r="A191" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="B191" t="s">
+      <c r="B191" s="1" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="192" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A192" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="20.25">
+      <c r="A192" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="B192" s="1" t="s">
+      <c r="B192" s="3" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="193" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A193" t="s">
+    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="19.5">
+      <c r="A193" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="B193" t="s">
+      <c r="B193" s="1" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="194" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A194" t="s">
+    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="19.5">
+      <c r="A194" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="B194" t="s">
+      <c r="B194" s="1" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="195" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A195" t="s">
+    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="19.5">
+      <c r="A195" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="B195" t="s">
+      <c r="B195" s="1" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="196" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A196" t="s">
+    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="19.5">
+      <c r="A196" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="B196" t="s">
+      <c r="B196" s="1" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="197" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A197" t="s">
+    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="19.5">
+      <c r="A197" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="B197" t="s">
+      <c r="B197" s="1" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="198" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A198" t="s">
+    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="19.5">
+      <c r="A198" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="B198" t="s">
+      <c r="B198" s="1" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="199" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A199" t="s">
+    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="19.5">
+      <c r="A199" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="B199" t="s">
+      <c r="B199" s="1" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="200" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A200" t="s">
+    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="19.5">
+      <c r="A200" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="B200" t="s">
+      <c r="B200" s="1" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="201" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A201" t="s">
+    <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="19.5">
+      <c r="A201" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B201" t="s">
+      <c r="B201" s="1" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="202" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A202" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="20.25">
+      <c r="A202" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="B202" s="1" t="s">
+      <c r="B202" s="3" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="203" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A203" t="s">
+    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="19.5">
+      <c r="A203" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="B203" t="s">
+      <c r="B203" s="1" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="204" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A204" t="s">
+    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="19.5">
+      <c r="A204" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="B204" t="s">
+      <c r="B204" s="1" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="205" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A205" t="s">
+    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="19.5">
+      <c r="A205" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="B205" t="s">
+      <c r="B205" s="1" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="206" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A206" t="s">
+    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="19.5">
+      <c r="A206" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="B206" t="s">
+      <c r="B206" s="1" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="207" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A207" t="s">
+    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="19.5">
+      <c r="A207" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="B207" t="s">
+      <c r="B207" s="1" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="208" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A208" t="s">
+    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="19.5">
+      <c r="A208" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="B208" t="s">
+      <c r="B208" s="1" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="209" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A209" t="s">
+    <row x14ac:dyDescent="0.25" r="209" customHeight="1" ht="18.75">
+      <c r="A209" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="B209" t="s">
+      <c r="B209" s="1" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="210" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A210" t="s">
+    <row x14ac:dyDescent="0.25" r="210" customHeight="1" ht="18.75">
+      <c r="A210" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="B210" t="s">
+      <c r="B210" s="1" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="211" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A211" t="s">
+    <row x14ac:dyDescent="0.25" r="211" customHeight="1" ht="18.75">
+      <c r="A211" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="B211" t="s">
+      <c r="B211" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="212" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A212" t="s">
+    <row x14ac:dyDescent="0.25" r="212" customHeight="1" ht="18.75">
+      <c r="A212" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="B212" t="s">
+      <c r="B212" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="213" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A213" t="s">
+    <row x14ac:dyDescent="0.25" r="213" customHeight="1" ht="18.75">
+      <c r="A213" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="B213" t="s">
+      <c r="B213" s="1" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="214" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A214" t="s">
+    <row x14ac:dyDescent="0.25" r="214" customHeight="1" ht="18.75">
+      <c r="A214" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="B214" t="s">
+      <c r="B214" s="1" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="215" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A215" t="s">
+    <row x14ac:dyDescent="0.25" r="215" customHeight="1" ht="18.75">
+      <c r="A215" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="B215" t="s">
+      <c r="B215" s="1" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="216" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A216" t="s">
+    <row x14ac:dyDescent="0.25" r="216" customHeight="1" ht="18.75">
+      <c r="A216" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="B216" t="s">
+      <c r="B216" s="1" t="s">
         <v>415</v>
       </c>
     </row>
-    <row r="217" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A217" t="s">
+    <row x14ac:dyDescent="0.25" r="217" customHeight="1" ht="18.75">
+      <c r="A217" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="B217" t="s">
+      <c r="B217" s="1" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="218" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A218" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="218" customHeight="1" ht="18.75">
+      <c r="A218" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="B218" s="3" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="219" customHeight="1" ht="18.75">
+      <c r="A219" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="B219" s="3" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="220" customHeight="1" ht="18.75">
+      <c r="A220" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="B220" s="1" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="221" customHeight="1" ht="19.5">
+      <c r="A221" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="B221" s="1" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="222" customHeight="1" ht="19.5">
+      <c r="A222" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="B222" s="1" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="223" customHeight="1" ht="19.5">
+      <c r="A223" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="B223" s="1" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="224" customHeight="1" ht="19.5">
+      <c r="A224" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="B224" s="1" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="225" customHeight="1" ht="19.5">
+      <c r="A225" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="B225" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="226" customHeight="1" ht="19.5">
+      <c r="A226" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="B226" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="227" customHeight="1" ht="19.5">
+      <c r="A227" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="B227" s="1" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="228" customHeight="1" ht="19.5">
+      <c r="A228" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="B218" s="1" t="s">
+      <c r="B228" s="1" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="219" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A219" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="229" customHeight="1" ht="19.5">
+      <c r="A229" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="B219" s="1" t="s">
+      <c r="B229" s="1" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="220" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A220" t="s">
+    <row x14ac:dyDescent="0.25" r="230" customHeight="1" ht="19.5">
+      <c r="A230" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="B220" t="s">
+      <c r="B230" s="1" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="221" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A221" t="s">
-        <v>418</v>
-      </c>
-      <c r="B221" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="222" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A222" t="s">
-        <v>420</v>
-      </c>
-      <c r="B222" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="223" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A223" t="s">
-        <v>422</v>
-      </c>
-      <c r="B223" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="224" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A224" t="s">
-        <v>424</v>
-      </c>
-      <c r="B224" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="225" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A225" t="s">
-        <v>426</v>
-      </c>
-      <c r="B225" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="226" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A226" t="s">
-        <v>428</v>
-      </c>
-      <c r="B226" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="227" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A227" t="s">
-        <v>430</v>
-      </c>
-      <c r="B227" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="228" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A228" t="s">
-        <v>432</v>
-      </c>
-      <c r="B228" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="229" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A229" t="s">
-        <v>434</v>
-      </c>
-      <c r="B229" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="230" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A230" t="s">
-        <v>436</v>
-      </c>
-      <c r="B230" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="231" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A231" t="s">
+    <row x14ac:dyDescent="0.25" r="231" customHeight="1" ht="18.75">
+      <c r="A231" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="B231" t="s">
+      <c r="B231" s="1" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="232" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A232" t="s">
+    <row x14ac:dyDescent="0.25" r="232" customHeight="1" ht="18.75">
+      <c r="A232" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="B232" t="s">
+      <c r="B232" s="1" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="233" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A233" t="s">
+    <row x14ac:dyDescent="0.25" r="233" customHeight="1" ht="18.75">
+      <c r="A233" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="B233" t="s">
+      <c r="B233" s="1" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="234" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A234" t="s">
+    <row x14ac:dyDescent="0.25" r="234" customHeight="1" ht="18.75">
+      <c r="A234" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="B234" t="s">
+      <c r="B234" s="1" t="s">
         <v>451</v>
       </c>
     </row>
-    <row r="235" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A235" t="s">
+    <row x14ac:dyDescent="0.25" r="235" customHeight="1" ht="18.75">
+      <c r="A235" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="B235" t="s">
+      <c r="B235" s="1" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="236" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A236" t="s">
+    <row x14ac:dyDescent="0.25" r="236" customHeight="1" ht="18.75">
+      <c r="A236" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="B236" t="s">
+      <c r="B236" s="1" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="237" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A237" t="s">
+    <row x14ac:dyDescent="0.25" r="237" customHeight="1" ht="18.75">
+      <c r="A237" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="B237" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="238" customHeight="1" ht="18.75">
+      <c r="A238" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B238" s="1" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="239" customHeight="1" ht="18.75">
+      <c r="A239" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B239" s="1" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="240" customHeight="1" ht="18.75">
+      <c r="A240" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="B240" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="241" customHeight="1" ht="18.75">
+      <c r="A241" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="B241" s="1" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="242" customHeight="1" ht="18.75">
+      <c r="A242" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="B242" s="1" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="243" customHeight="1" ht="18.75">
+      <c r="A243" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B243" s="1" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="244" customHeight="1" ht="18.75">
+      <c r="A244" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="245" customHeight="1" ht="18.75">
+      <c r="A245" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="B245" s="1" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="246" customHeight="1" ht="18.75">
+      <c r="A246" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="B246" s="1" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="247" customHeight="1" ht="18.75">
+      <c r="A247" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="B247" s="1" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="248" customHeight="1" ht="18.75">
+      <c r="A248" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="B248" s="1" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="249" customHeight="1" ht="18.75">
+      <c r="A249" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="B249" s="1" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="250" customHeight="1" ht="18.75">
+      <c r="A250" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="B250" s="1" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="251" customHeight="1" ht="18.75">
+      <c r="A251" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B251" s="1" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="252" customHeight="1" ht="18.75">
+      <c r="A252" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="B252" s="1" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="253" customHeight="1" ht="18.75">
+      <c r="A253" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B253" s="1" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="254" customHeight="1" ht="18.75">
+      <c r="A254" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="B254" s="1" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="255" customHeight="1" ht="18.75">
+      <c r="A255" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="B255" s="1" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="256" customHeight="1" ht="18.75">
+      <c r="A256" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="B256" s="1" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="257" customHeight="1" ht="18.75">
+      <c r="A257" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B257" s="1" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="258" customHeight="1" ht="18.75">
+      <c r="A258" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="B258" s="1" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="259" customHeight="1" ht="18.75">
+      <c r="A259" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="B259" s="1" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="260" customHeight="1" ht="18.75">
+      <c r="A260" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="B260" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="18.75">
+      <c r="A261" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="B261" s="3" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="18.75">
+      <c r="A262" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="B262" s="1" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="263" customHeight="1" ht="18.75">
+      <c r="A263" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="B263" s="3" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="264" customHeight="1" ht="18.75">
+      <c r="A264" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B264" s="3" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="265" customHeight="1" ht="18.75">
+      <c r="A265" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="B265" s="3" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="266" customHeight="1" ht="18.75">
+      <c r="A266" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="B266" s="1" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="267" customHeight="1" ht="18.75">
+      <c r="A267" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="B267" s="1" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="268" customHeight="1" ht="18.75">
+      <c r="A268" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="B268" s="1" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="269" customHeight="1" ht="18.75">
+      <c r="A269" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="B269" s="1" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="270" customHeight="1" ht="18.75">
+      <c r="A270" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="B270" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="271" customHeight="1" ht="18.75">
+      <c r="A271" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="B271" s="1" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="18.75">
+      <c r="A272" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="B272" s="1" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="273" customHeight="1" ht="18.75">
+      <c r="A273" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="B273" s="3" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="18.75">
+      <c r="A274" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="B274" s="1" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="275" customHeight="1" ht="18.75">
+      <c r="A275" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="B275" s="1" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="276" customHeight="1" ht="18.75">
+      <c r="A276" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="B276" s="1" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="277" customHeight="1" ht="18.75">
+      <c r="A277" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="B277" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="18.75">
+      <c r="A278" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="B278" s="1" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="279" customHeight="1" ht="18.75">
+      <c r="A279" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="B279" s="1" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="280" customHeight="1" ht="18.75">
+      <c r="A280" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="B280" s="1" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="281" customHeight="1" ht="18.75">
+      <c r="A281" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="B281" s="1" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="282" customHeight="1" ht="18.75">
+      <c r="A282" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="B282" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="283" customHeight="1" ht="18.75">
+      <c r="A283" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="B283" s="1" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="284" customHeight="1" ht="18.75">
+      <c r="A284" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="B284" s="1" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="285" customHeight="1" ht="18.75">
+      <c r="A285" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="B285" s="1" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="286" customHeight="1" ht="18.75">
+      <c r="A286" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="B286" s="1" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="287" customHeight="1" ht="18.75">
+      <c r="A287" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="B287" s="1" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="288" customHeight="1" ht="18.75">
+      <c r="A288" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="B288" s="1" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="289" customHeight="1" ht="18.75">
+      <c r="A289" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="B289" s="3" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="290" customHeight="1" ht="18.75">
+      <c r="A290" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="291" customHeight="1" ht="18.75">
+      <c r="A291" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="B291" s="1" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="292" customHeight="1" ht="18.75">
+      <c r="A292" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="B292" s="1" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="293" customHeight="1" ht="18.75">
+      <c r="A293" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="B293" s="3" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="294" customHeight="1" ht="18.75">
+      <c r="A294" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="B294" s="1" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="295" customHeight="1" ht="18.75">
+      <c r="A295" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="B295" s="1" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="296" customHeight="1" ht="18.75">
+      <c r="A296" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="B296" s="1" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="297" customHeight="1" ht="18.75">
+      <c r="A297" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="B297" s="1" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="298" customHeight="1" ht="18.75">
+      <c r="A298" s="1" t="s">
         <v>575</v>
       </c>
-      <c r="B237" t="s">
+      <c r="B298" s="1" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="238" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A238" t="s">
+    <row x14ac:dyDescent="0.25" r="299" customHeight="1" ht="18.75">
+      <c r="A299" s="1" t="s">
         <v>577</v>
       </c>
-      <c r="B238" t="s">
+      <c r="B299" s="1" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="239" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A239" t="s">
+    <row x14ac:dyDescent="0.25" r="300" customHeight="1" ht="18.75">
+      <c r="A300" s="1" t="s">
         <v>579</v>
       </c>
-      <c r="B239" t="s">
+      <c r="B300" s="1" t="s">
         <v>580</v>
       </c>
     </row>
-    <row r="240" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A240" t="s">
-        <v>456</v>
-      </c>
-      <c r="B240" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="241" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A241" t="s">
-        <v>458</v>
-      </c>
-      <c r="B241" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="242" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A242" t="s">
-        <v>460</v>
-      </c>
-      <c r="B242" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="243" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A243" t="s">
-        <v>462</v>
-      </c>
-      <c r="B243" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="244" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A244" t="s">
-        <v>464</v>
-      </c>
-      <c r="B244" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="245" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A245" t="s">
-        <v>466</v>
-      </c>
-      <c r="B245" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="246" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A246" t="s">
-        <v>468</v>
-      </c>
-      <c r="B246" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="247" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A247" t="s">
-        <v>470</v>
-      </c>
-      <c r="B247" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="248" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A248" t="s">
-        <v>472</v>
-      </c>
-      <c r="B248" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="249" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A249" t="s">
-        <v>474</v>
-      </c>
-      <c r="B249" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="250" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A250" t="s">
-        <v>476</v>
-      </c>
-      <c r="B250" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="251" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A251" t="s">
-        <v>478</v>
-      </c>
-      <c r="B251" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="252" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A252" t="s">
-        <v>480</v>
-      </c>
-      <c r="B252" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="253" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A253" t="s">
-        <v>482</v>
-      </c>
-      <c r="B253" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="254" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A254" t="s">
-        <v>484</v>
-      </c>
-      <c r="B254" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="255" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A255" t="s">
-        <v>486</v>
-      </c>
-      <c r="B255" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="256" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A256" t="s">
-        <v>488</v>
-      </c>
-      <c r="B256" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="257" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A257" t="s">
-        <v>490</v>
-      </c>
-      <c r="B257" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="258" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A258" t="s">
-        <v>492</v>
-      </c>
-      <c r="B258" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="259" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A259" s="1" t="s">
-        <v>493</v>
-      </c>
-      <c r="B259" s="1" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="260" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A260" t="s">
-        <v>495</v>
-      </c>
-      <c r="B260" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="261" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A261" s="1" t="s">
-        <v>497</v>
-      </c>
-      <c r="B261" s="1" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="262" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A262" s="1" t="s">
-        <v>499</v>
-      </c>
-      <c r="B262" s="1" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="263" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A263" s="1" t="s">
-        <v>501</v>
-      </c>
-      <c r="B263" s="1" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="264" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A264" t="s">
-        <v>503</v>
-      </c>
-      <c r="B264" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="265" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A265" t="s">
-        <v>505</v>
-      </c>
-      <c r="B265" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="266" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A266" t="s">
-        <v>507</v>
-      </c>
-      <c r="B266" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="267" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A267" t="s">
-        <v>509</v>
-      </c>
-      <c r="B267" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="268" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A268" t="s">
-        <v>511</v>
-      </c>
-      <c r="B268" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="269" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A269" t="s">
-        <v>512</v>
-      </c>
-      <c r="B269" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="270" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A270" t="s">
-        <v>514</v>
-      </c>
-      <c r="B270" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="271" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A271" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="B271" s="1" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="272" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A272" t="s">
-        <v>518</v>
-      </c>
-      <c r="B272" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="273" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A273" t="s">
-        <v>520</v>
-      </c>
-      <c r="B273" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="274" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A274" t="s">
-        <v>522</v>
-      </c>
-      <c r="B274" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="275" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A275" t="s">
-        <v>523</v>
-      </c>
-      <c r="B275" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="276" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A276" t="s">
-        <v>525</v>
-      </c>
-      <c r="B276" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="277" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A277" t="s">
-        <v>527</v>
-      </c>
-      <c r="B277" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="278" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A278" t="s">
-        <v>529</v>
-      </c>
-      <c r="B278" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="279" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A279" t="s">
-        <v>531</v>
-      </c>
-      <c r="B279" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="280" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A280" t="s">
-        <v>533</v>
-      </c>
-      <c r="B280" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="281" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A281" t="s">
-        <v>535</v>
-      </c>
-      <c r="B281" t="s">
-        <v>536</v>
-      </c>
-    </row>
-    <row r="282" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A282" t="s">
-        <v>537</v>
-      </c>
-      <c r="B282" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="283" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A283" t="s">
-        <v>539</v>
-      </c>
-      <c r="B283" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A284" t="s">
-        <v>541</v>
-      </c>
-      <c r="B284" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="285" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A285" t="s">
-        <v>543</v>
-      </c>
-      <c r="B285" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="286" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A286" t="s">
-        <v>545</v>
-      </c>
-      <c r="B286" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A287" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="B287" s="1" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="288" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A288" t="s">
-        <v>549</v>
-      </c>
-      <c r="B288" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="289" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A289" t="s">
-        <v>551</v>
-      </c>
-      <c r="B289" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A290" t="s">
-        <v>553</v>
-      </c>
-      <c r="B290" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="291" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A291" s="1" t="s">
-        <v>555</v>
-      </c>
-      <c r="B291" s="1" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="292" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A292" t="s">
-        <v>557</v>
-      </c>
-      <c r="B292" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="293" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A293" t="s">
-        <v>559</v>
-      </c>
-      <c r="B293" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="294" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A294" t="s">
-        <v>561</v>
-      </c>
-      <c r="B294" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="295" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A295" t="s">
-        <v>563</v>
-      </c>
-      <c r="B295" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="296" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A296" t="s">
-        <v>565</v>
-      </c>
-      <c r="B296" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="297" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A297" t="s">
-        <v>567</v>
-      </c>
-      <c r="B297" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="298" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A298" t="s">
-        <v>569</v>
-      </c>
-      <c r="B298" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="299" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A299" t="s">
-        <v>571</v>
-      </c>
-      <c r="B299" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="300" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A300" t="s">
-        <v>573</v>
-      </c>
-      <c r="B300" t="s">
-        <v>574</v>
+    <row x14ac:dyDescent="0.25" r="301" customHeight="1" ht="18.75">
+      <c r="A301" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="B301" s="1" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="302" customHeight="1" ht="18.75">
+      <c r="A302" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="B302" s="1" t="s">
+        <v>584</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MAUI-5787 Update datasets to exclude encounters from sensitive facilities (#253)
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -1,29 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia\Documents\GitHub\tamanu-source-dbt\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74409AB8-E8B9-4DE4-AACE-7B87B9E1ADBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14390" yWindow="-10" windowWidth="14420" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Translated String" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Translated String"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Translated String'!$A$1:$B$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="585">
   <si>
     <t>stringId</t>
   </si>
@@ -1009,18 +1003,18 @@
     <t>Edited by user</t>
   </si>
   <si>
+    <t>report.reporting.logChangeDateTime</t>
+  </si>
+  <si>
+    <t>Date and time edited</t>
+  </si>
+  <si>
     <t>report.reporting.logChangeRecordCreatedDateTime</t>
   </si>
   <si>
     <t>Date and time created</t>
   </si>
   <si>
-    <t>report.reporting.logChangeDateTime</t>
-  </si>
-  <si>
-    <t>Date and time edited</t>
-  </si>
-  <si>
     <t>report.reporting.medications</t>
   </si>
   <si>
@@ -1279,6 +1273,24 @@
     <t>Social security number</t>
   </si>
   <si>
+    <t>report.reporting.patientStreetVillage</t>
+  </si>
+  <si>
+    <t>Street / Village</t>
+  </si>
+  <si>
+    <t>report.reporting.patientSubDivision</t>
+  </si>
+  <si>
+    <t>Sub-division</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTitle</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
     <t>report.reporting.patientTotal</t>
   </si>
   <si>
@@ -1339,24 +1351,6 @@
     <t>Total patients with missing location</t>
   </si>
   <si>
-    <t>report.reporting.patientStreetVillage</t>
-  </si>
-  <si>
-    <t>Street / Village</t>
-  </si>
-  <si>
-    <t>report.reporting.patientSubDivision</t>
-  </si>
-  <si>
-    <t>Sub-division</t>
-  </si>
-  <si>
-    <t>report.reporting.patientTitle</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
     <t>report.reporting.patientVillage</t>
   </si>
   <si>
@@ -1393,6 +1387,36 @@
     <t>Tamanu user name</t>
   </si>
   <si>
+    <t>report.reporting.prescriptionDate</t>
+  </si>
+  <si>
+    <t>Prescription date</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedication</t>
+  </si>
+  <si>
+    <t>Medication</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedicationCode</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionQuantity</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionSelectedForDischarge</t>
+  </si>
+  <si>
+    <t>Prescription selected for discharge</t>
+  </si>
+  <si>
     <t>report.reporting.procedure</t>
   </si>
   <si>
@@ -1748,37 +1772,26 @@
   </si>
   <si>
     <t>Schedule</t>
-  </si>
-  <si>
-    <t>report.reporting.prescriptionMedication</t>
-  </si>
-  <si>
-    <t>Medication</t>
-  </si>
-  <si>
-    <t>report.reporting.prescriptionMedicationCode</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>report.reporting.prescriptionQuantity</t>
-  </si>
-  <si>
-    <t>Quantity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1814,24 +1827,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="5">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1842,10 +1860,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -1883,71 +1901,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1975,7 +1993,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1998,11 +2016,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -2011,13 +2029,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -2027,7 +2045,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -2036,7 +2054,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -2045,7 +2063,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -2053,10 +2071,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -2121,2415 +2139,2431 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B300"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:B302"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="64.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="4" width="64.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="35.71928571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+      <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+      <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+      <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+      <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+      <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+      <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+      <c r="A22" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+      <c r="A23" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+      <c r="A24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+      <c r="A25" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+      <c r="A26" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" t="s">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+      <c r="A27" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A28" t="s">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+      <c r="A28" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" t="s">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+      <c r="A29" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" t="s">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+      <c r="A30" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" t="s">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+      <c r="A31" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
+      <c r="A32" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" t="s">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
+      <c r="A33" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" t="s">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
+      <c r="A34" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
+      <c r="A35" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" t="s">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
+      <c r="A36" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" t="s">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
+      <c r="A37" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A38" t="s">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
+      <c r="A38" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A39" t="s">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
+      <c r="A39" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" t="s">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
+      <c r="A40" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" t="s">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
+      <c r="A41" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A42" t="s">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
+      <c r="A42" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A43" t="s">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
+      <c r="A43" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A44" t="s">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
+      <c r="A44" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A45" t="s">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
+      <c r="A45" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A46" t="s">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
+      <c r="A46" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A47" t="s">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
+      <c r="A47" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A48" t="s">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
+      <c r="A48" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A49" t="s">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
+      <c r="A49" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A50" t="s">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
+      <c r="A50" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A51" t="s">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
+      <c r="A51" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A52" t="s">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
+      <c r="A52" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A53" t="s">
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
+      <c r="A53" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A54" t="s">
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
+      <c r="A54" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A55" t="s">
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
+      <c r="A55" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A56" t="s">
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
+      <c r="A56" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A57" t="s">
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
+      <c r="A57" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="1" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A58" t="s">
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
+      <c r="A58" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A59" t="s">
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
+      <c r="A59" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A60" t="s">
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
+      <c r="A60" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A61" t="s">
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
+      <c r="A61" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B61" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A62" t="s">
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
+      <c r="A62" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B62" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A63" t="s">
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
+      <c r="A63" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B63" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A64" t="s">
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
+      <c r="A64" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B64" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A65" t="s">
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
+      <c r="A65" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A66" t="s">
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
+      <c r="A66" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A67" t="s">
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
+      <c r="A67" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B67" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A68" t="s">
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
+      <c r="A68" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A69" t="s">
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
+      <c r="A69" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A70" t="s">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
+      <c r="A70" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B70" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A71" t="s">
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
+      <c r="A71" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A72" t="s">
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
+      <c r="A72" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A73" t="s">
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
+      <c r="A73" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A74" t="s">
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
+      <c r="A74" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B74" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A75" t="s">
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
+      <c r="A75" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B75" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A76" t="s">
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
+      <c r="A76" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B76" s="1" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A77" t="s">
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
+      <c r="A77" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B77" s="1" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A78" t="s">
+    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
+      <c r="A78" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B78" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A79" t="s">
+    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
+      <c r="A79" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B79" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A80" t="s">
+    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
+      <c r="A80" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B80" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="81" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A81" t="s">
+    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
+      <c r="A81" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B81" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="82" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A82" t="s">
+    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
+      <c r="A82" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B82" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="83" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A83" t="s">
+    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
+      <c r="A83" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B83" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="84" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A84" t="s">
+    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
+      <c r="A84" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B84" s="1" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="85" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A85" t="s">
+    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
+      <c r="A85" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B85" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="86" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A86" t="s">
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
+      <c r="A86" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B86" s="1" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="87" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A87" t="s">
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
+      <c r="A87" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B87" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="88" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A88" t="s">
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
+      <c r="A88" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B88" s="1" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="89" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A89" t="s">
+    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
+      <c r="A89" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B89" s="1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="90" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A90" t="s">
+    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
+      <c r="A90" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="91" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A91" t="s">
+    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
+      <c r="A91" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B91" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="92" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A92" t="s">
+    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
+      <c r="A92" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B92" s="1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="93" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A93" t="s">
+    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
+      <c r="A93" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B93" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="94" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A94" t="s">
+    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
+      <c r="A94" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B94" s="1" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="95" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A95" t="s">
+    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
+      <c r="A95" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B95" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="96" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A96" t="s">
+    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
+      <c r="A96" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B96" s="1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="97" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A97" t="s">
+    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
+      <c r="A97" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B97" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="98" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A98" t="s">
+    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
+      <c r="A98" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B98" s="1" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="99" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A99" t="s">
+    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
+      <c r="A99" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B99" s="1" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="100" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A100" t="s">
+    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
+      <c r="A100" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B100" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="101" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A101" t="s">
+    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
+      <c r="A101" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B101" s="1" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="102" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A102" t="s">
+    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
+      <c r="A102" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B102" s="1" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="103" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A103" t="s">
+    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
+      <c r="A103" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="B103" t="s">
+      <c r="B103" s="1" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="104" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A104" t="s">
+    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
+      <c r="A104" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B104" s="1" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="105" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A105" t="s">
+    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
+      <c r="A105" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B105" s="1" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="106" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A106" t="s">
+    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
+      <c r="A106" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B106" s="1" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="107" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A107" t="s">
+    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
+      <c r="A107" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B107" s="1" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="108" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A108" t="s">
+    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75">
+      <c r="A108" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B108" s="1" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="109" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A109" t="s">
+    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75">
+      <c r="A109" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B109" s="1" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="110" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A110" t="s">
+    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
+      <c r="A110" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B110" s="1" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="111" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A111" t="s">
+    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
+      <c r="A111" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B111" s="1" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="112" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A112" t="s">
+    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
+      <c r="A112" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="B112" t="s">
+      <c r="B112" s="1" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="113" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A113" t="s">
+    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
+      <c r="A113" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="B113" t="s">
+      <c r="B113" s="1" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="114" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A114" t="s">
+    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
+      <c r="A114" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="B114" t="s">
+      <c r="B114" s="1" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="115" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A115" t="s">
+    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
+      <c r="A115" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B115" s="1" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="116" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A116" t="s">
+    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
+      <c r="A116" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B116" s="1" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="117" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A117" t="s">
+    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
+      <c r="A117" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B117" t="s">
+      <c r="B117" s="1" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="118" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A118" t="s">
+    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
+      <c r="A118" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="B118" t="s">
+      <c r="B118" s="1" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="119" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A119" t="s">
+    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
+      <c r="A119" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="B119" t="s">
+      <c r="B119" s="1" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="120" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A120" t="s">
+    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
+      <c r="A120" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="B120" t="s">
+      <c r="B120" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="121" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A121" t="s">
+    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
+      <c r="A121" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B121" s="1" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="122" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A122" t="s">
+    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
+      <c r="A122" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="B122" t="s">
+      <c r="B122" s="1" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="123" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A123" t="s">
+    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
+      <c r="A123" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="B123" t="s">
+      <c r="B123" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="124" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A124" t="s">
+    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
+      <c r="A124" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B124" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="125" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A125" t="s">
+    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
+      <c r="A125" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="B125" t="s">
+      <c r="B125" s="1" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="126" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A126" t="s">
+    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
+      <c r="A126" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="B126" t="s">
+      <c r="B126" s="1" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="127" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A127" t="s">
+    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
+      <c r="A127" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B127" t="s">
+      <c r="B127" s="1" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="128" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A128" t="s">
+    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
+      <c r="A128" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="B128" t="s">
+      <c r="B128" s="1" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="129" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A129" t="s">
+    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
+      <c r="A129" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="B129" t="s">
+      <c r="B129" s="1" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="130" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A130" t="s">
+    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75">
+      <c r="A130" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B130" s="1" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="131" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A131" t="s">
+    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18.75">
+      <c r="A131" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="B131" t="s">
+      <c r="B131" s="1" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="132" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A132" t="s">
+    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18.75">
+      <c r="A132" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="B132" t="s">
+      <c r="B132" s="1" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="133" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A133" t="s">
+    <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="18.75">
+      <c r="A133" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B133" s="1" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="134" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A134" t="s">
+    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18.75">
+      <c r="A134" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="B134" t="s">
+      <c r="B134" s="1" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="135" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A135" t="s">
+    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18.75">
+      <c r="A135" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B135" s="1" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="136" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A136" t="s">
+    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18.75">
+      <c r="A136" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="B136" t="s">
+      <c r="B136" s="1" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="137" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A137" t="s">
+    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18.75">
+      <c r="A137" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="B137" t="s">
+      <c r="B137" s="1" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="138" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A138" t="s">
+    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18.75">
+      <c r="A138" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B138" s="1" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="139" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A139" t="s">
+    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18.75">
+      <c r="A139" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B139" t="s">
+      <c r="B139" s="1" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="140" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A140" t="s">
+    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18.75">
+      <c r="A140" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="B140" t="s">
+      <c r="B140" s="1" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="141" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A141" t="s">
+    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18.75">
+      <c r="A141" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B141" t="s">
+      <c r="B141" s="1" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="142" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A142" t="s">
+    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18.75">
+      <c r="A142" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="B142" t="s">
+      <c r="B142" s="1" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="143" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A143" t="s">
+    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18.75">
+      <c r="A143" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="B143" t="s">
+      <c r="B143" s="1" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="144" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A144" t="s">
+    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="18.75">
+      <c r="A144" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="B144" t="s">
+      <c r="B144" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="145" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A145" t="s">
+    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="18.75">
+      <c r="A145" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="B145" t="s">
+      <c r="B145" s="1" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="146" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A146" t="s">
+    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="18.75">
+      <c r="A146" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="B146" t="s">
+      <c r="B146" s="1" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="147" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A147" t="s">
+    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="18.75">
+      <c r="A147" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="B147" t="s">
+      <c r="B147" s="1" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="148" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A148" t="s">
+    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="18.75">
+      <c r="A148" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="B148" t="s">
+      <c r="B148" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="149" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A149" t="s">
+    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="18.75">
+      <c r="A149" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="B149" t="s">
+      <c r="B149" s="1" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="150" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A150" t="s">
+    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18.75">
+      <c r="A150" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="B150" t="s">
+      <c r="B150" s="1" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="151" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A151" t="s">
+    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18.75">
+      <c r="A151" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="B151" t="s">
+      <c r="B151" s="1" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="152" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A152" t="s">
+    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18.75">
+      <c r="A152" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="B152" t="s">
+      <c r="B152" s="1" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="153" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A153" t="s">
+    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="18.75">
+      <c r="A153" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="B153" t="s">
+      <c r="B153" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="154" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A154" t="s">
+    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18.75">
+      <c r="A154" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="B154" t="s">
+      <c r="B154" s="1" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="155" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A155" t="s">
+    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18.75">
+      <c r="A155" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="B155" t="s">
+      <c r="B155" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="156" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A156" t="s">
+    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18.75">
+      <c r="A156" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="B156" t="s">
+      <c r="B156" s="1" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="157" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A157" t="s">
+    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18.75">
+      <c r="A157" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="B157" t="s">
+      <c r="B157" s="1" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="158" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A158" t="s">
+    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18.75">
+      <c r="A158" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="B158" t="s">
+      <c r="B158" s="1" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="159" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A159" t="s">
+    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18.75">
+      <c r="A159" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="B159" t="s">
+      <c r="B159" s="1" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="160" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A160" t="s">
+    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18.75">
+      <c r="A160" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="B160" t="s">
+      <c r="B160" s="1" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="161" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A161" t="s">
+    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18.75">
+      <c r="A161" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="B161" t="s">
+      <c r="B161" s="1" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="162" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A162" t="s">
+    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18.75">
+      <c r="A162" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="B162" t="s">
+      <c r="B162" s="1" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="163" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A163" t="s">
+    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75">
+      <c r="A163" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="B163" t="s">
+      <c r="B163" s="1" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="164" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A164" t="s">
+    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75">
+      <c r="A164" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="B164" t="s">
+      <c r="B164" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="165" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A165" t="s">
+    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75">
+      <c r="A165" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B165" t="s">
+      <c r="B165" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="166" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A166" t="s">
+    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75">
+      <c r="A166" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="B166" t="s">
+      <c r="B166" s="1" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="167" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A167" t="s">
+    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75">
+      <c r="A167" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="B167" t="s">
+      <c r="B167" s="1" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="168" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A168" t="s">
+    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="19.5">
+      <c r="A168" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B168" t="s">
+      <c r="B168" s="1" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="169" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A169" t="s">
+    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="19.5">
+      <c r="A169" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="B169" t="s">
+      <c r="B169" s="1" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="170" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A170" t="s">
+    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="19.5">
+      <c r="A170" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="B170" t="s">
+      <c r="B170" s="1" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="171" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A171" t="s">
+    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="19.5">
+      <c r="A171" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="B171" t="s">
+      <c r="B171" s="1" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="172" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="19.5">
       <c r="A172" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="20.25">
+      <c r="A173" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="B172" s="2" t="s">
+      <c r="B173" s="3" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="173" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A173" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="B173" s="1" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A174" t="s">
+    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="19.5">
+      <c r="A174" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="B174" t="s">
+      <c r="B174" s="1" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="175" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A175" t="s">
+    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="19.5">
+      <c r="A175" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="B175" t="s">
+      <c r="B175" s="1" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="176" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A176" t="s">
+    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="19.5">
+      <c r="A176" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="B176" t="s">
+      <c r="B176" s="1" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="177" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A177" t="s">
+    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="19.5">
+      <c r="A177" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B177" t="s">
+      <c r="B177" s="1" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="178" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A178" t="s">
+    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="19.5">
+      <c r="A178" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="B178" t="s">
+      <c r="B178" s="1" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="179" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A179" t="s">
+    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="19.5">
+      <c r="A179" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="B179" t="s">
+      <c r="B179" s="1" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="180" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A180" t="s">
+    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="19.5">
+      <c r="A180" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="B180" t="s">
+      <c r="B180" s="1" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="181" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A181" t="s">
+    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="19.5">
+      <c r="A181" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="B181" t="s">
+      <c r="B181" s="1" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="182" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A182" t="s">
+    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="19.5">
+      <c r="A182" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="B182" t="s">
+      <c r="B182" s="1" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="183" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A183" t="s">
+    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="19.5">
+      <c r="A183" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="B183" t="s">
+      <c r="B183" s="1" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="184" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A184" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="20.25">
+      <c r="A184" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="B184" s="1" t="s">
+      <c r="B184" s="3" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="185" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A185" t="s">
+    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="19.5">
+      <c r="A185" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="B185" t="s">
+      <c r="B185" s="1" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="186" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A186" t="s">
+    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="19.5">
+      <c r="A186" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="B186" t="s">
+      <c r="B186" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="187" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A187" t="s">
+    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="19.5">
+      <c r="A187" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="B187" t="s">
+      <c r="B187" s="1" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="188" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A188" t="s">
+    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="19.5">
+      <c r="A188" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="B188" t="s">
+      <c r="B188" s="1" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="189" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A189" t="s">
+    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="19.5">
+      <c r="A189" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="B189" t="s">
+      <c r="B189" s="1" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="190" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A190" t="s">
+    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="19.5">
+      <c r="A190" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="B190" t="s">
+      <c r="B190" s="1" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="191" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A191" t="s">
+    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="19.5">
+      <c r="A191" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="B191" t="s">
+      <c r="B191" s="1" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="192" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A192" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="20.25">
+      <c r="A192" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="B192" s="1" t="s">
+      <c r="B192" s="3" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="193" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A193" t="s">
+    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="19.5">
+      <c r="A193" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="B193" t="s">
+      <c r="B193" s="1" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="194" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A194" t="s">
+    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="19.5">
+      <c r="A194" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="B194" t="s">
+      <c r="B194" s="1" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="195" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A195" t="s">
+    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="19.5">
+      <c r="A195" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="B195" t="s">
+      <c r="B195" s="1" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="196" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A196" t="s">
+    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="19.5">
+      <c r="A196" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="B196" t="s">
+      <c r="B196" s="1" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="197" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A197" t="s">
+    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="19.5">
+      <c r="A197" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="B197" t="s">
+      <c r="B197" s="1" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="198" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A198" t="s">
+    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="19.5">
+      <c r="A198" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="B198" t="s">
+      <c r="B198" s="1" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="199" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A199" t="s">
+    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="19.5">
+      <c r="A199" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="B199" t="s">
+      <c r="B199" s="1" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="200" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A200" t="s">
+    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="19.5">
+      <c r="A200" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="B200" t="s">
+      <c r="B200" s="1" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="201" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A201" t="s">
+    <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="19.5">
+      <c r="A201" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B201" t="s">
+      <c r="B201" s="1" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="202" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A202" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="20.25">
+      <c r="A202" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="B202" s="1" t="s">
+      <c r="B202" s="3" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="203" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A203" t="s">
+    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="19.5">
+      <c r="A203" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="B203" t="s">
+      <c r="B203" s="1" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="204" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A204" t="s">
+    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="19.5">
+      <c r="A204" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="B204" t="s">
+      <c r="B204" s="1" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="205" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A205" t="s">
+    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="19.5">
+      <c r="A205" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="B205" t="s">
+      <c r="B205" s="1" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="206" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A206" t="s">
+    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="19.5">
+      <c r="A206" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="B206" t="s">
+      <c r="B206" s="1" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="207" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A207" t="s">
+    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="19.5">
+      <c r="A207" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="B207" t="s">
+      <c r="B207" s="1" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="208" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A208" t="s">
+    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="19.5">
+      <c r="A208" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="B208" t="s">
+      <c r="B208" s="1" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="209" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A209" t="s">
+    <row x14ac:dyDescent="0.25" r="209" customHeight="1" ht="18.75">
+      <c r="A209" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="B209" t="s">
+      <c r="B209" s="1" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="210" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A210" t="s">
+    <row x14ac:dyDescent="0.25" r="210" customHeight="1" ht="18.75">
+      <c r="A210" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="B210" t="s">
+      <c r="B210" s="1" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="211" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A211" t="s">
+    <row x14ac:dyDescent="0.25" r="211" customHeight="1" ht="18.75">
+      <c r="A211" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="B211" t="s">
+      <c r="B211" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="212" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A212" t="s">
+    <row x14ac:dyDescent="0.25" r="212" customHeight="1" ht="18.75">
+      <c r="A212" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="B212" t="s">
+      <c r="B212" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="213" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A213" t="s">
+    <row x14ac:dyDescent="0.25" r="213" customHeight="1" ht="18.75">
+      <c r="A213" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="B213" t="s">
+      <c r="B213" s="1" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="214" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A214" t="s">
+    <row x14ac:dyDescent="0.25" r="214" customHeight="1" ht="18.75">
+      <c r="A214" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="B214" t="s">
+      <c r="B214" s="1" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="215" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A215" t="s">
+    <row x14ac:dyDescent="0.25" r="215" customHeight="1" ht="18.75">
+      <c r="A215" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="B215" t="s">
+      <c r="B215" s="1" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="216" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A216" t="s">
+    <row x14ac:dyDescent="0.25" r="216" customHeight="1" ht="18.75">
+      <c r="A216" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="B216" t="s">
+      <c r="B216" s="1" t="s">
         <v>415</v>
       </c>
     </row>
-    <row r="217" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A217" t="s">
+    <row x14ac:dyDescent="0.25" r="217" customHeight="1" ht="18.75">
+      <c r="A217" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="B217" t="s">
+      <c r="B217" s="1" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="218" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A218" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="218" customHeight="1" ht="18.75">
+      <c r="A218" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="B218" s="3" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="219" customHeight="1" ht="18.75">
+      <c r="A219" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="B219" s="3" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="220" customHeight="1" ht="18.75">
+      <c r="A220" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="B220" s="1" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="221" customHeight="1" ht="19.5">
+      <c r="A221" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="B221" s="1" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="222" customHeight="1" ht="19.5">
+      <c r="A222" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="B222" s="1" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="223" customHeight="1" ht="19.5">
+      <c r="A223" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="B223" s="1" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="224" customHeight="1" ht="19.5">
+      <c r="A224" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="B224" s="1" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="225" customHeight="1" ht="19.5">
+      <c r="A225" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="B225" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="226" customHeight="1" ht="19.5">
+      <c r="A226" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="B226" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="227" customHeight="1" ht="19.5">
+      <c r="A227" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="B227" s="1" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="228" customHeight="1" ht="19.5">
+      <c r="A228" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="B218" s="1" t="s">
+      <c r="B228" s="1" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="219" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A219" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="229" customHeight="1" ht="19.5">
+      <c r="A229" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="B219" s="1" t="s">
+      <c r="B229" s="1" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="220" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A220" t="s">
+    <row x14ac:dyDescent="0.25" r="230" customHeight="1" ht="19.5">
+      <c r="A230" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="B220" t="s">
+      <c r="B230" s="1" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="221" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A221" t="s">
-        <v>418</v>
-      </c>
-      <c r="B221" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="222" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A222" t="s">
-        <v>420</v>
-      </c>
-      <c r="B222" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="223" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A223" t="s">
-        <v>422</v>
-      </c>
-      <c r="B223" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="224" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A224" t="s">
-        <v>424</v>
-      </c>
-      <c r="B224" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="225" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A225" t="s">
-        <v>426</v>
-      </c>
-      <c r="B225" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="226" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A226" t="s">
-        <v>428</v>
-      </c>
-      <c r="B226" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="227" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A227" t="s">
-        <v>430</v>
-      </c>
-      <c r="B227" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="228" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A228" t="s">
-        <v>432</v>
-      </c>
-      <c r="B228" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="229" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A229" t="s">
-        <v>434</v>
-      </c>
-      <c r="B229" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="230" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A230" t="s">
-        <v>436</v>
-      </c>
-      <c r="B230" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="231" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A231" t="s">
+    <row x14ac:dyDescent="0.25" r="231" customHeight="1" ht="18.75">
+      <c r="A231" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="B231" t="s">
+      <c r="B231" s="1" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="232" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A232" t="s">
+    <row x14ac:dyDescent="0.25" r="232" customHeight="1" ht="18.75">
+      <c r="A232" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="B232" t="s">
+      <c r="B232" s="1" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="233" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A233" t="s">
+    <row x14ac:dyDescent="0.25" r="233" customHeight="1" ht="18.75">
+      <c r="A233" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="B233" t="s">
+      <c r="B233" s="1" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="234" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A234" t="s">
+    <row x14ac:dyDescent="0.25" r="234" customHeight="1" ht="18.75">
+      <c r="A234" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="B234" t="s">
+      <c r="B234" s="1" t="s">
         <v>451</v>
       </c>
     </row>
-    <row r="235" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A235" t="s">
+    <row x14ac:dyDescent="0.25" r="235" customHeight="1" ht="18.75">
+      <c r="A235" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="B235" t="s">
+      <c r="B235" s="1" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="236" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A236" t="s">
+    <row x14ac:dyDescent="0.25" r="236" customHeight="1" ht="18.75">
+      <c r="A236" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="B236" t="s">
+      <c r="B236" s="1" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="237" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A237" t="s">
+    <row x14ac:dyDescent="0.25" r="237" customHeight="1" ht="18.75">
+      <c r="A237" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="B237" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="238" customHeight="1" ht="18.75">
+      <c r="A238" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B238" s="1" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="239" customHeight="1" ht="18.75">
+      <c r="A239" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B239" s="1" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="240" customHeight="1" ht="18.75">
+      <c r="A240" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="B240" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="241" customHeight="1" ht="18.75">
+      <c r="A241" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="B241" s="1" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="242" customHeight="1" ht="18.75">
+      <c r="A242" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="B242" s="1" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="243" customHeight="1" ht="18.75">
+      <c r="A243" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B243" s="1" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="244" customHeight="1" ht="18.75">
+      <c r="A244" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="245" customHeight="1" ht="18.75">
+      <c r="A245" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="B245" s="1" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="246" customHeight="1" ht="18.75">
+      <c r="A246" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="B246" s="1" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="247" customHeight="1" ht="18.75">
+      <c r="A247" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="B247" s="1" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="248" customHeight="1" ht="18.75">
+      <c r="A248" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="B248" s="1" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="249" customHeight="1" ht="18.75">
+      <c r="A249" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="B249" s="1" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="250" customHeight="1" ht="18.75">
+      <c r="A250" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="B250" s="1" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="251" customHeight="1" ht="18.75">
+      <c r="A251" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B251" s="1" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="252" customHeight="1" ht="18.75">
+      <c r="A252" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="B252" s="1" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="253" customHeight="1" ht="18.75">
+      <c r="A253" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B253" s="1" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="254" customHeight="1" ht="18.75">
+      <c r="A254" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="B254" s="1" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="255" customHeight="1" ht="18.75">
+      <c r="A255" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="B255" s="1" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="256" customHeight="1" ht="18.75">
+      <c r="A256" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="B256" s="1" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="257" customHeight="1" ht="18.75">
+      <c r="A257" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B257" s="1" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="258" customHeight="1" ht="18.75">
+      <c r="A258" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="B258" s="1" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="259" customHeight="1" ht="18.75">
+      <c r="A259" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="B259" s="1" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="260" customHeight="1" ht="18.75">
+      <c r="A260" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="B260" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="18.75">
+      <c r="A261" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="B261" s="3" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="18.75">
+      <c r="A262" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="B262" s="1" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="263" customHeight="1" ht="18.75">
+      <c r="A263" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="B263" s="3" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="264" customHeight="1" ht="18.75">
+      <c r="A264" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B264" s="3" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="265" customHeight="1" ht="18.75">
+      <c r="A265" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="B265" s="3" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="266" customHeight="1" ht="18.75">
+      <c r="A266" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="B266" s="1" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="267" customHeight="1" ht="18.75">
+      <c r="A267" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="B267" s="1" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="268" customHeight="1" ht="18.75">
+      <c r="A268" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="B268" s="1" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="269" customHeight="1" ht="18.75">
+      <c r="A269" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="B269" s="1" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="270" customHeight="1" ht="18.75">
+      <c r="A270" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="B270" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="271" customHeight="1" ht="18.75">
+      <c r="A271" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="B271" s="1" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="18.75">
+      <c r="A272" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="B272" s="1" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="273" customHeight="1" ht="18.75">
+      <c r="A273" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="B273" s="3" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="18.75">
+      <c r="A274" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="B274" s="1" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="275" customHeight="1" ht="18.75">
+      <c r="A275" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="B275" s="1" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="276" customHeight="1" ht="18.75">
+      <c r="A276" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="B276" s="1" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="277" customHeight="1" ht="18.75">
+      <c r="A277" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="B277" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="18.75">
+      <c r="A278" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="B278" s="1" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="279" customHeight="1" ht="18.75">
+      <c r="A279" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="B279" s="1" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="280" customHeight="1" ht="18.75">
+      <c r="A280" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="B280" s="1" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="281" customHeight="1" ht="18.75">
+      <c r="A281" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="B281" s="1" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="282" customHeight="1" ht="18.75">
+      <c r="A282" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="B282" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="283" customHeight="1" ht="18.75">
+      <c r="A283" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="B283" s="1" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="284" customHeight="1" ht="18.75">
+      <c r="A284" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="B284" s="1" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="285" customHeight="1" ht="18.75">
+      <c r="A285" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="B285" s="1" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="286" customHeight="1" ht="18.75">
+      <c r="A286" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="B286" s="1" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="287" customHeight="1" ht="18.75">
+      <c r="A287" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="B287" s="1" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="288" customHeight="1" ht="18.75">
+      <c r="A288" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="B288" s="1" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="289" customHeight="1" ht="18.75">
+      <c r="A289" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="B289" s="3" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="290" customHeight="1" ht="18.75">
+      <c r="A290" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="291" customHeight="1" ht="18.75">
+      <c r="A291" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="B291" s="1" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="292" customHeight="1" ht="18.75">
+      <c r="A292" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="B292" s="1" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="293" customHeight="1" ht="18.75">
+      <c r="A293" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="B293" s="3" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="294" customHeight="1" ht="18.75">
+      <c r="A294" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="B294" s="1" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="295" customHeight="1" ht="18.75">
+      <c r="A295" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="B295" s="1" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="296" customHeight="1" ht="18.75">
+      <c r="A296" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="B296" s="1" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="297" customHeight="1" ht="18.75">
+      <c r="A297" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="B297" s="1" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="298" customHeight="1" ht="18.75">
+      <c r="A298" s="1" t="s">
         <v>575</v>
       </c>
-      <c r="B237" t="s">
+      <c r="B298" s="1" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="238" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A238" t="s">
+    <row x14ac:dyDescent="0.25" r="299" customHeight="1" ht="18.75">
+      <c r="A299" s="1" t="s">
         <v>577</v>
       </c>
-      <c r="B238" t="s">
+      <c r="B299" s="1" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="239" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A239" t="s">
+    <row x14ac:dyDescent="0.25" r="300" customHeight="1" ht="18.75">
+      <c r="A300" s="1" t="s">
         <v>579</v>
       </c>
-      <c r="B239" t="s">
+      <c r="B300" s="1" t="s">
         <v>580</v>
       </c>
     </row>
-    <row r="240" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A240" t="s">
-        <v>456</v>
-      </c>
-      <c r="B240" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="241" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A241" t="s">
-        <v>458</v>
-      </c>
-      <c r="B241" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="242" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A242" t="s">
-        <v>460</v>
-      </c>
-      <c r="B242" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="243" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A243" t="s">
-        <v>462</v>
-      </c>
-      <c r="B243" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="244" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A244" t="s">
-        <v>464</v>
-      </c>
-      <c r="B244" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="245" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A245" t="s">
-        <v>466</v>
-      </c>
-      <c r="B245" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="246" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A246" t="s">
-        <v>468</v>
-      </c>
-      <c r="B246" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="247" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A247" t="s">
-        <v>470</v>
-      </c>
-      <c r="B247" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="248" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A248" t="s">
-        <v>472</v>
-      </c>
-      <c r="B248" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="249" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A249" t="s">
-        <v>474</v>
-      </c>
-      <c r="B249" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="250" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A250" t="s">
-        <v>476</v>
-      </c>
-      <c r="B250" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="251" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A251" t="s">
-        <v>478</v>
-      </c>
-      <c r="B251" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="252" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A252" t="s">
-        <v>480</v>
-      </c>
-      <c r="B252" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="253" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A253" t="s">
-        <v>482</v>
-      </c>
-      <c r="B253" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="254" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A254" t="s">
-        <v>484</v>
-      </c>
-      <c r="B254" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="255" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A255" t="s">
-        <v>486</v>
-      </c>
-      <c r="B255" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="256" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A256" t="s">
-        <v>488</v>
-      </c>
-      <c r="B256" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="257" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A257" t="s">
-        <v>490</v>
-      </c>
-      <c r="B257" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="258" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A258" t="s">
-        <v>492</v>
-      </c>
-      <c r="B258" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="259" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A259" s="1" t="s">
-        <v>493</v>
-      </c>
-      <c r="B259" s="1" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="260" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A260" t="s">
-        <v>495</v>
-      </c>
-      <c r="B260" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="261" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A261" s="1" t="s">
-        <v>497</v>
-      </c>
-      <c r="B261" s="1" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="262" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A262" s="1" t="s">
-        <v>499</v>
-      </c>
-      <c r="B262" s="1" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="263" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A263" s="1" t="s">
-        <v>501</v>
-      </c>
-      <c r="B263" s="1" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="264" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A264" t="s">
-        <v>503</v>
-      </c>
-      <c r="B264" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="265" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A265" t="s">
-        <v>505</v>
-      </c>
-      <c r="B265" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="266" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A266" t="s">
-        <v>507</v>
-      </c>
-      <c r="B266" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="267" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A267" t="s">
-        <v>509</v>
-      </c>
-      <c r="B267" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="268" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A268" t="s">
-        <v>511</v>
-      </c>
-      <c r="B268" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="269" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A269" t="s">
-        <v>512</v>
-      </c>
-      <c r="B269" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="270" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A270" t="s">
-        <v>514</v>
-      </c>
-      <c r="B270" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="271" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A271" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="B271" s="1" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="272" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A272" t="s">
-        <v>518</v>
-      </c>
-      <c r="B272" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="273" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A273" t="s">
-        <v>520</v>
-      </c>
-      <c r="B273" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="274" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A274" t="s">
-        <v>522</v>
-      </c>
-      <c r="B274" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="275" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A275" t="s">
-        <v>523</v>
-      </c>
-      <c r="B275" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="276" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A276" t="s">
-        <v>525</v>
-      </c>
-      <c r="B276" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="277" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A277" t="s">
-        <v>527</v>
-      </c>
-      <c r="B277" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="278" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A278" t="s">
-        <v>529</v>
-      </c>
-      <c r="B278" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="279" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A279" t="s">
-        <v>531</v>
-      </c>
-      <c r="B279" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="280" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A280" t="s">
-        <v>533</v>
-      </c>
-      <c r="B280" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="281" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A281" t="s">
-        <v>535</v>
-      </c>
-      <c r="B281" t="s">
-        <v>536</v>
-      </c>
-    </row>
-    <row r="282" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A282" t="s">
-        <v>537</v>
-      </c>
-      <c r="B282" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="283" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A283" t="s">
-        <v>539</v>
-      </c>
-      <c r="B283" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A284" t="s">
-        <v>541</v>
-      </c>
-      <c r="B284" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="285" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A285" t="s">
-        <v>543</v>
-      </c>
-      <c r="B285" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="286" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A286" t="s">
-        <v>545</v>
-      </c>
-      <c r="B286" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A287" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="B287" s="1" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="288" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A288" t="s">
-        <v>549</v>
-      </c>
-      <c r="B288" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="289" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A289" t="s">
-        <v>551</v>
-      </c>
-      <c r="B289" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A290" t="s">
-        <v>553</v>
-      </c>
-      <c r="B290" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="291" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A291" s="1" t="s">
-        <v>555</v>
-      </c>
-      <c r="B291" s="1" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="292" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A292" t="s">
-        <v>557</v>
-      </c>
-      <c r="B292" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="293" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A293" t="s">
-        <v>559</v>
-      </c>
-      <c r="B293" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="294" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A294" t="s">
-        <v>561</v>
-      </c>
-      <c r="B294" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="295" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A295" t="s">
-        <v>563</v>
-      </c>
-      <c r="B295" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="296" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A296" t="s">
-        <v>565</v>
-      </c>
-      <c r="B296" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="297" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A297" t="s">
-        <v>567</v>
-      </c>
-      <c r="B297" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="298" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A298" t="s">
-        <v>569</v>
-      </c>
-      <c r="B298" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="299" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A299" t="s">
-        <v>571</v>
-      </c>
-      <c r="B299" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="300" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A300" t="s">
-        <v>573</v>
-      </c>
-      <c r="B300" t="s">
-        <v>574</v>
+    <row x14ac:dyDescent="0.25" r="301" customHeight="1" ht="18.75">
+      <c r="A301" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="B301" s="1" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="302" customHeight="1" ht="18.75">
+      <c r="A302" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="B302" s="1" t="s">
+        <v>584</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MAUI-5787 Update datasets to exclude encounters from sensitive facilities (#253) (#258)
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -1,29 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julia\Documents\GitHub\tamanu-source-dbt\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74409AB8-E8B9-4DE4-AACE-7B87B9E1ADBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14390" yWindow="-10" windowWidth="14420" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Translated String" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Translated String"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Translated String'!$A$1:$B$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="585">
   <si>
     <t>stringId</t>
   </si>
@@ -1009,18 +1003,18 @@
     <t>Edited by user</t>
   </si>
   <si>
+    <t>report.reporting.logChangeDateTime</t>
+  </si>
+  <si>
+    <t>Date and time edited</t>
+  </si>
+  <si>
     <t>report.reporting.logChangeRecordCreatedDateTime</t>
   </si>
   <si>
     <t>Date and time created</t>
   </si>
   <si>
-    <t>report.reporting.logChangeDateTime</t>
-  </si>
-  <si>
-    <t>Date and time edited</t>
-  </si>
-  <si>
     <t>report.reporting.medications</t>
   </si>
   <si>
@@ -1279,6 +1273,24 @@
     <t>Social security number</t>
   </si>
   <si>
+    <t>report.reporting.patientStreetVillage</t>
+  </si>
+  <si>
+    <t>Street / Village</t>
+  </si>
+  <si>
+    <t>report.reporting.patientSubDivision</t>
+  </si>
+  <si>
+    <t>Sub-division</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTitle</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
     <t>report.reporting.patientTotal</t>
   </si>
   <si>
@@ -1339,24 +1351,6 @@
     <t>Total patients with missing location</t>
   </si>
   <si>
-    <t>report.reporting.patientStreetVillage</t>
-  </si>
-  <si>
-    <t>Street / Village</t>
-  </si>
-  <si>
-    <t>report.reporting.patientSubDivision</t>
-  </si>
-  <si>
-    <t>Sub-division</t>
-  </si>
-  <si>
-    <t>report.reporting.patientTitle</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
     <t>report.reporting.patientVillage</t>
   </si>
   <si>
@@ -1393,6 +1387,36 @@
     <t>Tamanu user name</t>
   </si>
   <si>
+    <t>report.reporting.prescriptionDate</t>
+  </si>
+  <si>
+    <t>Prescription date</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedication</t>
+  </si>
+  <si>
+    <t>Medication</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedicationCode</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionQuantity</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionSelectedForDischarge</t>
+  </si>
+  <si>
+    <t>Prescription selected for discharge</t>
+  </si>
+  <si>
     <t>report.reporting.procedure</t>
   </si>
   <si>
@@ -1748,37 +1772,26 @@
   </si>
   <si>
     <t>Schedule</t>
-  </si>
-  <si>
-    <t>report.reporting.prescriptionMedication</t>
-  </si>
-  <si>
-    <t>Medication</t>
-  </si>
-  <si>
-    <t>report.reporting.prescriptionMedicationCode</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>report.reporting.prescriptionQuantity</t>
-  </si>
-  <si>
-    <t>Quantity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1814,24 +1827,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="5">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1842,10 +1860,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -1883,71 +1901,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1975,7 +1993,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1998,11 +2016,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -2011,13 +2029,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -2027,7 +2045,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -2036,7 +2054,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -2045,7 +2063,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -2053,10 +2071,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -2121,2415 +2139,2431 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B300"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:B302"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="64.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" style="4" width="64.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="35.71928571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+      <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+      <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+      <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+      <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+      <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+      <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+      <c r="A22" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+      <c r="A23" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+      <c r="A24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+      <c r="A25" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+      <c r="A26" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" t="s">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+      <c r="A27" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A28" t="s">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+      <c r="A28" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" t="s">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+      <c r="A29" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" t="s">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+      <c r="A30" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" t="s">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+      <c r="A31" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
+      <c r="A32" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" t="s">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
+      <c r="A33" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" t="s">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
+      <c r="A34" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
+      <c r="A35" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" t="s">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
+      <c r="A36" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" t="s">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
+      <c r="A37" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A38" t="s">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
+      <c r="A38" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A39" t="s">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
+      <c r="A39" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" t="s">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
+      <c r="A40" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" t="s">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
+      <c r="A41" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A42" t="s">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
+      <c r="A42" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A43" t="s">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
+      <c r="A43" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A44" t="s">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
+      <c r="A44" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A45" t="s">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
+      <c r="A45" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A46" t="s">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
+      <c r="A46" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A47" t="s">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
+      <c r="A47" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A48" t="s">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
+      <c r="A48" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A49" t="s">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
+      <c r="A49" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A50" t="s">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
+      <c r="A50" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A51" t="s">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
+      <c r="A51" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A52" t="s">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
+      <c r="A52" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A53" t="s">
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
+      <c r="A53" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A54" t="s">
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
+      <c r="A54" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A55" t="s">
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
+      <c r="A55" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A56" t="s">
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
+      <c r="A56" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A57" t="s">
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
+      <c r="A57" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="1" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A58" t="s">
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
+      <c r="A58" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A59" t="s">
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
+      <c r="A59" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A60" t="s">
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
+      <c r="A60" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A61" t="s">
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
+      <c r="A61" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B61" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A62" t="s">
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
+      <c r="A62" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B62" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A63" t="s">
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
+      <c r="A63" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B63" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A64" t="s">
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
+      <c r="A64" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B64" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A65" t="s">
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
+      <c r="A65" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A66" t="s">
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
+      <c r="A66" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A67" t="s">
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
+      <c r="A67" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B67" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A68" t="s">
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
+      <c r="A68" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A69" t="s">
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
+      <c r="A69" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="1" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A70" t="s">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
+      <c r="A70" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B70" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A71" t="s">
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
+      <c r="A71" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A72" t="s">
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
+      <c r="A72" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="1" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A73" t="s">
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
+      <c r="A73" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A74" t="s">
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
+      <c r="A74" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B74" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A75" t="s">
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
+      <c r="A75" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B75" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A76" t="s">
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
+      <c r="A76" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B76" s="1" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A77" t="s">
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
+      <c r="A77" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B77" s="1" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A78" t="s">
+    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
+      <c r="A78" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B78" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A79" t="s">
+    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
+      <c r="A79" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B79" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A80" t="s">
+    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
+      <c r="A80" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B80" s="1" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="81" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A81" t="s">
+    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
+      <c r="A81" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B81" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="82" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A82" t="s">
+    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
+      <c r="A82" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B82" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="83" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A83" t="s">
+    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
+      <c r="A83" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B83" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="84" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A84" t="s">
+    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
+      <c r="A84" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B84" s="1" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="85" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A85" t="s">
+    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
+      <c r="A85" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B85" s="1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="86" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A86" t="s">
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
+      <c r="A86" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B86" s="1" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="87" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A87" t="s">
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
+      <c r="A87" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B87" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="88" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A88" t="s">
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
+      <c r="A88" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B88" s="1" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="89" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A89" t="s">
+    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
+      <c r="A89" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B89" s="1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="90" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A90" t="s">
+    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
+      <c r="A90" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="91" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A91" t="s">
+    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
+      <c r="A91" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B91" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="92" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A92" t="s">
+    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
+      <c r="A92" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B92" s="1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="93" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A93" t="s">
+    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
+      <c r="A93" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B93" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="94" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A94" t="s">
+    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
+      <c r="A94" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B94" s="1" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="95" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A95" t="s">
+    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
+      <c r="A95" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B95" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="96" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A96" t="s">
+    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
+      <c r="A96" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B96" s="1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="97" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A97" t="s">
+    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
+      <c r="A97" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B97" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="98" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A98" t="s">
+    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
+      <c r="A98" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B98" s="1" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="99" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A99" t="s">
+    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
+      <c r="A99" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B99" s="1" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="100" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A100" t="s">
+    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
+      <c r="A100" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B100" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="101" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A101" t="s">
+    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
+      <c r="A101" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B101" s="1" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="102" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A102" t="s">
+    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
+      <c r="A102" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B102" s="1" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="103" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A103" t="s">
+    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
+      <c r="A103" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="B103" t="s">
+      <c r="B103" s="1" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="104" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A104" t="s">
+    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
+      <c r="A104" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B104" s="1" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="105" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A105" t="s">
+    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
+      <c r="A105" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B105" s="1" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="106" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A106" t="s">
+    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
+      <c r="A106" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B106" s="1" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="107" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A107" t="s">
+    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
+      <c r="A107" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B107" s="1" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="108" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A108" t="s">
+    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75">
+      <c r="A108" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B108" s="1" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="109" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A109" t="s">
+    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75">
+      <c r="A109" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B109" s="1" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="110" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A110" t="s">
+    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
+      <c r="A110" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B110" s="1" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="111" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A111" t="s">
+    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
+      <c r="A111" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B111" s="1" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="112" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A112" t="s">
+    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
+      <c r="A112" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="B112" t="s">
+      <c r="B112" s="1" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="113" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A113" t="s">
+    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
+      <c r="A113" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="B113" t="s">
+      <c r="B113" s="1" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="114" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A114" t="s">
+    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
+      <c r="A114" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="B114" t="s">
+      <c r="B114" s="1" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="115" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A115" t="s">
+    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
+      <c r="A115" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B115" s="1" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="116" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A116" t="s">
+    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
+      <c r="A116" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B116" s="1" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="117" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A117" t="s">
+    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
+      <c r="A117" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B117" t="s">
+      <c r="B117" s="1" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="118" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A118" t="s">
+    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
+      <c r="A118" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="B118" t="s">
+      <c r="B118" s="1" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="119" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A119" t="s">
+    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
+      <c r="A119" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="B119" t="s">
+      <c r="B119" s="1" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="120" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A120" t="s">
+    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
+      <c r="A120" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="B120" t="s">
+      <c r="B120" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="121" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A121" t="s">
+    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
+      <c r="A121" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B121" s="1" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="122" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A122" t="s">
+    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
+      <c r="A122" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="B122" t="s">
+      <c r="B122" s="1" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="123" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A123" t="s">
+    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
+      <c r="A123" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="B123" t="s">
+      <c r="B123" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="124" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A124" t="s">
+    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
+      <c r="A124" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B124" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="125" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A125" t="s">
+    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
+      <c r="A125" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="B125" t="s">
+      <c r="B125" s="1" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="126" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A126" t="s">
+    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
+      <c r="A126" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="B126" t="s">
+      <c r="B126" s="1" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="127" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A127" t="s">
+    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
+      <c r="A127" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B127" t="s">
+      <c r="B127" s="1" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="128" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A128" t="s">
+    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
+      <c r="A128" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="B128" t="s">
+      <c r="B128" s="1" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="129" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A129" t="s">
+    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
+      <c r="A129" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="B129" t="s">
+      <c r="B129" s="1" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="130" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A130" t="s">
+    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75">
+      <c r="A130" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B130" s="1" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="131" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A131" t="s">
+    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18.75">
+      <c r="A131" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="B131" t="s">
+      <c r="B131" s="1" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="132" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A132" t="s">
+    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18.75">
+      <c r="A132" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="B132" t="s">
+      <c r="B132" s="1" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="133" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A133" t="s">
+    <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="18.75">
+      <c r="A133" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B133" s="1" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="134" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A134" t="s">
+    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18.75">
+      <c r="A134" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="B134" t="s">
+      <c r="B134" s="1" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="135" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A135" t="s">
+    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18.75">
+      <c r="A135" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B135" s="1" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="136" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A136" t="s">
+    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18.75">
+      <c r="A136" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="B136" t="s">
+      <c r="B136" s="1" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="137" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A137" t="s">
+    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18.75">
+      <c r="A137" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="B137" t="s">
+      <c r="B137" s="1" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="138" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A138" t="s">
+    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18.75">
+      <c r="A138" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B138" s="1" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="139" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A139" t="s">
+    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18.75">
+      <c r="A139" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B139" t="s">
+      <c r="B139" s="1" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="140" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A140" t="s">
+    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18.75">
+      <c r="A140" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="B140" t="s">
+      <c r="B140" s="1" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="141" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A141" t="s">
+    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18.75">
+      <c r="A141" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B141" t="s">
+      <c r="B141" s="1" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="142" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A142" t="s">
+    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18.75">
+      <c r="A142" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="B142" t="s">
+      <c r="B142" s="1" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="143" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A143" t="s">
+    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18.75">
+      <c r="A143" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="B143" t="s">
+      <c r="B143" s="1" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="144" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A144" t="s">
+    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="18.75">
+      <c r="A144" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="B144" t="s">
+      <c r="B144" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="145" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A145" t="s">
+    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="18.75">
+      <c r="A145" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="B145" t="s">
+      <c r="B145" s="1" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="146" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A146" t="s">
+    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="18.75">
+      <c r="A146" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="B146" t="s">
+      <c r="B146" s="1" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="147" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A147" t="s">
+    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="18.75">
+      <c r="A147" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="B147" t="s">
+      <c r="B147" s="1" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="148" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A148" t="s">
+    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="18.75">
+      <c r="A148" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="B148" t="s">
+      <c r="B148" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="149" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A149" t="s">
+    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="18.75">
+      <c r="A149" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="B149" t="s">
+      <c r="B149" s="1" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="150" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A150" t="s">
+    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18.75">
+      <c r="A150" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="B150" t="s">
+      <c r="B150" s="1" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="151" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A151" t="s">
+    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18.75">
+      <c r="A151" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="B151" t="s">
+      <c r="B151" s="1" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="152" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A152" t="s">
+    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18.75">
+      <c r="A152" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="B152" t="s">
+      <c r="B152" s="1" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="153" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A153" t="s">
+    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="18.75">
+      <c r="A153" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="B153" t="s">
+      <c r="B153" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="154" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A154" t="s">
+    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18.75">
+      <c r="A154" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="B154" t="s">
+      <c r="B154" s="1" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="155" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A155" t="s">
+    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18.75">
+      <c r="A155" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="B155" t="s">
+      <c r="B155" s="1" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="156" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A156" t="s">
+    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18.75">
+      <c r="A156" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="B156" t="s">
+      <c r="B156" s="1" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="157" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A157" t="s">
+    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18.75">
+      <c r="A157" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="B157" t="s">
+      <c r="B157" s="1" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="158" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A158" t="s">
+    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18.75">
+      <c r="A158" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="B158" t="s">
+      <c r="B158" s="1" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="159" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A159" t="s">
+    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18.75">
+      <c r="A159" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="B159" t="s">
+      <c r="B159" s="1" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="160" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A160" t="s">
+    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18.75">
+      <c r="A160" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="B160" t="s">
+      <c r="B160" s="1" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="161" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A161" t="s">
+    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18.75">
+      <c r="A161" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="B161" t="s">
+      <c r="B161" s="1" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="162" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A162" t="s">
+    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18.75">
+      <c r="A162" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="B162" t="s">
+      <c r="B162" s="1" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="163" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A163" t="s">
+    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75">
+      <c r="A163" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="B163" t="s">
+      <c r="B163" s="1" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="164" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A164" t="s">
+    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75">
+      <c r="A164" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="B164" t="s">
+      <c r="B164" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="165" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A165" t="s">
+    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75">
+      <c r="A165" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B165" t="s">
+      <c r="B165" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="166" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A166" t="s">
+    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75">
+      <c r="A166" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="B166" t="s">
+      <c r="B166" s="1" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="167" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A167" t="s">
+    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75">
+      <c r="A167" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="B167" t="s">
+      <c r="B167" s="1" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="168" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A168" t="s">
+    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="19.5">
+      <c r="A168" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B168" t="s">
+      <c r="B168" s="1" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="169" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A169" t="s">
+    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="19.5">
+      <c r="A169" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="B169" t="s">
+      <c r="B169" s="1" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="170" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A170" t="s">
+    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="19.5">
+      <c r="A170" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="B170" t="s">
+      <c r="B170" s="1" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="171" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A171" t="s">
+    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="19.5">
+      <c r="A171" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="B171" t="s">
+      <c r="B171" s="1" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="172" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="19.5">
       <c r="A172" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="20.25">
+      <c r="A173" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="B172" s="2" t="s">
+      <c r="B173" s="3" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="173" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A173" s="1" t="s">
-        <v>328</v>
-      </c>
-      <c r="B173" s="1" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A174" t="s">
+    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="19.5">
+      <c r="A174" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="B174" t="s">
+      <c r="B174" s="1" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="175" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A175" t="s">
+    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="19.5">
+      <c r="A175" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="B175" t="s">
+      <c r="B175" s="1" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="176" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A176" t="s">
+    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="19.5">
+      <c r="A176" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="B176" t="s">
+      <c r="B176" s="1" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="177" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A177" t="s">
+    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="19.5">
+      <c r="A177" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B177" t="s">
+      <c r="B177" s="1" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="178" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A178" t="s">
+    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="19.5">
+      <c r="A178" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="B178" t="s">
+      <c r="B178" s="1" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="179" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A179" t="s">
+    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="19.5">
+      <c r="A179" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="B179" t="s">
+      <c r="B179" s="1" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="180" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A180" t="s">
+    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="19.5">
+      <c r="A180" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="B180" t="s">
+      <c r="B180" s="1" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="181" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A181" t="s">
+    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="19.5">
+      <c r="A181" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="B181" t="s">
+      <c r="B181" s="1" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="182" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A182" t="s">
+    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="19.5">
+      <c r="A182" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="B182" t="s">
+      <c r="B182" s="1" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="183" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A183" t="s">
+    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="19.5">
+      <c r="A183" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="B183" t="s">
+      <c r="B183" s="1" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="184" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A184" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="20.25">
+      <c r="A184" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="B184" s="1" t="s">
+      <c r="B184" s="3" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="185" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A185" t="s">
+    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="19.5">
+      <c r="A185" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="B185" t="s">
+      <c r="B185" s="1" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="186" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A186" t="s">
+    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="19.5">
+      <c r="A186" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="B186" t="s">
+      <c r="B186" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="187" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A187" t="s">
+    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="19.5">
+      <c r="A187" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="B187" t="s">
+      <c r="B187" s="1" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="188" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A188" t="s">
+    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="19.5">
+      <c r="A188" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="B188" t="s">
+      <c r="B188" s="1" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="189" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A189" t="s">
+    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="19.5">
+      <c r="A189" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="B189" t="s">
+      <c r="B189" s="1" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="190" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A190" t="s">
+    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="19.5">
+      <c r="A190" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="B190" t="s">
+      <c r="B190" s="1" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="191" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A191" t="s">
+    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="19.5">
+      <c r="A191" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="B191" t="s">
+      <c r="B191" s="1" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="192" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A192" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="20.25">
+      <c r="A192" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="B192" s="1" t="s">
+      <c r="B192" s="3" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="193" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A193" t="s">
+    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="19.5">
+      <c r="A193" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="B193" t="s">
+      <c r="B193" s="1" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="194" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A194" t="s">
+    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="19.5">
+      <c r="A194" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="B194" t="s">
+      <c r="B194" s="1" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="195" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A195" t="s">
+    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="19.5">
+      <c r="A195" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="B195" t="s">
+      <c r="B195" s="1" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="196" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A196" t="s">
+    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="19.5">
+      <c r="A196" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="B196" t="s">
+      <c r="B196" s="1" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="197" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A197" t="s">
+    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="19.5">
+      <c r="A197" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="B197" t="s">
+      <c r="B197" s="1" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="198" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A198" t="s">
+    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="19.5">
+      <c r="A198" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="B198" t="s">
+      <c r="B198" s="1" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="199" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A199" t="s">
+    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="19.5">
+      <c r="A199" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="B199" t="s">
+      <c r="B199" s="1" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="200" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A200" t="s">
+    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="19.5">
+      <c r="A200" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="B200" t="s">
+      <c r="B200" s="1" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="201" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A201" t="s">
+    <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="19.5">
+      <c r="A201" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B201" t="s">
+      <c r="B201" s="1" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="202" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A202" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="20.25">
+      <c r="A202" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="B202" s="1" t="s">
+      <c r="B202" s="3" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="203" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A203" t="s">
+    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="19.5">
+      <c r="A203" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="B203" t="s">
+      <c r="B203" s="1" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="204" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A204" t="s">
+    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="19.5">
+      <c r="A204" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="B204" t="s">
+      <c r="B204" s="1" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="205" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A205" t="s">
+    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="19.5">
+      <c r="A205" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="B205" t="s">
+      <c r="B205" s="1" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="206" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A206" t="s">
+    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="19.5">
+      <c r="A206" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="B206" t="s">
+      <c r="B206" s="1" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="207" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A207" t="s">
+    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="19.5">
+      <c r="A207" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="B207" t="s">
+      <c r="B207" s="1" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="208" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A208" t="s">
+    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="19.5">
+      <c r="A208" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="B208" t="s">
+      <c r="B208" s="1" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="209" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A209" t="s">
+    <row x14ac:dyDescent="0.25" r="209" customHeight="1" ht="18.75">
+      <c r="A209" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="B209" t="s">
+      <c r="B209" s="1" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="210" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A210" t="s">
+    <row x14ac:dyDescent="0.25" r="210" customHeight="1" ht="18.75">
+      <c r="A210" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="B210" t="s">
+      <c r="B210" s="1" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="211" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A211" t="s">
+    <row x14ac:dyDescent="0.25" r="211" customHeight="1" ht="18.75">
+      <c r="A211" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="B211" t="s">
+      <c r="B211" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="212" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A212" t="s">
+    <row x14ac:dyDescent="0.25" r="212" customHeight="1" ht="18.75">
+      <c r="A212" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="B212" t="s">
+      <c r="B212" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="213" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A213" t="s">
+    <row x14ac:dyDescent="0.25" r="213" customHeight="1" ht="18.75">
+      <c r="A213" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="B213" t="s">
+      <c r="B213" s="1" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="214" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A214" t="s">
+    <row x14ac:dyDescent="0.25" r="214" customHeight="1" ht="18.75">
+      <c r="A214" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="B214" t="s">
+      <c r="B214" s="1" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="215" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A215" t="s">
+    <row x14ac:dyDescent="0.25" r="215" customHeight="1" ht="18.75">
+      <c r="A215" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="B215" t="s">
+      <c r="B215" s="1" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="216" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A216" t="s">
+    <row x14ac:dyDescent="0.25" r="216" customHeight="1" ht="18.75">
+      <c r="A216" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="B216" t="s">
+      <c r="B216" s="1" t="s">
         <v>415</v>
       </c>
     </row>
-    <row r="217" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A217" t="s">
+    <row x14ac:dyDescent="0.25" r="217" customHeight="1" ht="18.75">
+      <c r="A217" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="B217" t="s">
+      <c r="B217" s="1" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="218" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A218" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="218" customHeight="1" ht="18.75">
+      <c r="A218" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="B218" s="3" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="219" customHeight="1" ht="18.75">
+      <c r="A219" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="B219" s="3" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="220" customHeight="1" ht="18.75">
+      <c r="A220" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="B220" s="1" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="221" customHeight="1" ht="19.5">
+      <c r="A221" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="B221" s="1" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="222" customHeight="1" ht="19.5">
+      <c r="A222" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="B222" s="1" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="223" customHeight="1" ht="19.5">
+      <c r="A223" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="B223" s="1" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="224" customHeight="1" ht="19.5">
+      <c r="A224" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="B224" s="1" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="225" customHeight="1" ht="19.5">
+      <c r="A225" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="B225" s="1" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="226" customHeight="1" ht="19.5">
+      <c r="A226" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="B226" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="227" customHeight="1" ht="19.5">
+      <c r="A227" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="B227" s="1" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="228" customHeight="1" ht="19.5">
+      <c r="A228" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="B218" s="1" t="s">
+      <c r="B228" s="1" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="219" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A219" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="229" customHeight="1" ht="19.5">
+      <c r="A229" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="B219" s="1" t="s">
+      <c r="B229" s="1" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="220" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A220" t="s">
+    <row x14ac:dyDescent="0.25" r="230" customHeight="1" ht="19.5">
+      <c r="A230" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="B220" t="s">
+      <c r="B230" s="1" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="221" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A221" t="s">
-        <v>418</v>
-      </c>
-      <c r="B221" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="222" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A222" t="s">
-        <v>420</v>
-      </c>
-      <c r="B222" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="223" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A223" t="s">
-        <v>422</v>
-      </c>
-      <c r="B223" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="224" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A224" t="s">
-        <v>424</v>
-      </c>
-      <c r="B224" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="225" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A225" t="s">
-        <v>426</v>
-      </c>
-      <c r="B225" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="226" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A226" t="s">
-        <v>428</v>
-      </c>
-      <c r="B226" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="227" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A227" t="s">
-        <v>430</v>
-      </c>
-      <c r="B227" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="228" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A228" t="s">
-        <v>432</v>
-      </c>
-      <c r="B228" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="229" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A229" t="s">
-        <v>434</v>
-      </c>
-      <c r="B229" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="230" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A230" t="s">
-        <v>436</v>
-      </c>
-      <c r="B230" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="231" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A231" t="s">
+    <row x14ac:dyDescent="0.25" r="231" customHeight="1" ht="18.75">
+      <c r="A231" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="B231" t="s">
+      <c r="B231" s="1" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="232" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A232" t="s">
+    <row x14ac:dyDescent="0.25" r="232" customHeight="1" ht="18.75">
+      <c r="A232" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="B232" t="s">
+      <c r="B232" s="1" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="233" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A233" t="s">
+    <row x14ac:dyDescent="0.25" r="233" customHeight="1" ht="18.75">
+      <c r="A233" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="B233" t="s">
+      <c r="B233" s="1" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="234" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A234" t="s">
+    <row x14ac:dyDescent="0.25" r="234" customHeight="1" ht="18.75">
+      <c r="A234" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="B234" t="s">
+      <c r="B234" s="1" t="s">
         <v>451</v>
       </c>
     </row>
-    <row r="235" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A235" t="s">
+    <row x14ac:dyDescent="0.25" r="235" customHeight="1" ht="18.75">
+      <c r="A235" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="B235" t="s">
+      <c r="B235" s="1" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="236" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A236" t="s">
+    <row x14ac:dyDescent="0.25" r="236" customHeight="1" ht="18.75">
+      <c r="A236" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="B236" t="s">
+      <c r="B236" s="1" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="237" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A237" t="s">
+    <row x14ac:dyDescent="0.25" r="237" customHeight="1" ht="18.75">
+      <c r="A237" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="B237" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="238" customHeight="1" ht="18.75">
+      <c r="A238" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B238" s="1" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="239" customHeight="1" ht="18.75">
+      <c r="A239" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B239" s="1" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="240" customHeight="1" ht="18.75">
+      <c r="A240" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="B240" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="241" customHeight="1" ht="18.75">
+      <c r="A241" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="B241" s="1" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="242" customHeight="1" ht="18.75">
+      <c r="A242" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="B242" s="1" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="243" customHeight="1" ht="18.75">
+      <c r="A243" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B243" s="1" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="244" customHeight="1" ht="18.75">
+      <c r="A244" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="245" customHeight="1" ht="18.75">
+      <c r="A245" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="B245" s="1" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="246" customHeight="1" ht="18.75">
+      <c r="A246" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="B246" s="1" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="247" customHeight="1" ht="18.75">
+      <c r="A247" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="B247" s="1" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="248" customHeight="1" ht="18.75">
+      <c r="A248" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="B248" s="1" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="249" customHeight="1" ht="18.75">
+      <c r="A249" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="B249" s="1" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="250" customHeight="1" ht="18.75">
+      <c r="A250" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="B250" s="1" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="251" customHeight="1" ht="18.75">
+      <c r="A251" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B251" s="1" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="252" customHeight="1" ht="18.75">
+      <c r="A252" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="B252" s="1" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="253" customHeight="1" ht="18.75">
+      <c r="A253" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B253" s="1" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="254" customHeight="1" ht="18.75">
+      <c r="A254" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="B254" s="1" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="255" customHeight="1" ht="18.75">
+      <c r="A255" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="B255" s="1" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="256" customHeight="1" ht="18.75">
+      <c r="A256" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="B256" s="1" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="257" customHeight="1" ht="18.75">
+      <c r="A257" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B257" s="1" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="258" customHeight="1" ht="18.75">
+      <c r="A258" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="B258" s="1" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="259" customHeight="1" ht="18.75">
+      <c r="A259" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="B259" s="1" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="260" customHeight="1" ht="18.75">
+      <c r="A260" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="B260" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="18.75">
+      <c r="A261" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="B261" s="3" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="18.75">
+      <c r="A262" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="B262" s="1" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="263" customHeight="1" ht="18.75">
+      <c r="A263" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="B263" s="3" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="264" customHeight="1" ht="18.75">
+      <c r="A264" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="B264" s="3" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="265" customHeight="1" ht="18.75">
+      <c r="A265" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="B265" s="3" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="266" customHeight="1" ht="18.75">
+      <c r="A266" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="B266" s="1" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="267" customHeight="1" ht="18.75">
+      <c r="A267" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="B267" s="1" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="268" customHeight="1" ht="18.75">
+      <c r="A268" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="B268" s="1" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="269" customHeight="1" ht="18.75">
+      <c r="A269" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="B269" s="1" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="270" customHeight="1" ht="18.75">
+      <c r="A270" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="B270" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="271" customHeight="1" ht="18.75">
+      <c r="A271" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="B271" s="1" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="18.75">
+      <c r="A272" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="B272" s="1" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="273" customHeight="1" ht="18.75">
+      <c r="A273" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="B273" s="3" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="18.75">
+      <c r="A274" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="B274" s="1" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="275" customHeight="1" ht="18.75">
+      <c r="A275" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="B275" s="1" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="276" customHeight="1" ht="18.75">
+      <c r="A276" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="B276" s="1" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="277" customHeight="1" ht="18.75">
+      <c r="A277" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="B277" s="1" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="18.75">
+      <c r="A278" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="B278" s="1" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="279" customHeight="1" ht="18.75">
+      <c r="A279" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="B279" s="1" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="280" customHeight="1" ht="18.75">
+      <c r="A280" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="B280" s="1" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="281" customHeight="1" ht="18.75">
+      <c r="A281" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="B281" s="1" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="282" customHeight="1" ht="18.75">
+      <c r="A282" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="B282" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="283" customHeight="1" ht="18.75">
+      <c r="A283" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="B283" s="1" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="284" customHeight="1" ht="18.75">
+      <c r="A284" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="B284" s="1" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="285" customHeight="1" ht="18.75">
+      <c r="A285" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="B285" s="1" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="286" customHeight="1" ht="18.75">
+      <c r="A286" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="B286" s="1" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="287" customHeight="1" ht="18.75">
+      <c r="A287" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="B287" s="1" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="288" customHeight="1" ht="18.75">
+      <c r="A288" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="B288" s="1" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="289" customHeight="1" ht="18.75">
+      <c r="A289" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="B289" s="3" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="290" customHeight="1" ht="18.75">
+      <c r="A290" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="291" customHeight="1" ht="18.75">
+      <c r="A291" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="B291" s="1" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="292" customHeight="1" ht="18.75">
+      <c r="A292" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="B292" s="1" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="293" customHeight="1" ht="18.75">
+      <c r="A293" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="B293" s="3" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="294" customHeight="1" ht="18.75">
+      <c r="A294" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="B294" s="1" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="295" customHeight="1" ht="18.75">
+      <c r="A295" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="B295" s="1" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="296" customHeight="1" ht="18.75">
+      <c r="A296" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="B296" s="1" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="297" customHeight="1" ht="18.75">
+      <c r="A297" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="B297" s="1" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="298" customHeight="1" ht="18.75">
+      <c r="A298" s="1" t="s">
         <v>575</v>
       </c>
-      <c r="B237" t="s">
+      <c r="B298" s="1" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="238" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A238" t="s">
+    <row x14ac:dyDescent="0.25" r="299" customHeight="1" ht="18.75">
+      <c r="A299" s="1" t="s">
         <v>577</v>
       </c>
-      <c r="B238" t="s">
+      <c r="B299" s="1" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="239" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A239" t="s">
+    <row x14ac:dyDescent="0.25" r="300" customHeight="1" ht="18.75">
+      <c r="A300" s="1" t="s">
         <v>579</v>
       </c>
-      <c r="B239" t="s">
+      <c r="B300" s="1" t="s">
         <v>580</v>
       </c>
     </row>
-    <row r="240" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A240" t="s">
-        <v>456</v>
-      </c>
-      <c r="B240" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="241" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A241" t="s">
-        <v>458</v>
-      </c>
-      <c r="B241" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="242" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A242" t="s">
-        <v>460</v>
-      </c>
-      <c r="B242" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="243" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A243" t="s">
-        <v>462</v>
-      </c>
-      <c r="B243" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="244" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A244" t="s">
-        <v>464</v>
-      </c>
-      <c r="B244" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="245" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A245" t="s">
-        <v>466</v>
-      </c>
-      <c r="B245" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="246" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A246" t="s">
-        <v>468</v>
-      </c>
-      <c r="B246" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="247" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A247" t="s">
-        <v>470</v>
-      </c>
-      <c r="B247" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="248" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A248" t="s">
-        <v>472</v>
-      </c>
-      <c r="B248" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="249" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A249" t="s">
-        <v>474</v>
-      </c>
-      <c r="B249" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="250" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A250" t="s">
-        <v>476</v>
-      </c>
-      <c r="B250" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="251" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A251" t="s">
-        <v>478</v>
-      </c>
-      <c r="B251" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="252" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A252" t="s">
-        <v>480</v>
-      </c>
-      <c r="B252" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="253" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A253" t="s">
-        <v>482</v>
-      </c>
-      <c r="B253" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="254" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A254" t="s">
-        <v>484</v>
-      </c>
-      <c r="B254" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="255" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A255" t="s">
-        <v>486</v>
-      </c>
-      <c r="B255" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="256" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A256" t="s">
-        <v>488</v>
-      </c>
-      <c r="B256" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="257" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A257" t="s">
-        <v>490</v>
-      </c>
-      <c r="B257" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="258" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A258" t="s">
-        <v>492</v>
-      </c>
-      <c r="B258" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="259" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A259" s="1" t="s">
-        <v>493</v>
-      </c>
-      <c r="B259" s="1" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="260" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A260" t="s">
-        <v>495</v>
-      </c>
-      <c r="B260" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="261" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A261" s="1" t="s">
-        <v>497</v>
-      </c>
-      <c r="B261" s="1" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="262" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A262" s="1" t="s">
-        <v>499</v>
-      </c>
-      <c r="B262" s="1" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="263" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A263" s="1" t="s">
-        <v>501</v>
-      </c>
-      <c r="B263" s="1" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="264" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A264" t="s">
-        <v>503</v>
-      </c>
-      <c r="B264" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="265" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A265" t="s">
-        <v>505</v>
-      </c>
-      <c r="B265" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="266" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A266" t="s">
-        <v>507</v>
-      </c>
-      <c r="B266" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="267" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A267" t="s">
-        <v>509</v>
-      </c>
-      <c r="B267" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="268" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A268" t="s">
-        <v>511</v>
-      </c>
-      <c r="B268" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="269" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A269" t="s">
-        <v>512</v>
-      </c>
-      <c r="B269" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="270" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A270" t="s">
-        <v>514</v>
-      </c>
-      <c r="B270" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="271" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A271" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="B271" s="1" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="272" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A272" t="s">
-        <v>518</v>
-      </c>
-      <c r="B272" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="273" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A273" t="s">
-        <v>520</v>
-      </c>
-      <c r="B273" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="274" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A274" t="s">
-        <v>522</v>
-      </c>
-      <c r="B274" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="275" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A275" t="s">
-        <v>523</v>
-      </c>
-      <c r="B275" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="276" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A276" t="s">
-        <v>525</v>
-      </c>
-      <c r="B276" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="277" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A277" t="s">
-        <v>527</v>
-      </c>
-      <c r="B277" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="278" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A278" t="s">
-        <v>529</v>
-      </c>
-      <c r="B278" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="279" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A279" t="s">
-        <v>531</v>
-      </c>
-      <c r="B279" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="280" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A280" t="s">
-        <v>533</v>
-      </c>
-      <c r="B280" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="281" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A281" t="s">
-        <v>535</v>
-      </c>
-      <c r="B281" t="s">
-        <v>536</v>
-      </c>
-    </row>
-    <row r="282" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A282" t="s">
-        <v>537</v>
-      </c>
-      <c r="B282" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="283" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A283" t="s">
-        <v>539</v>
-      </c>
-      <c r="B283" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A284" t="s">
-        <v>541</v>
-      </c>
-      <c r="B284" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="285" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A285" t="s">
-        <v>543</v>
-      </c>
-      <c r="B285" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="286" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A286" t="s">
-        <v>545</v>
-      </c>
-      <c r="B286" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A287" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="B287" s="1" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="288" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A288" t="s">
-        <v>549</v>
-      </c>
-      <c r="B288" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="289" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A289" t="s">
-        <v>551</v>
-      </c>
-      <c r="B289" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A290" t="s">
-        <v>553</v>
-      </c>
-      <c r="B290" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="291" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A291" s="1" t="s">
-        <v>555</v>
-      </c>
-      <c r="B291" s="1" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="292" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A292" t="s">
-        <v>557</v>
-      </c>
-      <c r="B292" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="293" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A293" t="s">
-        <v>559</v>
-      </c>
-      <c r="B293" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="294" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A294" t="s">
-        <v>561</v>
-      </c>
-      <c r="B294" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="295" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A295" t="s">
-        <v>563</v>
-      </c>
-      <c r="B295" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="296" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A296" t="s">
-        <v>565</v>
-      </c>
-      <c r="B296" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="297" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A297" t="s">
-        <v>567</v>
-      </c>
-      <c r="B297" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="298" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A298" t="s">
-        <v>569</v>
-      </c>
-      <c r="B298" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="299" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A299" t="s">
-        <v>571</v>
-      </c>
-      <c r="B299" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="300" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A300" t="s">
-        <v>573</v>
-      </c>
-      <c r="B300" t="s">
-        <v>574</v>
+    <row x14ac:dyDescent="0.25" r="301" customHeight="1" ht="18.75">
+      <c r="A301" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="B301" s="1" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="302" customHeight="1" ht="18.75">
+      <c r="A302" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="B302" s="1" t="s">
+        <v>584</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add dose fields to prescription model
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="585">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="601">
   <si>
     <t>stringId</t>
   </si>
@@ -1393,6 +1393,36 @@
     <t>Prescription date</t>
   </si>
   <si>
+    <t>report.reporting.prescriptionDoseAmount</t>
+  </si>
+  <si>
+    <t>Dose amount</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionFrequency</t>
+  </si>
+  <si>
+    <t>Frequency</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionIsOngoing</t>
+  </si>
+  <si>
+    <t>Is ongoing</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionIsPRN</t>
+  </si>
+  <si>
+    <t>Is PRN</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionIsVariableDoses</t>
+  </si>
+  <si>
+    <t>Is variable dose</t>
+  </si>
+  <si>
     <t>report.reporting.prescriptionMedication</t>
   </si>
   <si>
@@ -1411,10 +1441,28 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>report.reporting.prescriptionRepeats</t>
+  </si>
+  <si>
+    <t>Repeats</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionRoute</t>
+  </si>
+  <si>
+    <t>Route</t>
+  </si>
+  <si>
     <t>report.reporting.prescriptionSelectedForDischarge</t>
   </si>
   <si>
     <t>Prescription selected for discharge</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionUnits</t>
+  </si>
+  <si>
+    <t>Units</t>
   </si>
   <si>
     <t>report.reporting.procedure</t>
@@ -1789,7 +1837,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -2143,7 +2191,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B302"/>
+  <dimension ref="A1:B310"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="4" width="64.43357142857143" customWidth="1" bestFit="1"/>
@@ -3566,7 +3614,7 @@
         <v>339</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18.75">
       <c r="A178" s="1" t="s">
         <v>340</v>
       </c>
@@ -3574,7 +3622,7 @@
         <v>341</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18.75">
       <c r="A179" s="1" t="s">
         <v>342</v>
       </c>
@@ -3582,7 +3630,7 @@
         <v>343</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18.75">
       <c r="A180" s="1" t="s">
         <v>344</v>
       </c>
@@ -3590,7 +3638,7 @@
         <v>345</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18.75">
       <c r="A181" s="1" t="s">
         <v>346</v>
       </c>
@@ -3598,7 +3646,7 @@
         <v>347</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18.75">
       <c r="A182" s="1" t="s">
         <v>348</v>
       </c>
@@ -3606,7 +3654,7 @@
         <v>349</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18.75">
       <c r="A183" s="1" t="s">
         <v>350</v>
       </c>
@@ -3614,7 +3662,7 @@
         <v>351</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="19.5">
       <c r="A184" s="3" t="s">
         <v>352</v>
       </c>
@@ -3622,7 +3670,7 @@
         <v>353</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18.75">
       <c r="A185" s="1" t="s">
         <v>354</v>
       </c>
@@ -3630,7 +3678,7 @@
         <v>355</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75">
       <c r="A186" s="1" t="s">
         <v>356</v>
       </c>
@@ -3638,7 +3686,7 @@
         <v>357</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18.75">
       <c r="A187" s="1" t="s">
         <v>358</v>
       </c>
@@ -3646,7 +3694,7 @@
         <v>359</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75">
       <c r="A188" s="1" t="s">
         <v>360</v>
       </c>
@@ -3654,7 +3702,7 @@
         <v>361</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75">
       <c r="A189" s="1" t="s">
         <v>362</v>
       </c>
@@ -3662,7 +3710,7 @@
         <v>363</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75">
       <c r="A190" s="1" t="s">
         <v>364</v>
       </c>
@@ -3670,7 +3718,7 @@
         <v>365</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18.75">
       <c r="A191" s="1" t="s">
         <v>366</v>
       </c>
@@ -3678,7 +3726,7 @@
         <v>367</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="19.5">
       <c r="A192" s="3" t="s">
         <v>368</v>
       </c>
@@ -3686,7 +3734,7 @@
         <v>369</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18.75">
       <c r="A193" s="1" t="s">
         <v>370</v>
       </c>
@@ -3694,7 +3742,7 @@
         <v>371</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="18.75">
       <c r="A194" s="1" t="s">
         <v>372</v>
       </c>
@@ -3702,7 +3750,7 @@
         <v>373</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18.75">
       <c r="A195" s="1" t="s">
         <v>374</v>
       </c>
@@ -3710,7 +3758,7 @@
         <v>375</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="18.75">
       <c r="A196" s="1" t="s">
         <v>376</v>
       </c>
@@ -3718,7 +3766,7 @@
         <v>377</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18.75">
       <c r="A197" s="1" t="s">
         <v>378</v>
       </c>
@@ -3726,7 +3774,7 @@
         <v>379</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="18.75">
       <c r="A198" s="1" t="s">
         <v>380</v>
       </c>
@@ -3734,7 +3782,7 @@
         <v>381</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="18.75">
       <c r="A199" s="1" t="s">
         <v>382</v>
       </c>
@@ -3742,7 +3790,7 @@
         <v>383</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="18.75">
       <c r="A200" s="1" t="s">
         <v>384</v>
       </c>
@@ -4227,78 +4275,78 @@
         <v>502</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>241</v>
+        <v>503</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="18.75">
-      <c r="A261" s="3" t="s">
-        <v>503</v>
-      </c>
-      <c r="B261" s="3" t="s">
+      <c r="A261" s="1" t="s">
         <v>504</v>
+      </c>
+      <c r="B261" s="1" t="s">
+        <v>505</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="18.75">
       <c r="A262" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="263" customHeight="1" ht="18.75">
-      <c r="A263" s="3" t="s">
-        <v>507</v>
-      </c>
-      <c r="B263" s="3" t="s">
+      <c r="A263" s="1" t="s">
         <v>508</v>
       </c>
+      <c r="B263" s="1" t="s">
+        <v>509</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="264" customHeight="1" ht="18.75">
-      <c r="A264" s="3" t="s">
-        <v>509</v>
-      </c>
-      <c r="B264" s="3" t="s">
+      <c r="A264" s="1" t="s">
         <v>510</v>
       </c>
+      <c r="B264" s="1" t="s">
+        <v>511</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="265" customHeight="1" ht="18.75">
-      <c r="A265" s="3" t="s">
-        <v>511</v>
-      </c>
-      <c r="B265" s="3" t="s">
+      <c r="A265" s="1" t="s">
         <v>512</v>
+      </c>
+      <c r="B265" s="1" t="s">
+        <v>513</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="266" customHeight="1" ht="18.75">
       <c r="A266" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B266" s="1" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="267" customHeight="1" ht="18.75">
       <c r="A267" s="1" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B267" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="268" customHeight="1" ht="18.75">
       <c r="A268" s="1" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B268" s="1" t="s">
-        <v>518</v>
+        <v>241</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="269" customHeight="1" ht="18.75">
-      <c r="A269" s="1" t="s">
+      <c r="A269" s="3" t="s">
         <v>519</v>
       </c>
-      <c r="B269" s="1" t="s">
+      <c r="B269" s="3" t="s">
         <v>520</v>
       </c>
     </row>
@@ -4307,119 +4355,119 @@
         <v>521</v>
       </c>
       <c r="B270" s="1" t="s">
-        <v>47</v>
+        <v>522</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="271" customHeight="1" ht="18.75">
-      <c r="A271" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="B271" s="1" t="s">
+      <c r="A271" s="3" t="s">
         <v>523</v>
       </c>
+      <c r="B271" s="3" t="s">
+        <v>524</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="18.75">
-      <c r="A272" s="1" t="s">
-        <v>524</v>
-      </c>
-      <c r="B272" s="1" t="s">
+      <c r="A272" s="3" t="s">
         <v>525</v>
+      </c>
+      <c r="B272" s="3" t="s">
+        <v>526</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="273" customHeight="1" ht="18.75">
       <c r="A273" s="3" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B273" s="3" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="18.75">
       <c r="A274" s="1" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B274" s="1" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="275" customHeight="1" ht="18.75">
       <c r="A275" s="1" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B275" s="1" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="276" customHeight="1" ht="18.75">
       <c r="A276" s="1" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B276" s="1" t="s">
-        <v>277</v>
+        <v>534</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="277" customHeight="1" ht="18.75">
       <c r="A277" s="1" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B277" s="1" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="18.75">
       <c r="A278" s="1" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B278" s="1" t="s">
-        <v>536</v>
+        <v>47</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="279" customHeight="1" ht="18.75">
       <c r="A279" s="1" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B279" s="1" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="280" customHeight="1" ht="18.75">
       <c r="A280" s="1" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B280" s="1" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="281" customHeight="1" ht="18.75">
-      <c r="A281" s="1" t="s">
-        <v>541</v>
-      </c>
-      <c r="B281" s="1" t="s">
+      <c r="A281" s="3" t="s">
         <v>542</v>
+      </c>
+      <c r="B281" s="3" t="s">
+        <v>543</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="282" customHeight="1" ht="18.75">
       <c r="A282" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="283" customHeight="1" ht="18.75">
       <c r="A283" s="1" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B283" s="1" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="284" customHeight="1" ht="18.75">
       <c r="A284" s="1" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B284" s="1" t="s">
-        <v>548</v>
+        <v>277</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="285" customHeight="1" ht="18.75">
@@ -4455,10 +4503,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="289" customHeight="1" ht="18.75">
-      <c r="A289" s="3" t="s">
+      <c r="A289" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="B289" s="3" t="s">
+      <c r="B289" s="1" t="s">
         <v>558</v>
       </c>
     </row>
@@ -4487,10 +4535,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="293" customHeight="1" ht="18.75">
-      <c r="A293" s="3" t="s">
+      <c r="A293" s="1" t="s">
         <v>565</v>
       </c>
-      <c r="B293" s="3" t="s">
+      <c r="B293" s="1" t="s">
         <v>566</v>
       </c>
     </row>
@@ -4519,10 +4567,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="297" customHeight="1" ht="18.75">
-      <c r="A297" s="1" t="s">
+      <c r="A297" s="3" t="s">
         <v>573</v>
       </c>
-      <c r="B297" s="1" t="s">
+      <c r="B297" s="3" t="s">
         <v>574</v>
       </c>
     </row>
@@ -4551,10 +4599,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="301" customHeight="1" ht="18.75">
-      <c r="A301" s="1" t="s">
+      <c r="A301" s="3" t="s">
         <v>581</v>
       </c>
-      <c r="B301" s="1" t="s">
+      <c r="B301" s="3" t="s">
         <v>582</v>
       </c>
     </row>
@@ -4564,6 +4612,70 @@
       </c>
       <c r="B302" s="1" t="s">
         <v>584</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="303" customHeight="1" ht="18.75">
+      <c r="A303" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="B303" s="1" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="304" customHeight="1" ht="18.75">
+      <c r="A304" s="1" t="s">
+        <v>587</v>
+      </c>
+      <c r="B304" s="1" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="305" customHeight="1" ht="18.75">
+      <c r="A305" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="B305" s="1" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="306" customHeight="1" ht="18.75">
+      <c r="A306" s="1" t="s">
+        <v>591</v>
+      </c>
+      <c r="B306" s="1" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="307" customHeight="1" ht="18.75">
+      <c r="A307" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="B307" s="1" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="308" customHeight="1" ht="18.75">
+      <c r="A308" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="B308" s="1" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="309" customHeight="1" ht="18.75">
+      <c r="A309" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="B309" s="1" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="310" customHeight="1" ht="18.75">
+      <c r="A310" s="1" t="s">
+        <v>599</v>
+      </c>
+      <c r="B310" s="1" t="s">
+        <v>600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add dose fields to prescription model (#269)
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="585">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="601">
   <si>
     <t>stringId</t>
   </si>
@@ -1393,6 +1393,36 @@
     <t>Prescription date</t>
   </si>
   <si>
+    <t>report.reporting.prescriptionDoseAmount</t>
+  </si>
+  <si>
+    <t>Dose amount</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionFrequency</t>
+  </si>
+  <si>
+    <t>Frequency</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionIsOngoing</t>
+  </si>
+  <si>
+    <t>Is ongoing</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionIsPRN</t>
+  </si>
+  <si>
+    <t>Is PRN</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionIsVariableDoses</t>
+  </si>
+  <si>
+    <t>Is variable dose</t>
+  </si>
+  <si>
     <t>report.reporting.prescriptionMedication</t>
   </si>
   <si>
@@ -1411,10 +1441,28 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>report.reporting.prescriptionRepeats</t>
+  </si>
+  <si>
+    <t>Repeats</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionRoute</t>
+  </si>
+  <si>
+    <t>Route</t>
+  </si>
+  <si>
     <t>report.reporting.prescriptionSelectedForDischarge</t>
   </si>
   <si>
     <t>Prescription selected for discharge</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionUnits</t>
+  </si>
+  <si>
+    <t>Units</t>
   </si>
   <si>
     <t>report.reporting.procedure</t>
@@ -1789,7 +1837,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -2143,7 +2191,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B302"/>
+  <dimension ref="A1:B310"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="4" width="64.43357142857143" customWidth="1" bestFit="1"/>
@@ -3566,7 +3614,7 @@
         <v>339</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18.75">
       <c r="A178" s="1" t="s">
         <v>340</v>
       </c>
@@ -3574,7 +3622,7 @@
         <v>341</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18.75">
       <c r="A179" s="1" t="s">
         <v>342</v>
       </c>
@@ -3582,7 +3630,7 @@
         <v>343</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18.75">
       <c r="A180" s="1" t="s">
         <v>344</v>
       </c>
@@ -3590,7 +3638,7 @@
         <v>345</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18.75">
       <c r="A181" s="1" t="s">
         <v>346</v>
       </c>
@@ -3598,7 +3646,7 @@
         <v>347</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18.75">
       <c r="A182" s="1" t="s">
         <v>348</v>
       </c>
@@ -3606,7 +3654,7 @@
         <v>349</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18.75">
       <c r="A183" s="1" t="s">
         <v>350</v>
       </c>
@@ -3614,7 +3662,7 @@
         <v>351</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="19.5">
       <c r="A184" s="3" t="s">
         <v>352</v>
       </c>
@@ -3622,7 +3670,7 @@
         <v>353</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18.75">
       <c r="A185" s="1" t="s">
         <v>354</v>
       </c>
@@ -3630,7 +3678,7 @@
         <v>355</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75">
       <c r="A186" s="1" t="s">
         <v>356</v>
       </c>
@@ -3638,7 +3686,7 @@
         <v>357</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18.75">
       <c r="A187" s="1" t="s">
         <v>358</v>
       </c>
@@ -3646,7 +3694,7 @@
         <v>359</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75">
       <c r="A188" s="1" t="s">
         <v>360</v>
       </c>
@@ -3654,7 +3702,7 @@
         <v>361</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75">
       <c r="A189" s="1" t="s">
         <v>362</v>
       </c>
@@ -3662,7 +3710,7 @@
         <v>363</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75">
       <c r="A190" s="1" t="s">
         <v>364</v>
       </c>
@@ -3670,7 +3718,7 @@
         <v>365</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18.75">
       <c r="A191" s="1" t="s">
         <v>366</v>
       </c>
@@ -3678,7 +3726,7 @@
         <v>367</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="19.5">
       <c r="A192" s="3" t="s">
         <v>368</v>
       </c>
@@ -3686,7 +3734,7 @@
         <v>369</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18.75">
       <c r="A193" s="1" t="s">
         <v>370</v>
       </c>
@@ -3694,7 +3742,7 @@
         <v>371</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="18.75">
       <c r="A194" s="1" t="s">
         <v>372</v>
       </c>
@@ -3702,7 +3750,7 @@
         <v>373</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18.75">
       <c r="A195" s="1" t="s">
         <v>374</v>
       </c>
@@ -3710,7 +3758,7 @@
         <v>375</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="18.75">
       <c r="A196" s="1" t="s">
         <v>376</v>
       </c>
@@ -3718,7 +3766,7 @@
         <v>377</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18.75">
       <c r="A197" s="1" t="s">
         <v>378</v>
       </c>
@@ -3726,7 +3774,7 @@
         <v>379</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="18.75">
       <c r="A198" s="1" t="s">
         <v>380</v>
       </c>
@@ -3734,7 +3782,7 @@
         <v>381</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="18.75">
       <c r="A199" s="1" t="s">
         <v>382</v>
       </c>
@@ -3742,7 +3790,7 @@
         <v>383</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="18.75">
       <c r="A200" s="1" t="s">
         <v>384</v>
       </c>
@@ -4227,78 +4275,78 @@
         <v>502</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>241</v>
+        <v>503</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="18.75">
-      <c r="A261" s="3" t="s">
-        <v>503</v>
-      </c>
-      <c r="B261" s="3" t="s">
+      <c r="A261" s="1" t="s">
         <v>504</v>
+      </c>
+      <c r="B261" s="1" t="s">
+        <v>505</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="18.75">
       <c r="A262" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="263" customHeight="1" ht="18.75">
-      <c r="A263" s="3" t="s">
-        <v>507</v>
-      </c>
-      <c r="B263" s="3" t="s">
+      <c r="A263" s="1" t="s">
         <v>508</v>
       </c>
+      <c r="B263" s="1" t="s">
+        <v>509</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="264" customHeight="1" ht="18.75">
-      <c r="A264" s="3" t="s">
-        <v>509</v>
-      </c>
-      <c r="B264" s="3" t="s">
+      <c r="A264" s="1" t="s">
         <v>510</v>
       </c>
+      <c r="B264" s="1" t="s">
+        <v>511</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="265" customHeight="1" ht="18.75">
-      <c r="A265" s="3" t="s">
-        <v>511</v>
-      </c>
-      <c r="B265" s="3" t="s">
+      <c r="A265" s="1" t="s">
         <v>512</v>
+      </c>
+      <c r="B265" s="1" t="s">
+        <v>513</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="266" customHeight="1" ht="18.75">
       <c r="A266" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B266" s="1" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="267" customHeight="1" ht="18.75">
       <c r="A267" s="1" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B267" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="268" customHeight="1" ht="18.75">
       <c r="A268" s="1" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B268" s="1" t="s">
-        <v>518</v>
+        <v>241</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="269" customHeight="1" ht="18.75">
-      <c r="A269" s="1" t="s">
+      <c r="A269" s="3" t="s">
         <v>519</v>
       </c>
-      <c r="B269" s="1" t="s">
+      <c r="B269" s="3" t="s">
         <v>520</v>
       </c>
     </row>
@@ -4307,119 +4355,119 @@
         <v>521</v>
       </c>
       <c r="B270" s="1" t="s">
-        <v>47</v>
+        <v>522</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="271" customHeight="1" ht="18.75">
-      <c r="A271" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="B271" s="1" t="s">
+      <c r="A271" s="3" t="s">
         <v>523</v>
       </c>
+      <c r="B271" s="3" t="s">
+        <v>524</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="18.75">
-      <c r="A272" s="1" t="s">
-        <v>524</v>
-      </c>
-      <c r="B272" s="1" t="s">
+      <c r="A272" s="3" t="s">
         <v>525</v>
+      </c>
+      <c r="B272" s="3" t="s">
+        <v>526</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="273" customHeight="1" ht="18.75">
       <c r="A273" s="3" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B273" s="3" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="18.75">
       <c r="A274" s="1" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B274" s="1" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="275" customHeight="1" ht="18.75">
       <c r="A275" s="1" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B275" s="1" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="276" customHeight="1" ht="18.75">
       <c r="A276" s="1" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B276" s="1" t="s">
-        <v>277</v>
+        <v>534</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="277" customHeight="1" ht="18.75">
       <c r="A277" s="1" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B277" s="1" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="18.75">
       <c r="A278" s="1" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B278" s="1" t="s">
-        <v>536</v>
+        <v>47</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="279" customHeight="1" ht="18.75">
       <c r="A279" s="1" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B279" s="1" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="280" customHeight="1" ht="18.75">
       <c r="A280" s="1" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B280" s="1" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="281" customHeight="1" ht="18.75">
-      <c r="A281" s="1" t="s">
-        <v>541</v>
-      </c>
-      <c r="B281" s="1" t="s">
+      <c r="A281" s="3" t="s">
         <v>542</v>
+      </c>
+      <c r="B281" s="3" t="s">
+        <v>543</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="282" customHeight="1" ht="18.75">
       <c r="A282" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="283" customHeight="1" ht="18.75">
       <c r="A283" s="1" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B283" s="1" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="284" customHeight="1" ht="18.75">
       <c r="A284" s="1" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B284" s="1" t="s">
-        <v>548</v>
+        <v>277</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="285" customHeight="1" ht="18.75">
@@ -4455,10 +4503,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="289" customHeight="1" ht="18.75">
-      <c r="A289" s="3" t="s">
+      <c r="A289" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="B289" s="3" t="s">
+      <c r="B289" s="1" t="s">
         <v>558</v>
       </c>
     </row>
@@ -4487,10 +4535,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="293" customHeight="1" ht="18.75">
-      <c r="A293" s="3" t="s">
+      <c r="A293" s="1" t="s">
         <v>565</v>
       </c>
-      <c r="B293" s="3" t="s">
+      <c r="B293" s="1" t="s">
         <v>566</v>
       </c>
     </row>
@@ -4519,10 +4567,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="297" customHeight="1" ht="18.75">
-      <c r="A297" s="1" t="s">
+      <c r="A297" s="3" t="s">
         <v>573</v>
       </c>
-      <c r="B297" s="1" t="s">
+      <c r="B297" s="3" t="s">
         <v>574</v>
       </c>
     </row>
@@ -4551,10 +4599,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="301" customHeight="1" ht="18.75">
-      <c r="A301" s="1" t="s">
+      <c r="A301" s="3" t="s">
         <v>581</v>
       </c>
-      <c r="B301" s="1" t="s">
+      <c r="B301" s="3" t="s">
         <v>582</v>
       </c>
     </row>
@@ -4564,6 +4612,70 @@
       </c>
       <c r="B302" s="1" t="s">
         <v>584</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="303" customHeight="1" ht="18.75">
+      <c r="A303" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="B303" s="1" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="304" customHeight="1" ht="18.75">
+      <c r="A304" s="1" t="s">
+        <v>587</v>
+      </c>
+      <c r="B304" s="1" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="305" customHeight="1" ht="18.75">
+      <c r="A305" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="B305" s="1" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="306" customHeight="1" ht="18.75">
+      <c r="A306" s="1" t="s">
+        <v>591</v>
+      </c>
+      <c r="B306" s="1" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="307" customHeight="1" ht="18.75">
+      <c r="A307" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="B307" s="1" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="308" customHeight="1" ht="18.75">
+      <c r="A308" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="B308" s="1" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="309" customHeight="1" ht="18.75">
+      <c r="A309" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="B309" s="1" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="310" customHeight="1" ht="18.75">
+      <c r="A310" s="1" t="s">
+        <v>599</v>
+      </c>
+      <c r="B310" s="1" t="s">
+        <v>600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add missing translations (#274)
</commit_message>
<xml_diff>
--- a/report_translations_standard.xlsx
+++ b/report_translations_standard.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="601">
   <si>
     <t>stringId</t>
   </si>
@@ -1003,18 +1003,18 @@
     <t>Edited by user</t>
   </si>
   <si>
+    <t>report.reporting.logChangeDateTime</t>
+  </si>
+  <si>
+    <t>Date and time edited</t>
+  </si>
+  <si>
     <t>report.reporting.logChangeRecordCreatedDateTime</t>
   </si>
   <si>
     <t>Date and time created</t>
   </si>
   <si>
-    <t>report.reporting.logChangeDateTime</t>
-  </si>
-  <si>
-    <t>Date and time edited</t>
-  </si>
-  <si>
     <t>report.reporting.medications</t>
   </si>
   <si>
@@ -1291,6 +1291,66 @@
     <t>Title</t>
   </si>
   <si>
+    <t>report.reporting.patientTotal</t>
+  </si>
+  <si>
+    <t>Total patients</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalBirthRegistrations</t>
+  </si>
+  <si>
+    <t>Total birth registrations</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalIncorrectRegistrationsForAgedUnder6Months</t>
+  </si>
+  <si>
+    <t>Total incorrect registrations for aged under 6 months</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalMerged</t>
+  </si>
+  <si>
+    <t>Total patients merged</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalPatientRegistrations</t>
+  </si>
+  <si>
+    <t>Total patient registrations</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithIncompleteName</t>
+  </si>
+  <si>
+    <t>Total patients with incomplete name</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithInvalidDateOfBirth</t>
+  </si>
+  <si>
+    <t>Total patients with invalid date of birth</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithMissingContact</t>
+  </si>
+  <si>
+    <t>Total patients with missing contact</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithMissingDateOfBirth</t>
+  </si>
+  <si>
+    <t>Total patients with missing date of birth</t>
+  </si>
+  <si>
+    <t>report.reporting.patientTotalWithMissingLocation</t>
+  </si>
+  <si>
+    <t>Total patients with missing location</t>
+  </si>
+  <si>
     <t>report.reporting.patientVillage</t>
   </si>
   <si>
@@ -1325,6 +1385,84 @@
   </si>
   <si>
     <t>Tamanu user name</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionDate</t>
+  </si>
+  <si>
+    <t>Prescription date</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionDoseAmount</t>
+  </si>
+  <si>
+    <t>Dose amount</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionFrequency</t>
+  </si>
+  <si>
+    <t>Frequency</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionIsOngoing</t>
+  </si>
+  <si>
+    <t>Is ongoing</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionIsPRN</t>
+  </si>
+  <si>
+    <t>Is PRN</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionIsVariableDose</t>
+  </si>
+  <si>
+    <t>Is variable dose</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedication</t>
+  </si>
+  <si>
+    <t>Medication</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionMedicationCode</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionQuantity</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionRepeats</t>
+  </si>
+  <si>
+    <t>Repeats</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionRoute</t>
+  </si>
+  <si>
+    <t>Route</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionSelectedForDischarge</t>
+  </si>
+  <si>
+    <t>Prescription selected for discharge</t>
+  </si>
+  <si>
+    <t>report.reporting.prescriptionUnits</t>
+  </si>
+  <si>
+    <t>Units</t>
   </si>
   <si>
     <t>report.reporting.procedure</t>
@@ -1689,13 +1827,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1731,12 +1875,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -2044,11 +2191,11 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:B287"/>
+  <dimension ref="A1:B310"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="58.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="64.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="35.71928571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -3387,7 +3534,7 @@
         <v>319</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="19.5">
       <c r="A168" s="1" t="s">
         <v>320</v>
       </c>
@@ -3395,7 +3542,7 @@
         <v>321</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="19.5">
       <c r="A169" s="1" t="s">
         <v>322</v>
       </c>
@@ -3403,7 +3550,7 @@
         <v>323</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="19.5">
       <c r="A170" s="1" t="s">
         <v>324</v>
       </c>
@@ -3411,7 +3558,7 @@
         <v>325</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="19.5">
       <c r="A171" s="1" t="s">
         <v>326</v>
       </c>
@@ -3427,15 +3574,15 @@
         <v>329</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18.75">
-      <c r="A173" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="20.25">
+      <c r="A173" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="B173" s="1" t="s">
+      <c r="B173" s="3" t="s">
         <v>331</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="19.5">
       <c r="A174" s="1" t="s">
         <v>332</v>
       </c>
@@ -3443,7 +3590,7 @@
         <v>333</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="19.5">
       <c r="A175" s="1" t="s">
         <v>334</v>
       </c>
@@ -3451,7 +3598,7 @@
         <v>335</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="19.5">
       <c r="A176" s="1" t="s">
         <v>336</v>
       </c>
@@ -3459,7 +3606,7 @@
         <v>337</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="19.5">
       <c r="A177" s="1" t="s">
         <v>338</v>
       </c>
@@ -3515,11 +3662,11 @@
         <v>351</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18.75">
-      <c r="A184" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="19.5">
+      <c r="A184" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="B184" s="2" t="s">
+      <c r="B184" s="3" t="s">
         <v>353</v>
       </c>
     </row>
@@ -3579,11 +3726,11 @@
         <v>367</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="18.75">
-      <c r="A192" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="19.5">
+      <c r="A192" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="B192" s="2" t="s">
+      <c r="B192" s="3" t="s">
         <v>369</v>
       </c>
     </row>
@@ -3659,15 +3806,15 @@
         <v>387</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="18.75">
-      <c r="A202" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="20.25">
+      <c r="A202" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="B202" s="2" t="s">
+      <c r="B202" s="3" t="s">
         <v>389</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="19.5">
       <c r="A203" s="1" t="s">
         <v>390</v>
       </c>
@@ -3675,7 +3822,7 @@
         <v>391</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="19.5">
       <c r="A204" s="1" t="s">
         <v>392</v>
       </c>
@@ -3683,7 +3830,7 @@
         <v>393</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="19.5">
       <c r="A205" s="1" t="s">
         <v>394</v>
       </c>
@@ -3691,7 +3838,7 @@
         <v>395</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="19.5">
       <c r="A206" s="1" t="s">
         <v>396</v>
       </c>
@@ -3699,7 +3846,7 @@
         <v>397</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="19.5">
       <c r="A207" s="1" t="s">
         <v>398</v>
       </c>
@@ -3707,7 +3854,7 @@
         <v>399</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="19.5">
       <c r="A208" s="1" t="s">
         <v>400</v>
       </c>
@@ -3788,18 +3935,18 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="218" customHeight="1" ht="18.75">
-      <c r="A218" s="2" t="s">
+      <c r="A218" s="3" t="s">
         <v>418</v>
       </c>
-      <c r="B218" s="2" t="s">
+      <c r="B218" s="3" t="s">
         <v>419</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="219" customHeight="1" ht="18.75">
-      <c r="A219" s="2" t="s">
+      <c r="A219" s="3" t="s">
         <v>420</v>
       </c>
-      <c r="B219" s="2" t="s">
+      <c r="B219" s="3" t="s">
         <v>421</v>
       </c>
     </row>
@@ -3811,7 +3958,7 @@
         <v>423</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="221" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="221" customHeight="1" ht="19.5">
       <c r="A221" s="1" t="s">
         <v>424</v>
       </c>
@@ -3819,7 +3966,7 @@
         <v>425</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="222" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="222" customHeight="1" ht="19.5">
       <c r="A222" s="1" t="s">
         <v>426</v>
       </c>
@@ -3827,7 +3974,7 @@
         <v>427</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="223" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="223" customHeight="1" ht="19.5">
       <c r="A223" s="1" t="s">
         <v>428</v>
       </c>
@@ -3835,7 +3982,7 @@
         <v>429</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="224" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="224" customHeight="1" ht="19.5">
       <c r="A224" s="1" t="s">
         <v>430</v>
       </c>
@@ -3843,7 +3990,7 @@
         <v>431</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="225" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="225" customHeight="1" ht="19.5">
       <c r="A225" s="1" t="s">
         <v>432</v>
       </c>
@@ -3851,7 +3998,7 @@
         <v>433</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="226" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="226" customHeight="1" ht="19.5">
       <c r="A226" s="1" t="s">
         <v>434</v>
       </c>
@@ -3859,7 +4006,7 @@
         <v>435</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="227" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="227" customHeight="1" ht="19.5">
       <c r="A227" s="1" t="s">
         <v>436</v>
       </c>
@@ -3867,7 +4014,7 @@
         <v>437</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="228" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="228" customHeight="1" ht="19.5">
       <c r="A228" s="1" t="s">
         <v>438</v>
       </c>
@@ -3875,7 +4022,7 @@
         <v>439</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="229" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="229" customHeight="1" ht="19.5">
       <c r="A229" s="1" t="s">
         <v>440</v>
       </c>
@@ -3883,7 +4030,7 @@
         <v>441</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="230" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="230" customHeight="1" ht="19.5">
       <c r="A230" s="1" t="s">
         <v>442</v>
       </c>
@@ -4008,319 +4155,319 @@
         <v>472</v>
       </c>
       <c r="B245" s="1" t="s">
-        <v>241</v>
+        <v>473</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="246" customHeight="1" ht="18.75">
-      <c r="A246" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="B246" s="2" t="s">
+      <c r="A246" s="1" t="s">
         <v>474</v>
+      </c>
+      <c r="B246" s="1" t="s">
+        <v>475</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="247" customHeight="1" ht="18.75">
       <c r="A247" s="1" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B247" s="1" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="248" customHeight="1" ht="18.75">
-      <c r="A248" s="2" t="s">
-        <v>477</v>
-      </c>
-      <c r="B248" s="2" t="s">
+      <c r="A248" s="1" t="s">
         <v>478</v>
       </c>
+      <c r="B248" s="1" t="s">
+        <v>479</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="249" customHeight="1" ht="18.75">
-      <c r="A249" s="2" t="s">
-        <v>479</v>
-      </c>
-      <c r="B249" s="2" t="s">
+      <c r="A249" s="1" t="s">
         <v>480</v>
       </c>
+      <c r="B249" s="1" t="s">
+        <v>481</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="250" customHeight="1" ht="18.75">
-      <c r="A250" s="2" t="s">
-        <v>481</v>
-      </c>
-      <c r="B250" s="2" t="s">
+      <c r="A250" s="1" t="s">
         <v>482</v>
+      </c>
+      <c r="B250" s="1" t="s">
+        <v>483</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="251" customHeight="1" ht="18.75">
       <c r="A251" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B251" s="1" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="252" customHeight="1" ht="18.75">
       <c r="A252" s="1" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B252" s="1" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="253" customHeight="1" ht="18.75">
       <c r="A253" s="1" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B253" s="1" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="254" customHeight="1" ht="18.75">
       <c r="A254" s="1" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B254" s="1" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="255" customHeight="1" ht="18.75">
       <c r="A255" s="1" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>47</v>
+        <v>493</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="256" customHeight="1" ht="18.75">
       <c r="A256" s="1" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B256" s="1" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="257" customHeight="1" ht="18.75">
       <c r="A257" s="1" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B257" s="1" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="258" customHeight="1" ht="18.75">
-      <c r="A258" s="2" t="s">
-        <v>496</v>
-      </c>
-      <c r="B258" s="2" t="s">
-        <v>497</v>
+      <c r="A258" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="B258" s="1" t="s">
+        <v>499</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="259" customHeight="1" ht="18.75">
       <c r="A259" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B259" s="1" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="260" customHeight="1" ht="18.75">
       <c r="A260" s="1" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="261" customHeight="1" ht="18.75">
       <c r="A261" s="1" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B261" s="1" t="s">
-        <v>277</v>
+        <v>505</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="262" customHeight="1" ht="18.75">
       <c r="A262" s="1" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="263" customHeight="1" ht="18.75">
       <c r="A263" s="1" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B263" s="1" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="264" customHeight="1" ht="18.75">
       <c r="A264" s="1" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="B264" s="1" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="265" customHeight="1" ht="18.75">
       <c r="A265" s="1" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="B265" s="1" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="266" customHeight="1" ht="18.75">
       <c r="A266" s="1" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="B266" s="1" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="267" customHeight="1" ht="18.75">
       <c r="A267" s="1" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="B267" s="1" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="268" customHeight="1" ht="18.75">
       <c r="A268" s="1" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="B268" s="1" t="s">
-        <v>516</v>
+        <v>241</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="269" customHeight="1" ht="18.75">
-      <c r="A269" s="1" t="s">
-        <v>517</v>
-      </c>
-      <c r="B269" s="1" t="s">
-        <v>518</v>
+      <c r="A269" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="B269" s="3" t="s">
+        <v>520</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="270" customHeight="1" ht="18.75">
       <c r="A270" s="1" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B270" s="1" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="271" customHeight="1" ht="18.75">
-      <c r="A271" s="1" t="s">
-        <v>521</v>
-      </c>
-      <c r="B271" s="1" t="s">
-        <v>522</v>
+      <c r="A271" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="B271" s="3" t="s">
+        <v>524</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="272" customHeight="1" ht="18.75">
-      <c r="A272" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="B272" s="1" t="s">
-        <v>524</v>
+      <c r="A272" s="3" t="s">
+        <v>525</v>
+      </c>
+      <c r="B272" s="3" t="s">
+        <v>526</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="273" customHeight="1" ht="18.75">
-      <c r="A273" s="1" t="s">
-        <v>525</v>
-      </c>
-      <c r="B273" s="1" t="s">
-        <v>526</v>
+      <c r="A273" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="B273" s="3" t="s">
+        <v>528</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="274" customHeight="1" ht="18.75">
-      <c r="A274" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="B274" s="2" t="s">
-        <v>528</v>
+      <c r="A274" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="B274" s="1" t="s">
+        <v>530</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="275" customHeight="1" ht="18.75">
       <c r="A275" s="1" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B275" s="1" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="276" customHeight="1" ht="18.75">
       <c r="A276" s="1" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B276" s="1" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="277" customHeight="1" ht="18.75">
       <c r="A277" s="1" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B277" s="1" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="278" customHeight="1" ht="18.75">
-      <c r="A278" s="2" t="s">
-        <v>535</v>
-      </c>
-      <c r="B278" s="2" t="s">
-        <v>536</v>
+      <c r="A278" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="B278" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="279" customHeight="1" ht="18.75">
       <c r="A279" s="1" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B279" s="1" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="280" customHeight="1" ht="18.75">
       <c r="A280" s="1" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B280" s="1" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="281" customHeight="1" ht="18.75">
-      <c r="A281" s="1" t="s">
-        <v>541</v>
-      </c>
-      <c r="B281" s="1" t="s">
+      <c r="A281" s="3" t="s">
         <v>542</v>
+      </c>
+      <c r="B281" s="3" t="s">
+        <v>543</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="282" customHeight="1" ht="18.75">
       <c r="A282" s="1" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="283" customHeight="1" ht="18.75">
       <c r="A283" s="1" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B283" s="1" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="284" customHeight="1" ht="18.75">
       <c r="A284" s="1" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B284" s="1" t="s">
-        <v>548</v>
+        <v>277</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="285" customHeight="1" ht="18.75">
@@ -4345,6 +4492,190 @@
       </c>
       <c r="B287" s="1" t="s">
         <v>554</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="288" customHeight="1" ht="18.75">
+      <c r="A288" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="B288" s="1" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="289" customHeight="1" ht="18.75">
+      <c r="A289" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="B289" s="1" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="290" customHeight="1" ht="18.75">
+      <c r="A290" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="291" customHeight="1" ht="18.75">
+      <c r="A291" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="B291" s="1" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="292" customHeight="1" ht="18.75">
+      <c r="A292" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="B292" s="1" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="293" customHeight="1" ht="18.75">
+      <c r="A293" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="B293" s="1" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="294" customHeight="1" ht="18.75">
+      <c r="A294" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="B294" s="1" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="295" customHeight="1" ht="18.75">
+      <c r="A295" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="B295" s="1" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="296" customHeight="1" ht="18.75">
+      <c r="A296" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="B296" s="1" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="297" customHeight="1" ht="18.75">
+      <c r="A297" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="B297" s="3" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="298" customHeight="1" ht="18.75">
+      <c r="A298" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="B298" s="1" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="299" customHeight="1" ht="18.75">
+      <c r="A299" s="1" t="s">
+        <v>577</v>
+      </c>
+      <c r="B299" s="1" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="300" customHeight="1" ht="18.75">
+      <c r="A300" s="1" t="s">
+        <v>579</v>
+      </c>
+      <c r="B300" s="1" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="301" customHeight="1" ht="18.75">
+      <c r="A301" s="3" t="s">
+        <v>581</v>
+      </c>
+      <c r="B301" s="3" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="302" customHeight="1" ht="18.75">
+      <c r="A302" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="B302" s="1" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="303" customHeight="1" ht="18.75">
+      <c r="A303" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="B303" s="1" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="304" customHeight="1" ht="18.75">
+      <c r="A304" s="1" t="s">
+        <v>587</v>
+      </c>
+      <c r="B304" s="1" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="305" customHeight="1" ht="18.75">
+      <c r="A305" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="B305" s="1" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="306" customHeight="1" ht="18.75">
+      <c r="A306" s="1" t="s">
+        <v>591</v>
+      </c>
+      <c r="B306" s="1" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="307" customHeight="1" ht="18.75">
+      <c r="A307" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="B307" s="1" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="308" customHeight="1" ht="18.75">
+      <c r="A308" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="B308" s="1" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="309" customHeight="1" ht="18.75">
+      <c r="A309" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="B309" s="1" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="310" customHeight="1" ht="18.75">
+      <c r="A310" s="1" t="s">
+        <v>599</v>
+      </c>
+      <c r="B310" s="1" t="s">
+        <v>600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>